<commit_message>
Add UNOC-011 to UNOC-020 to Unoccupied Property Case Database — Batch 2 complete
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Unoccupied_Property_Case_Database.xlsx
+++ b/knowledge/case-databases/Unoccupied_Property_Case_Database.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1661,6 +1661,1056 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>DRN-1623377</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>6 May 2020</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Unoccupied property insurance (undergoing refurbishment) — escape of water from attic pipe declined under Structural Works Clause endorsement; insurer maintained the clause excluded EOW/Trace and Access cover from the moment the endorsement was added, regardless of whether structural work had actually begun</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Property unoccupied from November 2018 policy inception pending refurbishment; structural work disclosed at inception but had not yet started when the February 2019 escape of water occurred</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Residential unoccupied property (pre-refurbishment)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Structural Works Clause endorsement excluded Escape of Water and Trace and Access cover 'until all the structural work, as disclosed to us, has been fully completed'; insurer applied this from the date the endorsement was added, not from the date work actually started</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Mr and Mrs S (via loss adjuster): endorsement should not bite until structural work had actually commenced; no work had started when the leak occurred. Lloyd's: endorsement applies 'at all times' from inception once disclosed, irrespective of whether work had started. FOS: Schedule of Cover endorsements section read as a whole is clear — EOW cover suspended 'at all times' and 'until all structural work has been completed'; the loss adjuster's on-site report did not confirm heating clause compliance and had not completed its assessment; insurer retained final decision-making authority over the loss adjuster's report</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Lloyd's correctly declined the escape of water claim under the terms of the Structural Works Clause endorsement</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>A Structural Works Clause endorsement that suspends Escape of Water and Trace and Access cover 'until all the structural work, as disclosed to us, has been fully completed' operates from the point the endorsement is added to the policy — it is not conditional on the disclosed works having actually started; reading the endorsements section as a whole (including the 'at all times' wording), a policyholder's honesty about future intended works does not prevent the exclusion applying immediately upon disclosure</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>A completed loss adjuster assessment confirming compliance with the Heating Clause (Unoccupied Property) — the adjuster's report did not resolve this point and instead awaited a plumber's report on causation, but this was ultimately immaterial once the Structural Works Clause was found to apply</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>Schedule of Cover stated endorsements apply 'at all times'; EOW/Trace and Access excluded until structural work fully completed, reinstated thereafter subject to the Heating Clause; no work had started but exclusion still applied per plain wording; loss adjuster's incomplete assessment was only one input into the insurer's overall decision, which properly considered the endorsement; claim correctly declined</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>When a Structural Works Clause or similar endorsement is added upon disclosure of intended future works, claims handlers must apply the exclusion from the endorsement's effective date, not from the date works commence — policyholders should be warned at point of disclosure that cover for related perils (EOW, Trace and Access) is suspended immediately, not only once work begins; an incomplete or inconclusive loss adjuster report does not prevent the insurer relying on a clear policy exclusion when it makes its final coverage decision</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>IF structural_works_clause_endorsement_added_on_disclosure_of_future_works AND policy_states_endorsements_apply_at_all_times THEN eow_and_trace_and_access_cover_excluded_from_endorsement_effective_date_regardless_of_whether_works_have_started; loss_adjuster_incomplete_assessment_does_not_override_clear_policy_exclusion_relied_upon_by_insurer_in_final_decision</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>DRN-1623377.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>DRN-1719844</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Internet Insurance Services UK Ltd</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>7 Jan 2021</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Broker mis-sale complaint — advised sale of buildings insurance policy (branded 'Residential Let Property Scheme') for a property that would be unoccupied during renovation; consumer alleged policy name implied it covered let properties and was therefore unsuitable/misleading, and that reduced cover (fire, lightning, explosion, aircraft only) for unoccupied periods wasn't adequately explained</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Property unoccupied during a renovation/extension project from April 2010; policy provided reduced unoccupied-property cover for the works period, reverting to full cover once the consumer moved back in; policy itself lapsed in 2011</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Residential property under renovation (unoccupied during works)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable to a coverage decline — dispute concerned suitability of the policy sold in 2010, discovered when a 2019 roof claim (caused by builder workmanship, not an insured peril) was declined as outside the fire/lightning/explosion/aircraft cover for unoccupied periods</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Ms S: policy name ('Residential Let Property Scheme') implied it was for let properties, which caused confusion and made her doubt suitability; wanted broader cover. IIS: call recordings show advisor clearly explained the reduced level of cover available during the unoccupied works period ('all this policy will cover... is fire, lightning, earthquake, explosion and property owners' liability... won't cover theft, malicious damage, escape of water or storm damage'); policy provided exactly the cover Ms S asked for (buildings cover while unoccupied and under renovation). FOS: advisor's explanation of scope of cover was clear; policy name may have been confusing but the substance of cover (not the name) is what matters for suitability; no requirement the property be let for the policy to apply; no evidence of detriment from the policy name in the ten years since sale</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — the policy sold was suitable for Ms S's stated need (buildings cover for an unoccupied property undergoing renovation); the level of cover was clearly explained on the calls even though the policy's product name may have caused some confusion</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>For an advised sale of unoccupied-property buildings cover, the broker must clearly explain the reduced scope of cover applicable during the unoccupied period (e.g. fire/lightning/explosion/aircraft only, excluding theft, malicious damage, escape of water and storm) — recorded confirmation of this explanation on the sales call is strong evidence of suitability; a confusing or unconventional product name (e.g. one associated with let properties) does not by itself render an unoccupied-property policy unsuitable where the substantive cover matches the consumer's stated needs and there is no requirement that the property actually be let</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>Evidence that Ms S specifically requested cover for the builder's workmanship or latent defects — absent; the extensively recorded pre-sale calls did not include this requirement</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>Two recorded calls showed IIS's advisor explained the unoccupied-period cover was limited to fire, lightning, earthquake, explosion and property owners' liability, excluding EOW/theft/storm; Ms S provided rebuild estimates and confirmed she'd return once works completed; policy matched her stated needs; the 'Residential Let Property Scheme' name was potentially confusing but its substance, not its name, governs suitability; no evidence of financial detriment from the name over ten years; not mis-sold</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>Brokers selling unoccupied-property cover under a product name that could imply a different purpose (e.g. a let-property scheme) should proactively clarify the name's origin at the point of sale, even where the substantive cover matches the consumer's needs, to avoid downstream confusion; suitability assessments for unoccupied-property add-ons should focus on whether the explained scope of cover (not the product branding) matches what the consumer told the broker they needed</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>IF broker_clearly_explains_reduced_unoccupied_period_cover_on_recorded_call AND cover_matches_consumers_stated_need THEN advised_sale_of_unoccupied_property_policy_is_suitable_regardless_of_potentially_confusing_product_name; policy_name_alone_does_not_establish_mis_sale_absent_evidence_the_substantive_cover_did_not_match_consumer_requirements</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
+        <is>
+          <t>DRN-1719844.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DRN1874552</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Ageas Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>19 Feb 2015</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Commercial property owners insurance (two self-contained units) — escape of water from multiple burst pipes over Christmas period in a unit undergoing renovation after tenants vacated; heating not switched on due to works; insurer declined claim citing unoccupied-property exclusion and drain-down condition breach</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>One of two self-contained units vacated by tenants and unoccupied for more than 30 consecutive days while undergoing building works; director visited at least daily during the Christmas holiday period when works paused; other unit remained tenanted and unaffected</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Commercial property (two self-contained units; one unoccupied during renovation)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Policy excluded escape of water/freezing damage to premises unoccupied, untenanted, or not in active use for 30+ consecutive days; company was also in breach of the condition requiring water systems to be drained in unoccupied properties</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>B (via advisers): had been in occupation during building works and a director visited at least daily over Christmas, so the unit wasn't 'unoccupied'; exclusion/condition not market standard and not properly drawn to attention at inception; loss adjusters gave inconsistent reasons for declining. Ageas: unit was untenanted and had not been in active use in connection with the property-owner business for 30+ days; frequent visits for building-site purposes are not equivalent to occupation. FOS: policy's 'unoccupied' definition is disjunctive — meeting any one of unoccupied/untenanted/not in active use for 30+ days triggers the exclusion; the unit was untenanted regardless of the other tenanted unit; daily inspection visits to what was 'essentially a building site' do not amount to occupation; exclusion not unusual and broker (not insurer) was responsible for explaining standard policy terms</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Ageas was entitled to decline the claim; the unit was unoccupied under the policy's disjunctive definition and the exclusion applied</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>A disjunctive definition of 'unoccupied' (unoccupied OR untenanted OR not in active use for the relevant business for 30+ consecutive days) is satisfied if any single limb is met — a property does not need to be literally empty of all activity to be classed as unoccupied where it has been untenanted for the qualifying period, even if other visits (e.g. by a director carrying out or overseeing building works) occur frequently; frequent inspection visits to premises that are 'essentially a building site' do not constitute occupation; where only one part of a multi-unit building is untenanted, the unoccupied exclusion can apply to that part alone regardless of continued occupation elsewhere in the building; standard, non-unusual unoccupied-property exclusions and conditions sold via a broker do not need to be separately highlighted by the insurer</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>Evidence that active occupation-level use (rather than periodic inspection during renovation) continued in the untenanted unit — absent; B accepted the unit had been vacated by tenants more than 30 days before the loss</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>Definition applies if 'any…part of the building' is unoccupied/untenanted/not in active use for 30+ days; the vacated unit was untenanted for the qualifying period; building-works activity and daily director visits over Christmas did not equate to normal commercial occupation; loss adjusters' inconsistent explanations did not prejudice B given it had expert advisers; exclusion and drain-down condition were standard and did not require specific insurer highlighting when sold through a broker; claim properly declined</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>Multi-unit or multi-tenant commercial property policies should be assessed unit-by-unit for unoccupancy purposes — continued occupation of one unit does not preserve cover for a vacated unit under a disjunctive 'unoccupied' definition; claims handlers should distinguish between genuine occupation-level activity and periodic building-site inspection visits when assessing whether the unoccupancy threshold has been met; loss adjusters should give consistent, clearly-referenced reasons for declining a claim even where the policyholder has expert representation</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>IF policy_defines_unoccupied_disjunctively_as_unoccupied_OR_untenanted_OR_not_in_active_use_for_30_plus_days THEN any_single_limb_being_met_triggers_the_unoccupied_exclusion; IF only_activity_at_property_is_periodic_inspection_during_building_works THEN this_does_not_constitute_occupation_or_active_use; IF one_unit_of_multi_unit_property_is_untenanted_for_qualifying_period THEN unoccupied_exclusion_applies_to_that_unit_regardless_of_occupation_status_of_other_units</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>DRN1874552.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-014</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>DRN2281195</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>18 Jul 2019</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Unoccupied property insurance (converted from a tenanted policy at renewal after Lloyd's discovered extended unoccupancy) — arson fire started by intruders/vandals; insurer declined citing breach of conditions requiring removal of refuse/waste materials and notification of illegal occupiers</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Property unoccupied since November 2016 (previously let); renewed under a tenanted policy in May 2017 without Lloyd's being told of the unoccupancy; Lloyd's treated the claim as if an unoccupied-property policy had applied, since it would not have offered a tenanted policy had it known</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Residential unoccupied property (previously let; undergoing refurbishment at time of fire)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Breach of unoccupied-property policy condition requiring all refuse and waste materials to be removed from the interior; photographs showed a large quantity of burnt rubbish, discarded timber, waste products, plastic buckets and ripped-out kitchen carcasses; fire brigade report found the fire started with paper/cardboard, which contributed to the fire's spread</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Mr G: unaware of the unoccupied-property conditions since he hadn't been told the property was being treated as unoccupied; items were retained for refurbishment (kitchen units to be fitted) and books/comics intended for charity, not waste; fire was started deliberately by third parties regardless of the property's contents. Lloyd's: would only have offered an unoccupied-property policy on renewal had it known of the unoccupancy, and did not offer a tenanted policy for empty properties; photographic evidence showed materials consistent with waste, not solely refurbishment items. FOS (provisional and final): fair to treat the claim as if under an unoccupied-property policy since the alternative was no cover at all; volume of debris exceeded what would reasonably be expected from refurbishment alone; breach of the waste-removal condition was materially connected to the fire loss since waste paper was the ignition source and fed the fire's spread; only one breached condition is needed to justify declining a claim</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Lloyd's fairly treated the claim under the terms applicable to an unoccupied property and was entitled to decline it for breach of the waste-removal condition, which was materially connected to the fire loss</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>Where an insurer discovers after a loss that a property was unoccupied when a tenanted (not unoccupied) policy was in force, and it would only have offered unoccupied-property cover (with its own conditions) had it known, it is reasonable to assess the claim as though the unoccupied-property policy terms applied — the policyholder's unawareness of those specific conditions does not excuse compliance, since notifying the insurer of the true occupancy status was the policyholder's own responsibility; a condition requiring removal of refuse and waste materials from an unoccupied property is a risk-control measure specifically aimed at reducing arson risk, and a breach of it will bar a claim for fire damage where the ignition source and its spread are materially connected to the retained waste — this differs from breach of an unrelated condition (e.g. a burglar alarm requirement) in a flood claim, which would not be materially connected</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>Clear itemised inventory distinguishing genuine refurbishment materials from discarded waste at the time of the fire — absent; the photographic evidence was relied upon instead and showed volumes inconsistent with refurbishment alone</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>Property unoccupied since November 2016; renewed as tenanted May 2017 without notification; Lloyd's would not have offered a tenanted policy for an empty property, so treating the claim under unoccupied-property terms was reasonable; photographs showed 'heavily loaded' debris, rubbish and loose combustible materials disproportionate to refurbishment needs; fire brigade confirmed paper/cardboard ignition; breach of the waste-removal condition materially connected to the fire since it fed the blaze; only one condition breach needed to support declining the claim; insured's lack of connection to the arson itself is irrelevant where a separate condition breach applies</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>When an insurer discovers post-loss that a tenanted policy was incorrectly in force over what was actually an unoccupied property, it is fair to assess the claim against the unoccupied-property terms it would have offered, rather than refusing cover outright — but this means the policyholder is held to conditions (e.g. waste removal, illegal-occupier notification) they were never told about, so materiality of any breach to the specific loss becomes the key fairness test; claims handlers must show a breach of a risk-control condition (like waste removal) is causally connected to the peril claimed for (fire) before relying on it to decline</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_discovers_post_loss_that_tenanted_policy_was_in_force_over_actually_unoccupied_property AND insurer_would_only_have_offered_unoccupied_property_terms_if_notified THEN claim_may_fairly_be_assessed_against_unoccupied_property_policy_conditions_even_though_policyholder_was_unaware_of_them; IF waste_removal_condition_breached_AND_waste_materials_were_ignition_source_or_fuel_for_the_fire THEN breach_is_materially_connected_to_fire_loss_and_insurer_may_decline_claim; only_one_materially_connected_condition_breach_is_required_to_justify_declining_a_claim</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>DRN2281195.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>DRN2912517</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>7 Aug 2017</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Commercial property insurance — escape of sewage from a tenanted shop/basement discovered by local authority after buildup over two-three months; insurer declined citing breach of unoccupied-property notification, inspection and reasonable-precautions conditions after determining the property had in fact been unoccupied</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Property unoccupied for an extended period (tenant hadn't paid rent since February 2014; some evidence of a year or more of unoccupancy) but the policyholder (landlord) says it only became aware of the unoccupancy when the local authority contacted it in January 2016; tenant later explained he had been abroad in India due to a family medical emergency</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Commercial let property (shop with basement)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>UKI concluded the property had been unoccupied when the sewage escape occurred and said P had breached obligations to notify of a change in occupation, to inspect the unoccupied property every 14 days, and to take reasonable precautions to prevent damage</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>P: unaware the property was unoccupied until notified by the local authority in January 2016; had been accommodating the tenant's personal difficulties over unpaid rent since February 2014 and only instructed solicitors in June 2015 over the rent arrears, not because it knew the property was empty; director lived some distance away and had no reason to suspect external signs of vacancy. UKI: tenant hadn't paid rent since February 2014; neighbours reported the shop had been closed for a year or more; instructing solicitors over unpaid rent in June 2015 should have prompted notification of a change in risk. FOS: policy's notification obligation and 'unaffected by act/omission of a tenant' proviso both require actual awareness of a change in occupation before the obligation to notify arises; no evidence P knew the property was unoccupied before January 2016; instructing solicitors over unpaid rent is not equivalent to knowing a property is unoccupied; without awareness, the 14-day inspection and general reasonable-precautions obligations could not reasonably have been triggered either</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>UKI required to accept the claim, reimburse any invoices already paid by P directly with 8% simple interest from the date of payment to settlement, and continue providing cover for the repair work</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>A policy condition requiring notification of a change in occupation 'as soon as they become aware' only bites once the insured has actual knowledge of the change — a policy provision stating cover 'will not be prejudiced by any act or omission unknown to or beyond the control of the Insured on the part of a tenant' reinforces that unawareness of a tenant's own conduct (including abandoning the property) does not constitute a breach; obligations to inspect unoccupied premises at least every 14 days and take reasonable precautions for unoccupied properties cannot fairly be relied upon by an insurer where the policyholder did not know, and had no reasonable means of knowing, that the property had become unoccupied; non-payment of rent alone, or instructing solicitors to recover arrears, does not equate to knowledge that a property is unoccupied</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>Evidence that P had actual knowledge of the unoccupancy before the local authority's January 2016 contact — absent; UKI relied only on inferences from non-payment of rent and neighbour reports, not on anything shown to have reached P</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>Tenant hadn't paid rent since Feb 2014, and neighbours suggested the shop had been shut for a year or more, but P's director lived some distance away and had no reason to suspect the property (as opposed to the tenant's rent account) was actually vacant; solicitor instruction in June 2015 concerned unpaid rent, not unoccupancy; policy's notification duty and the 'unknown to or beyond control of the Insured' proviso both turn on actual awareness; without awareness, the 14-day inspection and reasonable-precautions conditions specific to vacant/disused locations could not reasonably apply either; UKI could not rely on any of the three clauses to decline; claim should be accepted with interest on any invoices already paid</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>When investigating suspected non-disclosure of unoccupancy, insurers must establish that the policyholder had actual knowledge of the change in occupation, not merely that objective indicators (unpaid rent, neighbour reports of closure) existed which the insurer itself later uncovered — a landlord's tolerance of a struggling tenant's rent arrears, or instructing solicitors to recover unpaid rent, is not on its own evidence of knowledge that the property has become physically unoccupied; distance between a landlord's residence and the let property is a relevant factor in assessing whether the landlord could reasonably have known of unoccupancy</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>IF policy_notification_duty_is_conditioned_on_insured_becoming_aware_of_change_in_occupation AND insurer_cannot_show_actual_knowledge_by_policyholder_of_unoccupancy THEN insurer_cannot_decline_claim_for_breach_of_notification_condition; IF policyholder_lacked_actual_knowledge_of_unoccupancy THEN inspection_and_reasonable_precautions_conditions_specific_to_unoccupied_properties_cannot_be_relied_upon_either; non_payment_of_rent_or_solicitor_instruction_over_arrears_does_not_by_itself_establish_landlord_knowledge_that_property_is_unoccupied</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>DRN2912517.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="80" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>DRN-2973838</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>AmTrust Europe Limited</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>22 Oct 2021</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Commercial buildings insurance (let flats) — theft of pipework and fixed appliances during the void period following an accepted fire damage claim, before reinstatement works began; insurer declined the theft claim under the policy's unoccupancy exclusion, regardless of the reason for the unoccupancy</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Property unoccupied following fire damage that forced tenants to move out; unoccupancy exceeded the policy's 60-day threshold (defined as empty/disused/unoccupied/unfurnished/untenanted for 60+ days) while awaiting claim assessment and reinstatement; theft occurred during this period, before repairs started</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Residential let property, multiple self-contained flats</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Policy excluded theft where the buildings had become 'Unoccupied' (empty/disused/unfurnished/untenanted for 60+ days) under Endorsement 011b and the Change of Definition — Unoccupied clause; theft occurred after the 60-day threshold had been passed while the property remained vacant pending fire-claim reinstatement</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Mr R: unoccupancy only arose because of an insured peril (fire) which he could not control, and was compounded by claim-handling delays; AmTrust should not rely on the exclusion in these circumstances. AmTrust: unoccupancy exclusion applies regardless of the underlying cause of the unoccupancy; offered £100 compensation for acknowledged claim-handling delays but maintained the theft exclusion applied. FOS: policy wording is clear and contains no exception for unoccupancy caused by an insured peril; even absent any avoidable delay, the loss adjuster estimated repairs would take around four months — well beyond the 60-day threshold — so the property would have remained unoccupied past the threshold regardless of AmTrust's handling</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — AmTrust correctly declined the theft claim under the unoccupancy exclusion; £100 already offered for acknowledged claim-handling delays stands but the theft claim itself is not payable, since even without those delays the 60-day threshold would still have been exceeded given the scale of the fire repairs</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>An unoccupancy exclusion tied to a fixed time threshold (e.g. 60 days empty/disused/unfurnished/untenanted) applies regardless of the reason the property became unoccupied — including where unoccupancy results from an earlier insured peril (such as fire) that is entirely outside the policyholder's control; there is no implied exception for unoccupancy caused by a covered event unless the policy expressly provides for one; where an insurer has caused some avoidable claim-handling delay, this will not assist the policyholder in disputing an unoccupancy exclusion unless the delay can be shown to have caused the property to cross the relevant unoccupancy threshold that it would not otherwise have crossed</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>Evidence that, absent AmTrust's acknowledged handling delays, reinstatement could have been completed and the property reoccupied within 60 days of the fire — absent; the loss adjuster's own repair-time estimate (approximately four months) showed the threshold would have been exceeded regardless</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>Policy and Endorsement 011b unambiguously excluded theft cover once the property met the 60-day unoccupancy definition, with no carve-out based on cause; property became unoccupied due to fire damage, an event outside either party's control at the time of the theft; AmTrust's acknowledged handling delays did not causally extend the unoccupancy period beyond what the fire damage itself would have caused, since repairs were independently estimated at around four months; £100 already offered for the delays was proportionate and not increased since no material impact from the delay was shown</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>Claims handlers should confirm whether a fixed-threshold unoccupancy exclusion contains any carve-out for unoccupancy arising from a prior insured peril before declining a subsequent claim on that ground — where no such carve-out exists, the exclusion applies regardless of blamelessness; where a policyholder alleges that insurer-caused delay extended the unoccupancy period past the relevant threshold, handlers should obtain and rely on independent repair-time estimates to assess whether the threshold would have been crossed in any event</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
+        <is>
+          <t>IF unoccupancy_exclusion_is_defined_by_a_fixed_time_threshold_with_no_cause_based_carve_out THEN exclusion_applies_regardless_of_whether_unoccupancy_arose_from_a_separate_insured_peril; IF policyholder_alleges_insurer_delay_caused_unoccupancy_threshold_to_be_exceeded AND independent_repair_estimate_shows_threshold_would_have_been_exceeded_regardless_of_delay THEN delay_argument_does_not_defeat_the_unoccupancy_exclusion</t>
+        </is>
+      </c>
+      <c r="U17" s="3" t="inlineStr">
+        <is>
+          <t>DRN-2973838.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3053282</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>29 Dec 2021</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Property Owners insurance — mid-term policy adjustment dispute (not a declined claim); at renewal the insured disclosed the commercial rental property was unoccupied, so Aviva applied an Unoccupied Premises Cover Restriction (fire/lightning/explosion/earthquake only); when the property became occupied again four months later, Aviva reinstated full cover but also raised the escape of water and storm/flood excesses to £2,500 (later reduced EOW excess back to £500 but kept storm/flood at £2,500 due to an open prior storm claim); policyholder complained the mid-term excess increase was unfair</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Commercial rental property unoccupied at the point of annual renewal; became occupied again approximately four months into the policy year, at which point full cover (subject to revised excesses) was reinstated</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Commercial rental property</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — no claim was declined; the dispute concerned whether a mid-term increase to policy excesses, applied when cover was upgraded from the Unoccupied Premises Cover Restriction back to full standard cover, was permitted and fair under the policy's Alteration of Risk clause</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Ms B: unoccupancy endorsement could simply have remained dormant and not applied once the property became occupied again, without any excess increase; combined with a separate £2,500 loss-of-rent excess, a storm claim could cost her £5,000 in excesses; if the policy term permitted this, the term itself was unfair. Aviva: at renewal, cover was restricted to fire/lightning/explosion/earthquake only because the property was unoccupied, so EOW and storm/flood risk (and any related claim history) hadn't been priced in; when occupancy resumed, it reassessed the risk for those newly-reinstated perils, taking into account an open prior storm claim, and set higher excesses accordingly; reduced the EOW excess back to standard once it recognised the open claim was for storm damage only. FOS: the policy's Alteration of Risk clause expressly permits new terms and conditions (including premium/excess changes) once notified of a change in risk; moving from unoccupied to occupied is itself a notifiable change in risk that engaged this clause; increasing the storm/flood excess for a fresh, previously-unpriced risk in light of an open storm claim was a legitimate commercial underwriting decision, not something FOS can second-guess on quantum</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Aviva was entitled under the policy's Alteration of Risk clause to reassess and adjust excesses for perils newly reinstated when the property became occupied again, and did so fairly by relying on the open storm claim history</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>An Alteration of Risk clause permitting new terms and conditions (including premium and excess changes) upon notification of a change in risk extends to a policyholder's notification that a previously unoccupied insured property has become occupied again — because perils excluded during the Unoccupied Premises Cover Restriction period (such as escape of water and storm/flood) were never priced into the restricted-cover premium, the insurer is entitled to reassess and reprice those specific perils, including by reference to claims history, when reinstating full cover; FOS will not adjudicate on the appropriateness of the excess amount itself, only on whether the policy permitted the adjustment and whether the process was fair</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — the material facts (unoccupancy at renewal, restricted cover applied, subsequent notification of reoccupation, and an open prior storm claim) were undisputed; the complaint turned on interpretation of the Alteration of Risk clause rather than any factual gap</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Policy renewed on the basis of unoccupancy with a restricted level of cover; Alteration of Risk clause allows new terms/conditions upon notification of a change in risk; occupancy resuming is a notifiable change; EOW and storm/flood cover (and any pricing for prior claims) was not factored in while the restriction applied, so it was reasonable for Aviva to reassess these specific perils on reinstatement; EOW excess was corrected once Aviva recognised the open claim was storm-only; storm/flood excess increase for a peril newly brought back into scope, informed by claims history, was fair and within Aviva's commercial discretion</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>Underwriters restricting cover for an unoccupied property should record which specific perils are excluded from pricing during the restriction so that, on reinstatement following reoccupation, only the newly-reinstated perils are subject to fresh risk assessment and excess adjustment — clear documentation of this distinction (as Aviva ultimately demonstrated by correcting the EOW excess once the storm-only nature of the open claim was recognised) helps resolve excess disputes without recourse to FOS</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>IF policyholder_notifies_insurer_that_previously_unoccupied_property_has_become_occupied_again AND alteration_of_risk_clause_permits_new_terms_on_notified_change_in_risk THEN insurer_may_reassess_and_reprice_perils_that_were_excluded_or_unpriced_during_the_unoccupied_restricted_cover_period; excess_or_premium_adjustments_for_perils_newly_reinstated_on_reoccupation_informed_by_open_claims_history_are_not_unfair_merely_because_they_increase_cost_to_policyholder</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3053282.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="80" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>DRN-3101941</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>9 Nov 2021</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Residential leasehold flat insurance — accidental damage claim for a gable-end wall partially collapsing after the dormer roof of a long-unoccupied, derelict neighbouring property caved in; council issued a Dangerous Building Notice requiring residents to leave; AXA declined the claim, attributing the wall collapse to gradual water ingress/general wear rather than a one-off event, even though two of the other three flat owners in the same building had the same damage accepted by their own insurers</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Not the insured's own property — the causative unoccupied property was a neighbouring building that had stood empty and derelict for some years (subject to two prior fires in 2013 and 2016, and long-standing local media coverage of its disrepair) before its dormer roof caved in and caused the shared gable-end wall to partially collapse</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Residential leasehold flat (one of four units in a shared building; damage caused by an adjoining unoccupied, derelict property)</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Causation Dispute</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>AXA considered the wall damage was not a one-off accidental event but resulted from water ingress accumulating over a number of years, softening the brickwork and ultimately causing the wall to collapse — treated as gradual/maintenance-related damage excluded under the policy</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Mr D and Mr R: two other flat owners in the same building, sharing the same damage to the same gable-end wall from the same event (the neighbouring dormer roof collapse), had their claims accepted by their own insurers, one of whom used the same loss adjuster as AXA; inconsistent for AXA alone to decline. AXA: maintained the damage was gradual water-ingress deterioration excluded under the policy, and that other insurers' decisions did not bind it. FOS (provisional, confirmed in final decision): the two properties were immediately adjoining, so deterioration of the shared wall would likely not have been visible until the dormer roof partially collapsed; no evidence of any internal signs of damage beforehand; a June 2018 survey found the chimney in fair condition; media reports confirmed the developer of the derelict property withdrew after the collapse 'damaged neighbouring homes'; all four flat owners share responsibility for, and are claiming for, the identical damage to the identical wall arising from the identical event, so it must be assessed identically; AXA's continued refusal despite two other insurers (including one using AXA's own loss adjuster) accepting the same damage as accidental was inconsistent and unfair</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>AXA required to accept and pay Mr D and Mr R's claim in line with the settlements already made to the other flat owners for the same damage, under the remaining terms of the policy</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>Where multiple co-owners in the same building each hold separate buildings insurance policies and all are claiming for the identical damage arising from the identical single event (here, the collapse of a neighbouring long-unoccupied, derelict property's roof onto a shared structural wall), an insurer that treats the damage as gradual/excluded while other insurers covering the same wall and the same event have accepted the claim as accidental is acting inconsistently; good industry practice and treating customers fairly requires consistent treatment of identical damage from an identical shared event across the different insurers involved, absent a clear, insurer-specific reason for departing from that consistency; the fact that a wall was hidden from view (and therefore its deteriorating condition could not have been observed or maintained by the policyholder) prior to a sudden triggering event supports treating the resulting damage as a one-off accidental loss rather than gradual deterioration</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>AXA did not produce independent engineering or surveying evidence specific to Mr D and Mr R's portion of the wall to justify treating their claim differently from the two accepted claims for the same wall and the same event; it relied solely on its own opinion that gradual water ingress caused the wall's softening</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="inlineStr">
+        <is>
+          <t>Site adjacency meant the wall's deteriorating condition would not have been visible until the neighbouring dormer roof partially collapsed; no internal signs of damage were shown to exist beforehand; 2018 survey found the chimney in fair condition; media reports confirmed a developer withdrew from the derelict site citing damage to neighbouring homes from the collapse; two of the four flat owners, including one sharing AXA's own loss adjuster, had the identical damage accepted as accidental by their insurers; AXA maintained its gradual-damage position without new evidence after the provisional decision; fair and reasonable outcome required AXA to treat Mr D and Mr R consistently with the other owners and pay the claim</t>
+        </is>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>Where damage originates from a long-unoccupied, derelict neighbouring property affecting multiple co-owned or shared-structure units, claims handlers should proactively check how other insurers covering the same building or wall have treated equivalent claims for the same triggering event before relying on a gradual-damage or wear-and-tear exclusion — inconsistency across insurers assessing identical damage from an identical cause is a strong indicator of an unfair declinature; adjacency and lack of visibility of a shared structural element prior to a sudden triggering event (e.g. a neighbouring roof collapse) should be weighed heavily in favour of treating resulting damage as a one-off accidental event</t>
+        </is>
+      </c>
+      <c r="T19" s="3" t="inlineStr">
+        <is>
+          <t>IF multiple_co_owners_of_a_shared_structural_element_hold_separate_policies AND all_are_claiming_for_identical_damage_from_an_identical_single_triggering_event THEN insurer_declining_on_gradual_damage_grounds_while_other_insurers_covering_the_same_element_and_event_have_accepted_the_claim_is_likely_unfair_absent_specific_contrary_evidence; IF damage_originates_from_a_long_unoccupied_derelict_neighbouring_property_and_shared_wall_condition_was_not_visible_or_inspectable_before_a_sudden_triggering_event THEN resulting_damage_should_generally_be_treated_as_a_one_off_accidental_loss_rather_than_gradual_deterioration</t>
+        </is>
+      </c>
+      <c r="U19" s="3" t="inlineStr">
+        <is>
+          <t>DRN-3101941.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="80" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3113837</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>16 Dec 2021</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Home insurance — policyholder notified insurer she was moving out (property becoming unoccupied); call handler misadvised her that staying at the property for a couple of nights every 60 days would reset the occupancy requirement and preserve cover; insurer's underwriting department later overturned this advice and cancelled the policy because the property was no longer her permanent home</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Property became unoccupied as Mrs Y moved to live elsewhere on a permanent basis; she visited for a 10-day period at one point, incurring travel costs, believing (based on the misadvice) that periodic overnight stays preserved her cover</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (owner relocating; no longer permanent home)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable to a coverage decline — AXA's underwriting department determined the policy did not meet its underwriting rules once it understood Mrs Y did not intend to return to the property on a permanent basis, and issued a cancellation notice rather than declining any specific claim</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Mrs Y: was told by a call handler that staying at the property for a couple of nights every 60 days would preserve cover, then was shocked to later receive a cancellation letter; sought reimbursement of travel costs incurred visiting the property in reliance on the (incorrect) advice. AXA: accepted the original advice was a mistake — the property no longer being Mrs Y's permanent home did not meet its underwriting criteria regardless of periodic overnight stays; confirmed cover remained in place and would have responded to any claim up to the cancellation date; waived the cancellation fee, refunded part of the premium, and (during the FOS process) offered £150 compensation for failing to offer this when it first responded to the complaint. FOS: AXA's initial advice was incorrect and it was reasonable for the underwriting department to correct it once identified; Mrs Y did have the benefit of cover throughout the period up to cancellation; travel costs were not reimbursable since she had the benefit of the policy regardless of whether she needed to claim, and could have chosen alternative arrangements; £150 was reasonable redress for the misadvice and the inconvenience it caused</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>AXA to pay Mrs Y the £150 compensation it offered, if she wishes to accept it; no further redress (including travel costs) required</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>Where a call handler gives incorrect advice about what preserves cover for a property becoming unoccupied (e.g. a periodic-overnight-stay 'reset' of the occupancy clock that does not reflect the insurer's actual underwriting rules), the insurer's underwriting department correcting that advice and issuing a cancellation notice is not itself unfair, provided the policyholder had the benefit of cover (and any claims would have been honoured) up to the cancellation date; compensation for the resulting confusion and inconvenience is appropriate, but travel costs incurred by a policyholder visiting a property in reliance on incorrect advice are not recoverable where the policyholder had the benefit of the policy throughout and had the option of alternative arrangements not requiring travel</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>Evidence that Mrs Y attempted to make, or was prevented from making, a claim during the period cover remained in force under the misadvised terms — absent; FOS therefore could not consider any substantive claim-handling issue, only the misadvice and cancellation process itself</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>Call handler's advice about a 60-day overnight-stay reset did not reflect AXA's actual underwriting position that the property needed to remain Mrs Y's permanent home; underwriting department was entitled to correct this and cancel once it understood her true circumstances; cover and claims-handling remained available up to the cancellation date, so Mrs Y suffered no loss of substantive cover; £150 (offered during the FOS process, after AXA accepted it should have provided redress in its complaint response) was fair for the confusion and inconvenience; travel costs not recoverable since the policy benefit was received regardless of use, and alternative non-travel arrangements existed</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>Call handlers giving advice about occupancy-preserving conditions (such as periodic overnight stays resetting an unoccupancy clock) must ensure the advice matches actual underwriting rules — incorrect advice of this kind should be identified and corrected as early as possible, ideally before the policyholder relies on it or incurs costs; when an insurer accepts it gave incorrect advice, redress should be offered proactively at the complaint-response stage rather than only once a case reaches the ombudsman service, to avoid a second layer of complaint about the redress process itself</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>IF call_handler_advises_that_periodic_overnight_stays_reset_the_unoccupancy_clock AND this_advice_does_not_reflect_actual_underwriting_rules THEN advice_is_incorrect_and_insurer_correcting_it_via_underwriting_review_and_cancellation_is_not_unfair_provided_cover_remained_honoured_up_to_cancellation; travel_costs_incurred_in_reliance_on_incorrect_occupancy_advice_are_not_recoverable_where_policyholder_had_uninterrupted_benefit_of_cover_throughout; compensation_for_confusion_and_inconvenience_from_misadvice_should_be_offered_at_first_complaint_response_not_only_after_referral_to_fos</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3113837.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="80" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-020</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>DRN3273371</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Lloyds Bank General Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>28 Jul 2018</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Home contents insurance — theft claim declined after policyholder moved out of the insured property (matrimonial separation) but continued visiting daily/every other day to care for animals and remained on the council tax; insurer applied the 30-day unoccupied exclusion; also cited lack of reasonable care and a family member's deliberate act as alternative grounds</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder moved out in November 2016 and had not lived at the property (in the sense of sleeping and washing there most of the week) for roughly three months by the time of the theft, despite visiting on a daily or every-other-day basis and remaining on the council tax; estranged family member (Mr K) restricted her access to remove her belongings</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Residential home (matrimonial property, policyholder relocated but retained access/visiting rights)</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Policy excluded theft cover where the home had not been 'lived in' for more than 30 days; Ms K had not lived in the property since November 2016, roughly three months before the claim</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Ms K: visited the property at least every other day (evidenced by ongoing care of animals kept there) and remained on the property's council tax, so she did not consider it unoccupied; a court order did not require immediate removal of all belongings; Mr K prevented her from accessing the property to retrieve her belongings. Lloyds: three separate exclusions applied — the 30-day unoccupied exclusion, a lack-of-reasonable-care exclusion, and an exclusion for theft caused by a deliberate act of a family member. FOS: the relevant test is whether the policyholder was 'living' in the property — i.e. sleeping and washing there most of the week — not merely visiting regularly or remaining registered for council tax; on the evidence, Ms K was living at another property and only visiting the insured property, which does not defeat the unoccupied exclusion; since the unoccupied exclusion alone was sufficient to justify declining the claim, the other two exclusions did not need to be separately addressed</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Lloyds was entitled to rely on the 30-day unoccupied exclusion to decline the contents theft claim</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>Where a policy's unoccupancy exclusion turns on whether the home has been 'lived in,' the relevant test is whether the policyholder was actually sleeping and washing at the property most of the week — regular visits (even daily or every-other-day) for a specific purpose such as caring for animals, and remaining registered for council tax at the address, do not by themselves establish that a policyholder was 'living' at the property if their primary residence has genuinely moved elsewhere; where an unoccupied-property exclusion alone is sufficient to justify declining a claim, the ombudsman need not separately determine whether other exclusions relied upon by the insurer (e.g. lack of reasonable care, deliberate act by a family member) would also independently apply</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>Evidence that Ms K was sleeping and washing at the insured property for the majority of the relevant period — absent; her evidence went only to frequency of visits and council tax registration, neither of which establishes 'living' at the property</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="inlineStr">
+        <is>
+          <t>Ms K had not lived in the property since November 2016, roughly three months before the theft; visiting daily or every other day to care for animals and remaining on the council tax record are consistent with regular visits to a property she no longer lived in, not with actually living there; the 'lived in' test requires sleeping and washing there most of the week, which was not met; unoccupied exclusion could reasonably be relied upon; no need to consider the two further exclusions Lloyds also cited since the unoccupied exclusion was sufficient on its own</t>
+        </is>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>When assessing whether a policyholder has 'lived in' a property for the purposes of an unoccupancy exclusion, claims handlers should apply a sleeping-and-washing-there test rather than treating regular visits, care of pets/animals kept at the property, or continued council tax registration as sufficient evidence of continued occupation; where multiple exclusions could independently justify declining a claim, it is efficient (and sufficient for a fair outcome) to establish that one applies without needing to separately evidence the others</t>
+        </is>
+      </c>
+      <c r="T21" s="3" t="inlineStr">
+        <is>
+          <t>IF policyholder_visits_property_regularly_for_a_specific_purpose_such_as_animal_care_or_remains_registered_for_council_tax BUT_sleeps_and_washes_primarily_at_another_address THEN property_is_not_lived_in_by_that_policyholder_for_unoccupancy_exclusion_purposes; IF one_policy_exclusion_is_independently_sufficient_to_justify_declining_a_claim THEN fos_and_insurer_need_not_separately_establish_additional_exclusions_also_relied_upon</t>
+        </is>
+      </c>
+      <c r="U21" s="3" t="inlineStr">
+        <is>
+          <t>DRN3273371.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add UNOC-021 to UNOC-030 to Unoccupied Property Case Database — Batch 3 complete
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Unoccupied_Property_Case_Database.xlsx
+++ b/knowledge/case-databases/Unoccupied_Property_Case_Database.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2711,6 +2711,1056 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="80" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>DRN3308022</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Ageas Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>4 Nov 2018</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Home insurance (rental property let to family) — escape of water discovered ~1 month after policy inception; insurer declined citing numerous inconsistencies in the policyholders' account of occupancy and compliance with policy conditions, without conclusively establishing the property had actually been unoccupied or unfurnished for the qualifying period</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Property let to family; policy incepted only about a month before the escape of water was discovered; insurer suspected the property was not genuinely occupied as claimed (citing a friend's inconsistent account of how often he stayed, and the property being under renovation) but could not show unoccupancy or lack of furnishing had lasted more than 90 consecutive days, since the policy itself had only been in force for about a month</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Residential rental property (let to family)</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Insurer said there were too many inconsistencies in the claim and it hadn't been shown the property was occupied as described or that policy conditions had been complied with — including doubts over the intended letting to family, a friend's account of overnight stays, renovation works in progress, and a three-month historical gap in insurance cover</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Mr and Mrs H: property was going to be let to family, doubts raised by the insurer were misunderstandings or explicable (e.g. quoting the plumber a repair estimate as an experienced builder wanting an accurate figure); gap in insurance history was inadvertent given Mr H's serious health issues. Ageas: multiple inconsistencies (letting intentions, friend's stay frequency, ongoing renovation, plumber quote conversation, insurance history) meant it hadn't been shown the property was occupied as claimed or that conditions were met. FOS: the 90-day unoccupied/unfurnished exclusion operates as an exclusion, so the burden is on the insurer to show, on the balance of probabilities, that the property was unoccupied or unfurnished for more than 90 days — since the policy had only started about a month before the loss, that could not have been the case regardless of the other inconsistencies; inconsistencies alone are not usually sufficient grounds to refuse a claim absent strong grounds that doing so is fair and reasonable</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Ageas required to settle Mr and Mrs H's claim in accordance with the remaining policy terms and conditions</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>Where an unoccupied/unfurnished exclusion requires the property to have been unoccupied or unfurnished for more than a specified number of consecutive days (here 90), that condition operates as an exclusion rather than a coverage precondition, meaning the burden of proof lies with the insurer to show, on the balance of probabilities, that the qualifying period was met — where the policy itself has only been in force for a shorter period than the qualifying threshold, the insurer cannot discharge that burden regardless of how many other inconsistencies exist in the policyholder's account; general inconsistencies in a policyholder's evidence, without more, do not meet this service's threshold of 'strong grounds' required to justify refusing an otherwise valid claim</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>Evidence that the property had actually been unoccupied or unfurnished for more than 90 consecutive days — could not exist given the policy had only been in force for about a month before the loss was discovered</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>Policy covered EOW unless the property had been left unfurnished or unoccupied for more than 90 consecutive days; this operates as an exclusion, so it fell to Ageas to prove the qualifying period on the balance of probabilities; since the policy had only incepted about a month earlier, this was structurally impossible regardless of the unresolved inconsistencies about furnishing, letting intentions, or the plumber conversation; the insurance-history gap was more likely an oversight given Mr H's health issues than a deliberate misrepresentation; overall, inconsistencies are not themselves strong grounds to decline a claim</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>Where an unoccupied/unfurnished exclusion is time-qualified (e.g. 90 consecutive days), claims handlers must first check whether the policy has even been in force long enough for the qualifying period to have elapsed before investigating disputed factual inconsistencies about occupancy — if the policy is younger than the qualifying period, the exclusion cannot apply regardless of what is eventually established about the property's actual use; unresolved inconsistencies in a policyholder's account should be weighed against this service's 'strong grounds' threshold rather than treated as automatically fatal to a claim</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>IF unoccupied_or_unfurnished_exclusion_requires_qualifying_period_of_N_consecutive_days AND policy_has_been_in_force_for_fewer_than_N_days_since_inception THEN exclusion_cannot_apply_regardless_of_disputed_occupancy_evidence; unoccupied_unfurnished_exclusion_operates_as_an_exclusion_so_burden_of_proof_is_on_insurer_not_policyholder; general_unresolved_inconsistencies_in_policyholder_account_do_not_alone_meet_strong_grounds_threshold_to_decline_a_claim</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>DRN3308022.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="80" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-022</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>DRN3390381</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Swinton Group Ltd</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>7 Sep 2019</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Broker complaint (not a declined claim) — policyholder alleged Swinton misled her into believing unoccupied buildings cover was only available through it and overcharged her for short-term (3/6-month) unoccupied property policies compared to a cheaper annual policy she later obtained from another provider</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Property insured on a rolling 6-month then 3-month unoccupied buildings basis from April 2015 until Swinton would no longer renew short-term cover from January 2017 (requiring a 12-month term instead), at which point she obtained a cheaper annual policy elsewhere</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Unoccupied property (type not further specified in decision)</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable to a coverage decline — dispute concerned whether Swinton misrepresented itself as the sole provider of unoccupied buildings cover and whether its short-term premiums were unfairly high compared to annual cover available elsewhere</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>Miss G: was told she could only get unoccupied buildings cover through Swinton, and it had overcharged her (over £1,200/year for short-term cover vs £170/year annual cover elsewhere). Swinton: found no evidence it told her it was the sole provider; it could only advise on its own panel prices, not the wider market; premium was accurately calculated to reflect risk plus a reasonable profit margin, and short-term policies generate more administrative work reflected in price; she had a 14-day cooling-off period each renewal to shop around. FOS: no recording existed of the original call, but it was more likely Swinton said only one insurer on its panel offered the product, not that it was the only provider in the market; premium calculation checked and found accurate and fair; even had Swinton flagged that an annual policy would be cheaper, Miss G was hoping to sell the property before each policy expired and had chosen short-term cover deliberately, so she would likely not have acted differently — this was confirmed when, even after Swinton stopped offering short-term cover, she sought another short-term provider rather than take a 12-month policy through Swinton</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — no evidence Swinton misrepresented itself as the sole provider, its premiums were fairly calculated, and Miss G would not have acted differently even with fuller information about annual pricing</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P23" s="3" t="inlineStr">
+        <is>
+          <t>A broker is entitled to price short-term (e.g. 3 or 6-month) unoccupied property cover higher on a pro-rata basis than an equivalent annual policy, reflecting the additional administrative burden of more frequent renewals, provided the pricing methodology is shown to be applied consistently and fairly; a broker is not obliged to advise on whether a competitor or an alternative policy term would offer better value, only to price its own panel accurately — where a consumer's own stated circumstances (e.g. an intention to sell the property imminently) make it unlikely she would have chosen a different term even with fuller comparative information, a failure to proactively highlight cheaper alternatives does not cause a compensable loss</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>A recording of the original 2015 sales call — absent, requiring the ombudsman to decide on the balance of probabilities what was most likely said</t>
+        </is>
+      </c>
+      <c r="R23" s="3" t="inlineStr">
+        <is>
+          <t>No call recording existed for the initial 2015 contact; more likely Swinton said only one panel insurer offered the product rather than claiming market exclusivity, since a simple check would have disproved a false exclusivity claim; premium calculation reviewed confidentially and found accurate, reflecting risk plus profit and short-term administrative costs; Miss G renewed on a short-term basis each time because she hoped to sell soon, and even after Swinton withdrew short-term cover she sought another short-term provider rather than accept a cheaper annual Swinton policy — demonstrating she valued the short-term flexibility over price and would not have acted differently with better information</t>
+        </is>
+      </c>
+      <c r="S23" s="3" t="inlineStr">
+        <is>
+          <t>Where a broker complaint alleges a misleading claim of market exclusivity but no call recording exists, assess plausibility against what a reasonable broker would say and what a quick market check would reveal — an exclusivity claim that could be trivially disproved is inherently less likely to have been made; when assessing detriment from an alleged pricing non-disclosure, look at what the consumer's subsequent actual choices reveal about what she would have done with fuller information, not just her stated hindsight preference</t>
+        </is>
+      </c>
+      <c r="T23" s="3" t="inlineStr">
+        <is>
+          <t>IF broker_prices_short_term_unoccupied_property_cover_higher_per_month_than_equivalent_annual_cover AND pricing_methodology_is_shown_to_be_accurate_and_consistently_applied THEN higher_short_term_pricing_is_not_unfair_even_without_proactive_comparison_to_annual_cover; IF consumers_subsequent_choices_show_she_continued_to_prefer_short_term_cover_even_after_being_offered_a_cheaper_annual_alternative THEN broker_failure_to_earlier_highlight_annual_cover_savings_did_not_cause_a_compensable_loss</t>
+        </is>
+      </c>
+      <c r="U23" s="3" t="inlineStr">
+        <is>
+          <t>DRN3390381.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="80" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3516774</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>4 Jul 2022</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Unoccupied Property insurance — escape of water from a loft leak discovered by policyholder's daughter during a routine check; insurer avoided the policy from inception (and separately from renewal) for misrepresentation about intended occupancy, and identified alternative grounds (Water Turn Off Clause breach, 30-day inspection condition breach) that would likely also have defeated the claim</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Policyholder took out Unoccupied Property insurance in December 2019 while working abroad for about a year; Statement of Fact recorded the property would become occupied in 9-12 months and was not occupied from inception; at the December 2020 renewal, the Statement of Fact recorded the property had been unoccupied for 'more than 1 year', but the policyholder was in fact staying at the property around that renewal date (returned to the UK November 2020, remained until 5 February 2021) — contrary to the Unoccupied Property policy's definition of 'occupied' as lived in for more than 7 consecutive days</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Residential property intended to be unoccupied while owner worked abroad</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Lloyd's avoided the policy from inception, concluding Mr M hadn't disclosed at the 2019 inception that he intended to occupy the property every 3-4 months for more than 7 days at a time, and separately that the 2020 renewal Statement of Fact incorrectly recorded the property as unoccupied for 'more than 1 year' when he was in fact living there around the renewal date; Lloyd's said it would only have offered a Holiday Home Policy (which excludes escape of water) had accurate information been given</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Mr M: told his broker at inception he'd be working abroad for a year; told the broker at the 2020 renewal he was temporarily occupying the house but was renewing on the basis he was about to leave the UK again; renewed in good faith and the leak occurred while the property was genuinely unoccupied. Lloyd's: no recording exists of either the 2019 inception or 2020 renewal calls; the written Statement of Fact for each year is the best contemporaneous record and recorded (2019) occupation expected in 9-12 months and (2020) unoccupied for 'more than 1 year' — both materially inaccurate given the policy's 7-consecutive-day 'occupied' definition and Mr M's own account of returning every 3-4 months and being present around the 2020 renewal date; an internal business-file note appearing to support Mr M was subsequently clarified by Lloyd's as a typographical error. FOS (provisional and final): without a recording, the Statement of Fact — which Mr M confirmed reading, understanding and agreeing to a disclosure declaration on — is the more reliable record; on that record Mr M did not disclose an intention to occupy for more than 7 days at a time at either inception or renewal, and the 2020 Statement was objectively wrong since his own account showed he was living in the property around the renewal date; this was a careless misrepresentation entitling Lloyd's to avoid the policy under CIDRA; even had the policy been valid, a screen report found the stop cock may not have been fully closed (Water Turn Off Clause breach) and there was no record of the required 30-day inspections, either of which would likely also have defeated the claim</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Lloyd's fairly avoided the policy from inception for careless misrepresentation about intended and actual occupancy, and correctly declined the claim; premiums for both policy years were refunded, which was fair</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>An Unoccupied Property policy defining 'occupied' as lived in for more than 7 consecutive days is designed specifically to exclude anyone who intends, or turns out, to stay at the property for extended periods — a policyholder's own evidence that they intended to return every 3-4 months for stays exceeding 7 days, or that they were actually staying at the property around a renewal date, is itself sufficient to show the Unoccupied Property policy was unsuitable and that a misrepresentation as to occupancy occurred; where no recording exists of a sales or renewal call, a written Statement of Fact that the policyholder has confirmed reading, understanding and agreeing to (as part of a CIDRA-compliant disclosure declaration) is the more reliable contemporaneous record of what was disclosed, and will generally be preferred over a policyholder's later recollection where the two conflict; for a misrepresentation to justify avoidance under CIDRA, the insurer must show it is a qualifying misrepresentation — i.e., that accurate disclosure would have changed whether or on what terms cover was offered — and an insurer's evidence that it would only have offered a different product (here, a Holiday Home Policy excluding escape of water) satisfies this</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>Recordings of the 2019 inception call and the 2020 renewal call — neither was available, requiring reliance on the Statements of Fact as the best contemporaneous written record</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>2019 Statement of Fact recorded the property not occupied from inception and expected to become occupied in 9-12 months; this is inconsistent with Mr M's claimed intention (later stated) to return every 3-4 months for over 7 days at a time; 2020 renewal Statement of Fact recorded unoccupied for 'more than 1 year', but Mr M's own account confirmed he was staying at the property from November 2020 until 5 February 2021, spanning the December 2020 renewal date — objectively incorrect; Lloyd's underwriters confirmed they would not have offered the Unoccupied Property product (or would have offered a Holiday Home Policy instead) had accurate information been given, satisfying the qualifying misrepresentation test under CIDRA; fair for Lloyd's to avoid the policy at both inception and renewal and decline the claim, while returning all premiums paid; additionally, the stop cock may not have been fully closed and 30-day inspection records were unavailable, either of which would likely have independently defeated the claim even absent misrepresentation</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>When assessing a suspected misrepresentation about intended occupancy for an Unoccupied Property policy, compare the policyholder's own account of their actual movements (dates present at the property) against the policy's numeric 'occupied' definition (e.g. more than 7 consecutive days) — a policyholder's own narrative can itself supply the evidence of misrepresentation without need for a call recording; renewal Statements of Fact should be checked against events the policyholder has independently confirmed (e.g. return travel dates) since a renewal declaration can become inaccurate due to intervening circumstances (such as pandemic travel restrictions) even if accurate at a prior renewal; where alternative independent grounds for declining a claim exist (e.g. a specific safety condition breach), documenting these strengthens the fairness of an avoidance decision even where the primary ground is misrepresentation</t>
+        </is>
+      </c>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>IF unoccupied_property_policy_defines_occupied_as_lived_in_for_more_than_N_consecutive_days AND policyholders_own_account_shows_they_were_present_at_the_property_for_periods_exceeding_N_days_around_inception_or_renewal THEN this_is_evidence_of_a_qualifying_misrepresentation_about_intended_or_actual_occupancy_justifying_avoidance; IF no_call_recording_exists_for_inception_or_renewal THEN a_statement_of_fact_the_policyholder_confirmed_reading_and_agreeing_to_is_the_preferred_contemporaneous_record_over_later_recollection; insurer_avoiding_policy_for_misrepresentation_must_show_it_would_have_offered_different_terms_or_a_different_product_if_accurately_informed_to_satisfy_the_qualifying_misrepresentation_test</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3516774.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="80" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-024</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>DRN3646077</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Adrian Flux Insurance Services Group</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>3 Nov 2019</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Broker mis-sale complaint — buildings insurance for an inherited unoccupied property; escape of water from a burst loft pipe in March 2018 declined because the property wasn't kept heated above 15°C (or mains drained) during the winter exclusion period; executors/solicitor-representative said they were unaware of this requirement</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Property inherited January 2017, stood empty while the estate was administered; unoccupied buildings cover arranged through the broker, renewed January 2018; water supply remained connected but heating was turned off during the relevant winter period</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Residential property, unoccupied pending estate administration</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable to a coverage decline — dispute concerned whether the broker adequately notified the policyholders' representative (AL) of the winter heating/mains-drain condition, not whether the insurer correctly applied it</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>AL (executors' solicitor): unaware of the 15°C heating/mains-drain requirement at inception or renewal; would have kept the heating on had they known. Flux: the requirement was clearly set out as an 'Additional Notes' item in the January 2017 quotation ('Important Information' section) sent the day before AL phoned to accept the policy, and repeated in the same location in the January 2018 renewal documentation; AL confirmed on the renewal call that he was happy with the terms and conditions. FOS: the clause itself is not unusual for an unoccupied property policy (it mitigates a well-known frost-damage risk) but the requirement to maintain constant heating for five winter months is onerous, so it needed to be clearly notified — it was clearly highlighted, in the same place, at both the original quotation stage and the renewal stage, and AL confirmed acceptance of terms and conditions on the renewal call; Flux was entitled to assume the policy was purchased after AL read and agreed to that information</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Flux did enough to clearly highlight the onerous winter heating/mains-drain condition at both inception and renewal; it was not responsible for the reduced property sale price</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="inlineStr">
+        <is>
+          <t>A winter escape-of-water exclusion for unoccupied properties, requiring either mains water to be turned off and drained or the property to be kept heated at a minimum temperature (e.g. 15°C) throughout a defined winter period, is not itself an unusual clause for this type of policy since it mitigates a well-recognised frost-damage risk — but the heating-maintenance option is an onerous condition (given the potential cost of five months' continuous heating) and so must be clearly notified to the policyholder or their representative; specifically highlighting the requirement in an 'Important Information' or equivalent section of both the original quotation and each renewal document, in the same consistent location, is sufficient to discharge the broker's duty to notify — even where the same wording is not repeated in every subsequent communication (e.g. the policy schedule itself)</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>Evidence that AL specifically read the 'Additional Notes' section of the quotation and renewal documents — not directly available, but AL's acceptance of the policy the day after receiving the quotation, and his confirmation of being happy with 'terms and conditions' on the renewal call, supported an inference that the notification had been received and accepted</t>
+        </is>
+      </c>
+      <c r="R25" s="3" t="inlineStr">
+        <is>
+          <t>Clause required mains off/drained or heating maintained at 15°C from 1 November to 31 March; turning mains off is not onerous but constant heating for five months is; clause was set out clearly under 'Additional Notes'/'Important Information' at both the January 2017 quotation (a day before AL accepted the policy by phone) and the January 2018 renewal documentation (in the 'Excesses, endorsements and conditions' section); AL confirmed on the renewal call he was happy with the terms and conditions; taken together this was sufficient to discharge Flux's duty to notify AL of the condition at both inception and renewal; Flux therefore not responsible for the declined claim or the reduced property sale price</t>
+        </is>
+      </c>
+      <c r="S25" s="3" t="inlineStr">
+        <is>
+          <t>For onerous winter heating/mains-drain conditions on unoccupied property policies, brokers should highlight the condition in a consistently-located 'Important Information' or 'Additional Notes' section at both initial quotation and every renewal — doing so in the same place each time, combined with a policyholder's acceptance of 'terms and conditions' on a renewal call, is generally sufficient evidence of adequate notification even without the condition being separately repeated in every other communication (e.g. the policy schedule or a covering email)</t>
+        </is>
+      </c>
+      <c r="T25" s="3" t="inlineStr">
+        <is>
+          <t>IF onerous_winter_heating_or_mains_drain_condition_is_clearly_set_out_in_a_consistently_located_important_information_section_at_both_quotation_and_each_renewal AND policyholder_or_representative_confirms_acceptance_of_terms_and_conditions_on_the_renewal_call THEN broker_has_discharged_its_duty_to_notify_the_condition_even_if_not_repeated_in_every_other_document; unoccupied_property_winter_escape_of_water_conditions_requiring_mains_off_or_maintained_heating_are_not_unusual_but_the_heating_maintenance_option_is_onerous_and_must_be_clearly_highlighted</t>
+        </is>
+      </c>
+      <c r="U25" s="3" t="inlineStr">
+        <is>
+          <t>DRN3646077.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="80" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3848349</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>T&amp;R Direct Ltd</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>10 Mar 2023</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Broker mis-sale complaint — unoccupied property owner's policy arranged (non-advised, per the broker) for a property undergoing renovation; theft of new kitchen appliances (still boxed, delivered but not yet installed) declined because the policyholder had selected 'standard' cover (fire/lightning/explosion/aircraft only) on the proposal form and had not opted for the available theft extension</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Property unoccupied and undergoing renovation from around June 2021; theft of appliances occurred December 2021 while the property remained empty pending completion of works</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Residential property under renovation (unoccupied)</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable to a coverage decline by the insurer — the underlying theft coverage decision was the subject of a separate complaint; this complaint concerned only whether the broker's conduct in arranging the policy amounted to a mis-sale</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Mr F: expected the new policy to match his previous (occupied) contents cover; felt T&amp;R had sent him a 'misleading and poorly structured' proposal form and effectively directed him to take the policy without adequately explaining that 'standard' cover excluded theft, a major exclusion; his own insurance adviser considered a policy clause showed theft was included and that T&amp;R should have highlighted theft as a major exclusion. T&amp;R: the proposal form clearly defined 'standard' cover (fire/lightning/explosion/aircraft only) and offered a separate theft extension Mr F did not select; the policy was arranged on a non-advised basis — Mr F completed and signed the form himself, and a recorded call showed he had actively turned his mind to security, stating there was 'nothing of substantial value' left at the property besides office equipment, furniture and books, locked in a third-floor room. FOS: the policy itself was not inherently unsuitable — it did provide unoccupied-property cover and a theft extension was available; Mr F made clear, hand-written elections on the form for a new and different type of policy; the word 'only' in the standard-cover definition emphasised its limits; Mr F was capable and engaged (adding handwritten comments, asking specific questions about excess and financial cover) but did not ask about theft; the sale was non-advised since no cover-level advice was given and the declaration/documentation did not indicate an advised sale; it would have been better practice for T&amp;R to flag at the point of claim that theft cover hadn't been selected, but this did not amount to mis-sale or attract compensation</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — T&amp;R didn't mis-sell the policy; it was arranged on a non-advised basis, the proposal form clearly defined the standard cover limits and offered a theft extension Mr F chose not to select, and Mr F's own engagement with the form and call showed an informed choice</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>Where an unoccupied property owner's policy proposal form clearly defines 'standard' cover as limited to specific perils (e.g. 'fire, lightning, explosion, aircraft only') and separately offers an optional theft extension that the policyholder does not select, a broker arranging the policy on a non-advised basis is not required to specifically flag that theft is excluded from standard cover — the onus falls on the consumer to review the cover options and select accordingly, particularly where the policyholder's own recorded comments show they turned their mind to the security of contents at the property; a sale is non-advised where the broker does not recommend specific cover-level choices and the policyholder independently completes and signs the proposal form; it would be good practice, though not a mis-sale, for a broker to flag at the point of a claim that a relevant extension wasn't selected, to manage the policyholder's expectations before the insurer's claims decision</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>Clear evidence that Mr F specifically requested theft cover matching his previous occupied-property policy — absent; his own recorded comments about there being 'nothing of substantial value' at the property were, if anything, evidence he had actively (if perhaps mistakenly) turned his mind away from needing theft cover</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>Proposal form clearly defined standard cover (fire/lightning/explosion/aircraft 'only') separately from an extended-cover option that included theft, which Mr F did not tick; recorded call showed Mr F actively considered and downplayed the value of contents left at the property; Mr F engaged meaningfully with the form (handwritten comments, specific questions on excess and financial cover level) but not on theft; sale was non-advised — no cover-level recommendation from T&amp;R, form completed and signed by Mr F, declaration onus on him to check completeness/accuracy or consult an adviser if in doubt; T&amp;R could have done more at the claims stage to flag the missing theft cover but this is a best-practice observation, not a basis for compensation or a mis-sale finding</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>For non-advised sales of unoccupied property owner's policies, brokers should still consider flagging, at the point a claim is first reported, whether the relevant peril extension was selected on the original proposal — this manages the policyholder's expectations and avoids unnecessary distress even where it is not required to avoid a mis-sale finding; a policyholder's own recorded statements about the value or nature of contents at a property can be persuasive evidence that they made an informed (if potentially mistaken) choice not to select an available cover extension</t>
+        </is>
+      </c>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>IF proposal_form_clearly_defines_standard_cover_perils_and_separately_offers_an_optional_extension_covering_the_peril_later_claimed_for AND policyholder_completed_and_signed_the_form_without_broker_recommendation_on_cover_level THEN sale_is_non_advised_and_broker_is_not_liable_for_policyholder_not_selecting_the_extension; policyholders_own_recorded_statements_about_the_value_of_contents_at_the_property_can_evidence_an_informed_choice_not_to_select_an_available_extension; broker_failing_to_flag_at_claim_stage_that_a_relevant_extension_was_not_selected_is_a_best_practice_gap_not_a_mis_sale</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3848349.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="80" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-026</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>DRN-3999409</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Affinity Insurance Solutions Limited</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>1 May 2023</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Broker mis-sale complaint — home insurance arranged by phone for an inherited unoccupied property; escape of water declined by the underwriter because the property had been unoccupied for more than 60 consecutive days, which the policyholder said she wasn't warned about at the point of sale</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Property inherited following a bereavement in April 2021; insured as unoccupied from inception (June 2021), renewed July 2022; escape of water discovered mid-December 2022 while the property remained unoccupied, though visited regularly by the family for upkeep</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Residential property (inherited, unoccupied)</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable to a coverage decline by the underwriter directly — this complaint concerned whether the broker adequately explained the 60-day unoccupied-property escape-of-water exclusion at the point of sale, not the underwriter's application of it</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Mrs K (via her husband, who arranged the policy on her behalf): wasn't made aware an escape of water wouldn't be covered if the property was unoccupied for more than 60 consecutive days; both she and her husband were vulnerable at the time, dealing with bereavement, grief and ill health. Affinity: its call handler told Mr K on at least two occasions during the sales call that a restriction applied to cover where a property was unoccupied for more than 60 consecutive days, and Mr K confirmed 'that's fine' and proceeded; the subsequent 46-page policy booklet, sent by email, also clearly set out the exclusion and advised the policyholder to check the cover was right for her, consistent with a non-advised sale. FOS (having listened to the recorded call): the restriction was clearly stated at least three times during the call and Mr K confirmed acceptance each time; the policy documentation was significantly more detailed than what was said on the call (a 46-page booklet, not unusual) and clearly excluded EOW after 60 days' unoccupancy — a common feature of unoccupied-property policies generally; Mrs K had a cooling-off period to review and cancel if the cover wasn't suitable; while sympathetic to the bereavement and ill health, there wasn't enough evidence that the couple's circumstances precluded understanding the clearly-stated restriction</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Affinity clearly explained the 60-day unoccupied-property restriction on the recorded sales call (at least three times) and in the subsequent policy documentation; the policy was not mis-sold</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P27" s="3" t="inlineStr">
+        <is>
+          <t>Where a call recording shows an unoccupied-property time-limited exclusion (e.g. 60 consecutive days for escape of water) was clearly stated multiple times during a sales call and acknowledged by the person arranging the policy, and the subsequent policy documentation also clearly sets out the same restriction, a broker has discharged its duty to provide clear, fair and not misleading information — this remains the case even where the policy was arranged by a family member on behalf of a vulnerable consumer affected by bereavement and ill health, provided there's no evidence the vulnerability precluded understanding what was communicated at the time; a cooling-off period during which the policyholder could review documentation and cancel without penalty is a further opportunity for the consumer to identify unsuitable terms, reducing the broker's residual responsibility</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>Evidence that Mr and Mrs K's vulnerability (grief, ill health) at the time of the June 2021 sales call was so severe as to preclude understanding the restriction that was repeated multiple times and expressly acknowledged — absent</t>
+        </is>
+      </c>
+      <c r="R27" s="3" t="inlineStr">
+        <is>
+          <t>Recorded call (good quality, provided to Mrs K in the interests of candour) showed the 60-day unoccupied restriction stated at least three times, with Mr K responding 'that's fine' and confirming he was happy to proceed; 46-page policy booklet (not unusually long) and covering letter advising the policyholder to check cover was 'right for you' were sent after inception; this pattern is consistent with a non-advised sale where the onus fell on Mrs K to review the documentation; while sympathetic to the family's grief and Mr K's evident concern for his wife's wellbeing, there was no evidence their circumstances prevented them from understanding a restriction repeated multiple times on the call; not mis-sold</t>
+        </is>
+      </c>
+      <c r="S27" s="3" t="inlineStr">
+        <is>
+          <t>When a family member arranges an unoccupied-property policy on behalf of a bereaved or vulnerable consumer, a broker's obligations are assessed against what was communicated to the person actually on the call and in subsequent documentation — repeating a material time-limited exclusion multiple times during the call and echoing it in the policy booklet, combined with a cooling-off period, is strong evidence of a fair sale even in circumstances of bereavement, absent specific evidence that the vulnerability itself impaired understanding of what was said at the time</t>
+        </is>
+      </c>
+      <c r="T27" s="3" t="inlineStr">
+        <is>
+          <t>IF recorded_sales_call_shows_time_limited_unoccupied_property_exclusion_stated_multiple_times_and_acknowledged_by_the_person_arranging_the_policy AND subsequent_policy_documentation_also_clearly_sets_out_the_same_exclusion THEN broker_has_provided_clear_fair_and_not_misleading_information_regardless_of_the_policyholders_bereavement_or_vulnerability_absent_specific_evidence_the_vulnerability_impaired_understanding_at_the_time; cooling_off_period_availability_further_reduces_broker_residual_responsibility_for_a_clearly_disclosed_unoccupancy_restriction</t>
+        </is>
+      </c>
+      <c r="U27" s="3" t="inlineStr">
+        <is>
+          <t>DRN-3999409.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="80" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>DRN4133004</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>St Andrew's Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>16 Oct 2019</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Buildings insurance — escape of water discovered by policyholder's son (holding power of attorney) during a maintenance visit; property had been empty for around 18 months (owner in a care home) while being maintained/decorated by family with a view to renting or selling; insurer declined citing the 30-day unoccupied exclusion and separately cancelled/backdated the policy to its one-year maximum unoccupied-cover period</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Owner entered a care home in August 2016; property unoccupied thereafter for around 18 months by the time of the February 2018 loss, though visited every other day by family for maintenance and decoration; property retained essential living items (cooking appliances, sanitary fittings, beds)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (owner in care home; family maintaining for future rental or sale)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Escape of water excluded as the property had been unoccupied (not lived in) for more than 30 days; separately, St Andrew's said it would only have insured an unoccupied property for a maximum of one year and so backdated cancellation of the policy to August 2017, refunding premiums paid since then</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Mr G (via his son/attorney): family visited every other day to maintain and decorate the property with a view to letting or selling it, so it shouldn't be classed as unoccupied; the broker (not St Andrew's) had been told about the change in 2016 and hadn't passed this on or warned of the unoccupancy consequences — a separate complaint. St Andrew's: to meet the policy's 'occupied' definition the property must be lived in by the owner or a family member and contain essential living items; regular maintenance visits, however frequent, are not the same as living there; had it known the property was unoccupied, it would only have covered EOW-type damage if additional risk-reduction steps had been taken (water turned off, regular inspections recorded), and would in any event have limited cover to one year from the start of unoccupancy, consistent with its underwriting notes. FOS: property had the essential items for normal living (satisfying that limb of the definition) but visiting to carry out maintenance, however frequently, does not amount to 'living' there; the water hadn't been turned off, so the breach of the unoccupied-property risk-reduction condition was directly connected to the type of loss claimed (an EOW-prevention measure not taken); backdating cancellation to August 2017 (one year from actual unoccupancy) and refunding premiums paid thereafter was a fair reflection of what St Andrew's would have done had it known the true position at the time</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — St Andrew's fairly declined the EOW claim under the 30-day unoccupied exclusion and fairly cancelled/backdated the policy to its one-year unoccupied-cover maximum, refunding premiums paid after that date</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>An 'occupied'/'lived in' definition requiring both (a) actual habitation by the owner or an authorised family member and (b) the presence of essential items for normal living (cooking appliances, sanitary fittings, beds) is a conjunctive test — satisfying the furnishing limb alone does not meet the definition if no one is actually living there; family members visiting every other day to carry out maintenance or decoration, however frequently, does not constitute 'living' in a property for this purpose; where an insurer's maximum unoccupied-property cover period (e.g. one year) is a documented underwriting practice, it is fair for the insurer to backdate a cancellation to the actual date unoccupancy began (as established by the evidence) once it discovers the true position, and to refund premiums paid for the period it would not otherwise have covered; a breach of a risk-reduction condition specific to unoccupied properties (e.g. failing to turn off the water supply) is materially connected to, and can bar, a claim for the very type of damage (escape of water) that the condition was designed to prevent</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>Evidence that the water supply had been turned off, or an alternative continuous-heating arrangement maintained, during the unoccupied period — absent; this breach was directly connected to the escape of water loss</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>Property contained essential living items but was only visited, not lived in, by family members carrying out maintenance and decoration over roughly 18 months; the 'occupied' definition requires both limbs to be met and 'living in' was not established by visits alone; had St Andrew's known of the unoccupancy it would only have covered EOW-type losses subject to additional conditions (water off, regular recorded inspections) which were not met, and the failure to turn off the water was directly connected to the loss claimed; St Andrew's underwriting notes confirmed a one-year maximum unoccupied-cover policy, so backdating cancellation to August 2017 (the true start of unoccupancy) and refunding premiums paid since was the fair outcome reflecting what would have happened had it been told at the time; broker's alleged failure to pass on notification was a separate matter not attributable to St Andrew's</t>
+        </is>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>When assessing an 'occupied'/'lived in' definition requiring both habitation and essential furnishing, confirm both limbs separately — a well-furnished, well-maintained property is not thereby 'occupied' if no one is actually residing there; regular family visits for maintenance or decoration purposes should be distinguished from residence when assessing unoccupancy thresholds; where an insurer discovers post-loss that a property was unoccupied for longer than its maximum unoccupied-cover period, backdating cancellation to the actual (not notified) start date of unoccupancy and refunding the resulting unearned premium is a fair remedy, provided supported by documented underwriting practice</t>
+        </is>
+      </c>
+      <c r="T28" s="2" t="inlineStr">
+        <is>
+          <t>IF policy_occupied_definition_requires_both_actual_habitation_AND_presence_of_essential_living_items AND only_the_furnishing_limb_is_satisfied THEN property_is_not_occupied_for_policy_purposes_regardless_of_frequency_of_maintenance_visits; IF insurer_has_a_documented_maximum_unoccupied_cover_period AND discovers_post_loss_that_property_exceeded_that_period THEN backdating_cancellation_to_the_actual_start_of_unoccupancy_and_refunding_premiums_paid_thereafter_is_a_fair_remedy; breach_of_an_unoccupied_property_risk_reduction_condition_directly_connected_to_the_type_of_loss_claimed_bars_the_claim</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>DRN4133004.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="80" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-028</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>DRN-4195324</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Accredited Insurance (Europe) Ltd</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>22 Aug 2023</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — water leak claim; insurer investigated and concluded the policyholder didn't actually live at the insured property (contrary to what was declared as her main residence), avoided the policy for deliberate/reckless misrepresentation, and separately suggested the claim would also be excluded under an unoccupancy condition</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Insurer's investigator concluded the property wasn't the policyholder's main residence and may have been used for business purposes or otherwise unoccupied for a period before the water damage was discovered (evidenced, it said, by mould growth and discrepancies over when the loss occurred) — but the ombudsman found the insurer's occupancy investigation itself was flawed and unproven</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Residential property (occupancy status disputed)</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Accredited avoided the policy (treated it as if it never existed) on the basis that Miss V had misrepresented that the property was her main residence, which it said was a deliberate/reckless qualifying misrepresentation entitling it to refuse all claims; it separately argued that even if the policy were valid, the claim would be excluded under the unoccupancy condition given delay in the damage being discovered</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Miss V: disputed the investigator's conclusions about where she lived and the fairness/conduct of the investigation (including an allegation of bullying during an interview). Accredited: its investigator compared her circumstances to another property it believed she lived at, and relied on a neighbour's account and inconsistencies it identified; said it wouldn't have offered a household policy had it known the property wasn't her main residence, and that even if cover existed, unoccupancy (evidenced by mould growth and timeline discrepancies) would exclude the claim. FOS (provisional and final): repeatedly asked Accredited to justify its investigation methodology and to produce its underwriting criteria to show the alleged misrepresentation was a 'qualifying' one under CIDRA (i.e., that it would have changed whether or on what terms cover was offered); Accredited initially said it couldn't access its underwriting information, then supplied a document that turned out not to be the underwriting criteria, and only after repeated requests produced its actual underwriting guide and endorsements; that document's list of decline reasons did not include unoccupancy, its general guidelines said it would cover most non-standard risks including unoccupied properties, and none of the unoccupied-property endorsements referenced said cover would be declined outright (some referred to reduced cover and protective measures only); Accredited therefore failed to show the alleged misrepresentation was a qualifying one, and also failed to justify the reasonableness of its occupancy investigation itself</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Accredited required to remove references to the policy avoidance from internal and external databases, reinstate the policy, consider the claim, and pay Miss V £200 compensation</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>To avoid a policy for misrepresentation under CIDRA, an insurer must show not only that the policyholder failed to take reasonable care in answering a question (e.g. about main residence status) but also that the misrepresentation was a 'qualifying' one — meaning the insurer would have offered the policy on different terms, or not at all, had accurate information been given; an insurer's unoccupancy-related underwriting guidance that identifies reduced cover and protective measures (rather than outright decline) for unoccupied or non-standard-occupancy properties undermines a claim that a misrepresentation about occupancy/residence status was 'qualifying' in the CIDRA sense; an insurer relying on avoidance for misrepresentation bears the burden of promptly producing its actual underwriting criteria to substantiate that claim — repeated failure or delay in producing this evidence, or producing the wrong document, undermines the insurer's position and supports a finding against it</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>Accredited's genuine underwriting criteria — initially claimed unavailable, then a non-underwriting document was supplied, and only after repeated requests was the correct document produced; even then, it did not support the claim that the alleged misrepresentation was a qualifying one</t>
+        </is>
+      </c>
+      <c r="R29" s="3" t="inlineStr">
+        <is>
+          <t>Multiple issues identified with how Accredited investigated occupancy (including the investigator personally following up a bullying allegation raised against himself), and Accredited did not adequately justify the conclusions reached; even setting aside the reasonable-care question, Accredited failed — despite repeated requests and after supplying an incorrect document — to show the misrepresentation was a qualifying one; the underwriting guide's list of decline reasons did not include unoccupancy, its general position was to cover most non-standard risks including unoccupied properties, and none of the referenced unoccupied-property endorsements provided for outright decline; therefore avoidance and claim decline were not reasonable; a related, not-yet-actioned suggestion that endorsements might have been applied for unoccupancy was irrelevant since that action was never actually taken</t>
+        </is>
+      </c>
+      <c r="S29" s="3" t="inlineStr">
+        <is>
+          <t>When an insurer relies on misrepresentation to avoid a policy connected to disputed occupancy or residence status, it must be prepared to promptly produce its actual underwriting criteria to demonstrate the misrepresentation was 'qualifying' — repeated failure to do so, or supplying incorrect documents, will be treated as undermining the insurer's position rather than neutral; underwriting guidance that provides for reduced cover or protective conditions (rather than outright decline) for unoccupied or non-standard-occupancy properties is strong evidence against a claim that misrepresenting occupancy status was a qualifying misrepresentation; claims investigations into disputed occupancy should not be conducted or self-validated by the same individual against whom a conduct complaint (e.g. bullying) has been raised</t>
+        </is>
+      </c>
+      <c r="T29" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_avoids_policy_for_misrepresentation_about_occupancy_or_residence_status AND insurer_cannot_promptly_produce_underwriting_criteria_showing_the_misrepresentation_would_have_changed_terms_or_offer THEN avoidance_is_not_a_qualifying_misrepresentation_under_cidra_and_should_not_be_upheld; IF underwriting_guidance_for_unoccupied_or_non_standard_occupancy_properties_provides_for_reduced_cover_or_protective_conditions_rather_than_outright_decline THEN this_undermines_a_claim_that_misrepresenting_occupancy_status_was_a_qualifying_misrepresentation; insurer_repeatedly_failing_to_produce_or_misidentifying_its_own_underwriting_document_when_requested_weighs_against_the_insurers_position</t>
+        </is>
+      </c>
+      <c r="U29" s="3" t="inlineStr">
+        <is>
+          <t>DRN-4195324.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="80" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>DRN4242877</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Stride Limited</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>25 Oct 2018</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Broker mis-sale complaint — home insurance for an empty property; vandalism damage claim (paint splashed from an incident targeting a neighbour's car) attracted a £1,000 increased excess for unoccupied-property risks (theft, vandalism, malicious damage, accidental damage) under the policy; policyholders felt the policy had been mis-sold as unsuitable for an unoccupied property, though the insurer reduced the excess to £100 given the collateral nature of the damage and the small claim (£300) was not pursued</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Property already unoccupied for some time when the policy was taken out in November 2017, as recorded on the statement of fact</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Residential property, unoccupied</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable to a coverage decline — the underlying vandalism claim was not declined (a reduced £100 excess was offered and the claim, worth £300, was simply not pursued by the policyholders); the complaint concerned whether the policy itself was mis-sold as unsuitable for an unoccupied property</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Mr and Mrs H: believed the policy became entirely invalid after 45 days' unoccupancy, and hadn't received the policy wording until after the claim, making it an unsuitable/mis-sold policy. Stride: statement of facts and policy schedule (with a link to the full policy wording) were emailed at inception and referenced by Mr and Mrs H in their own correspondence, so were likely received; the schedule itself stated cover for certain losses (theft, vandalism, malicious damage, accidental damage) while unoccupied for more than 45 days continued but with an increased £1,000 excess, not that cover was withdrawn entirely; this was the most competitive policy Stride could source for an unoccupied property. FOS: the policy schedule made clear the property was insured as unoccupied and that certain risks carried a higher excess (not exclusion) after 45 days — so the policy was not invalid or unsuitable for an unoccupied property, contrary to Mr and Mrs H's belief; even accepting they weren't specifically told about the increased excess in advance, the increased excess and inspection/drain-down conditions are common unoccupied-property policy terms, and it was unlikely they'd have obtained materially better terms elsewhere at a comparable price</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — the policy was a suitable, valid unoccupied-property policy (not invalidated after 45 days, merely subject to an increased excess for certain perils); no mis-sale established and no refund or claim-record amendment required</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>An unoccupied-property home insurance policy that imposes an increased excess (rather than a blanket exclusion) for certain perils such as theft, vandalism, malicious damage and accidental damage once the property has been unoccupied for more than a stated period (e.g. 45 days) remains a valid and suitable policy for an unoccupied property — a policyholder's mistaken belief that the policy became wholly invalid after that period does not, without more, establish mis-sale; an increased excess and standard unoccupied-property conditions (regular inspection, mains drain-down over winter) are common industry terms, and a broker is not required to show it could have sourced materially better terms at a comparable price to defeat a suitability complaint</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>Clear evidence Mr and Mrs H did not in fact receive the statement of facts and policy schedule (with link to policy wording) at inception — undermined by their own correspondence referencing that document, and by the absence of any record of them chasing Stride for a missing link to the full wording</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>Statement of facts and schedule sent by email at inception and referenced by the policyholders themselves; schedule clearly stated the property was unoccupied and that certain perils carried an increased £1,000 excess (not exclusion) once unoccupied more than 45 days — this contradicted the policyholders' belief that the policy became entirely invalid; even assuming they weren't specifically warned of the increased excess in advance, the terms were common for this type of policy and it was unlikely a materially better-value alternative existed; the insurer's willingness to reduce the excess to £100 given the collateral nature of the damage, and the policyholders' own decision not to pursue the £300 claim, meant there was no declined claim to remedy; no basis to require a premium refund or claim-record amendment since the policy remained valid throughout</t>
+        </is>
+      </c>
+      <c r="S30" s="2" t="inlineStr">
+        <is>
+          <t>When a policyholder alleges an unoccupied-property policy is invalid or unsuitable because of a time-triggered condition, check whether that condition is actually an exclusion (no cover at all) or merely an increased excess/reduced-scope condition (cover continues, on different terms) — many unoccupancy complaints stem from this misunderstanding rather than an actual coverage gap; where a small claim is voluntarily not pursued because a reduced excess still exceeds the claim value, this should not be treated as an unresolved declined claim when assessing a related mis-sale complaint</t>
+        </is>
+      </c>
+      <c r="T30" s="2" t="inlineStr">
+        <is>
+          <t>IF unoccupied_property_policy_schedule_states_certain_perils_carry_an_increased_excess_rather_than_exclusion_after_a_stated_unoccupancy_period THEN policy_remains_valid_and_suitable_for_an_unoccupied_property_and_is_not_thereby_mis_sold; policyholder_mistaken_belief_that_a_time_triggered_excess_increase_equals_total_policy_invalidity_does_not_by_itself_establish_broker_mis_sale; IF policyholder_voluntarily_declines_to_pursue_a_small_claim_because_the_reduced_excess_exceeds_the_claim_value THEN this_is_not_a_declined_claim_requiring_remedy_in_a_related_mis_sale_complaint</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>DRN4242877.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="80" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-030</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>DRN-4660265</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Amtrust Europe Limited</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>3 May 2024</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Holiday homes property owners insurance — escape of water claim; insurer asked the policyholder (a property business) to provide evidence of compliance with the policy's unoccupied-property endorsement (including that the water supply was turned off at the mains, or heating maintained) before considering the claim further, since it believed the property may not have been lived in throughout the run-up to the loss, spanning a switch from an unoccupied property policy to a holiday home owners policy</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Property let to a company that appeared to intend renting it out via Airbnb, under a lease/arrangement commencing before the November 2022 policy switch; insurer's loss adjusters found evidence the property may not have been lived in at any point between that arrangement starting and the mid-December 2022 escape of water; policyholder argued the 30-consecutive-day unoccupancy clock should only start running from the November 2022 policy inception date, not before</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Holiday home / rental property (occupancy status disputed around a policy switch)</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable to a final coverage decline — Amtrust had not declined the claim but was requesting evidence of compliance with the unoccupied-property endorsement (or evidence the property had been lived in within the 30 days before the loss) before resuming consideration of the claim</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>G (property business): it was unreasonable to require proof of compliance with the unoccupied endorsement because the 30 consecutive unoccupied days could only reasonably be counted from the date the holiday home owners policy was taken out (30 November 2022), not from any earlier point under the prior unoccupied property policy. Amtrust: the property may not have been lived in at any point since the letting/Airbnb arrangement began, well before the policy switch; the policy wording placed no restriction on when the 30-day unoccupancy count could start, and requiring renewed occupation evidence made sense given the risk the endorsement was designed to guard against continued regardless of which policy was technically in force on a given date. FOS: nothing in the policy wording supported G's argument that the inception date reset the 30-day clock — the endorsement simply requires compliance if the property 'isn't lived in for 30 days or more', with no stated limitation on when that period can start; it would make no sense from a risk-appetite perspective for the 30 days to only start at policy inception, since the underlying risk (an unoccupied property) is unaffected by a mid-run change of insurer or product; it was therefore reasonable for Amtrust to ask G for evidence of occupation in the 30 days before the loss, or compliance with the endorsement (e.g. mains water off, or heating maintained), before resuming its consideration of the claim</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Amtrust acted reasonably in requiring evidence of occupation or endorsement compliance before resuming consideration of the claim; the policy inception date does not reset the 30-day unoccupancy clock</t>
+        </is>
+      </c>
+      <c r="N31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P31" s="3" t="inlineStr">
+        <is>
+          <t>Where a policy's unoccupied-property endorsement is triggered by the property 'not being lived in for 30 days or more' with no wording limiting when that period can start, the count is not reset by the inception date of a new policy or a mid-term switch between policy types (e.g. from an unoccupied property policy to a holiday home owners policy) — the risk the endorsement addresses (an unoccupied property being more vulnerable to loss) exists independently of which specific policy or insurer happens to be on risk at a given moment, so an insurer is entitled to look at the full run of consecutive unoccupied days, including periods before the current policy's inception, when assessing endorsement compliance</t>
+        </is>
+      </c>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>Evidence, at the time of the ombudsman's decision, that the property had been lived in at some point in the 30 days before the 16 December 2022 loss, or that G had complied with the endorsement's requirements (e.g. mains water turned off, or heating maintained at a steady level) — not yet provided by G; the ombudsman noted Amtrust would be expected to resume considering the claim if such evidence were subsequently produced</t>
+        </is>
+      </c>
+      <c r="R31" s="3" t="inlineStr">
+        <is>
+          <t>Property let to a company that appeared to intend Airbnb-style rental from before the November 2022 policy switch; Amtrust's loss adjusters found evidence the property may not have been lived in at any point during that arrangement; G's argument that the policy inception date restarts the 30-day unoccupancy clock is not supported by anything in the policy wording, and makes no sense in terms of the insurer's risk appetite, since the underlying unoccupancy risk is unaffected by which policy is technically on risk on a given date; therefore reasonable for Amtrust to ask for evidence of occupation or endorsement compliance (mains water off/heating maintained) before resuming consideration of the claim; complaint not upheld, but the claim itself remains open pending that evidence</t>
+        </is>
+      </c>
+      <c r="S31" s="3" t="inlineStr">
+        <is>
+          <t>When a property changes insurer or policy type (e.g. switching from an unoccupied property policy to a holiday home owners policy) without a change in actual physical occupancy, claims handlers assessing a subsequent unoccupancy-endorsement question should look at the full continuous run of unoccupied days across the switch, not just days since the current policy's inception — a policyholder cannot rely on a policy switch to reset an unoccupancy clock where there was no actual change in whether the property was being lived in; where a claim is not yet formally declined but is paused pending evidence of a condition (such as endorsement compliance), this should be recorded as an open evidentiary request rather than a coverage decision</t>
+        </is>
+      </c>
+      <c r="T31" s="3" t="inlineStr">
+        <is>
+          <t>IF unoccupied_property_endorsement_is_triggered_by_property_not_being_lived_in_for_N_or_more_consecutive_days AND policy_wording_places_no_limitation_on_when_that_period_can_start THEN the_count_includes_days_before_the_current_policys_inception_and_is_not_reset_by_a_mid_run_policy_or_insurer_switch; IF property_changes_insurer_or_product_type_without_any_actual_change_in_physical_occupancy THEN insurer_may_require_evidence_of_occupation_or_endorsement_compliance_covering_the_full_continuous_unoccupied_period_not_just_the_period_since_the_current_policys_inception</t>
+        </is>
+      </c>
+      <c r="U31" s="3" t="inlineStr">
+        <is>
+          <t>DRN-4660265.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete unoccupied property case database extraction
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Unoccupied_Property_Case_Database.xlsx
+++ b/knowledge/case-databases/Unoccupied_Property_Case_Database.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3761,6 +3761,3156 @@
         </is>
       </c>
     </row>
+    <row r="32" ht="80" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4825238</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>27 Jun 2024</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Home insurance — property inherited from the policyholder's late father and insured while unoccupied pending probate and sale; escape of water from a burst cold-water loft pipe; insurer declined citing breach of a policy endorsement requiring either the water turned off/drained or the central heating kept running continuously at a minimum of 15°C</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Property inherited October 2022 following the father's death; taken out on a specific policy to cover the unoccupied property pending probate and sale; escape of water discovered December 2022 from a burst lagged cold-water pipe in a sealed loft space above 300mm of insulation</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (inherited, unoccupied pending probate/sale)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Policyholder hadn't complied with the policy endorsement requiring the water to be turned off/drained or the central heating run continuously at a minimum of 15°C; utility bills indicated usage too low to have sustained that temperature</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Mr W: wasn't made aware of the endorsement at the point of sale (Aviva accepted this) and only received notice of it in a letter sent weeks later, which he says he never received; the burst pipe was a cold-water feed in a sealed loft above 300mm of insulation, and his plumber said it would have burst regardless of the house's heating level since the insulation was designed to stop residual heat reaching the loft. Aviva: the depth of loft insulation was irrelevant to the required heating setting, and it would not have changed the outcome of the claim even had the insurer known about it in advance. FOS: accepted the endorsement was breached, but found Aviva had provided no evidence connecting that breach to the specific loss — the purpose of loft insulation is to keep heat inside the house below it, so the pipe above the insulation would likely have frozen and burst regardless of whether the heating was kept at 15°C</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Aviva required to cash-settle the claim in line with the policy's terms and conditions, add 8% simple interest from the date the claim was declined to the date of settlement, and pay Mr W £400 for distress and inconvenience</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>It is unreasonable for an insurer to decline a claim for breach of a policy condition or endorsement (such as a minimum-heating or mains-off requirement for an unoccupied property) unless it can show the circumstances of the claim are actually connected to that breach — an insurer's assertion that a factor (e.g. loft insulation depth) was irrelevant to the required heating setting does not, by itself, establish that maintaining the required temperature would have prevented the specific loss claimed</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>Evidence from Aviva that keeping the heating at the required 15°C would have prevented the cold-water loft pipe from freezing and bursting — not provided, despite being asked to comment specifically on this point</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>Aviva acknowledged Mr W wasn't told about the endorsement when he took out the policy by phone, and the letter notifying him of it wasn't recorded as received; energy usage suggested heating was on but likely for frost protection rather than a full 15°C; regardless of awareness, the endorsement was likely breached, but the relevant test is whether the breach was material to the loss — Aviva did not engage with Mr W's point that the burst pipe was in a loft above thick insulation and would have frozen regardless of the house's internal temperature, and provided no evidence to the contrary even when asked directly; not fair to rely on the breach to decline the claim</t>
+        </is>
+      </c>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>When an insurer declines an unoccupied-property escape-of-water claim for breach of a minimum-heating or mains-off endorsement, check whether the loss occurred in a location (e.g. an insulated loft space) where the general heating requirement would not plausibly have prevented the specific failure — an insurer's bare assertion that a factor was 'irrelevant' to its policy requirement is not evidence that the breach caused or contributed to the loss, and the burden remains on the insurer to show that connection</t>
+        </is>
+      </c>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>IF unoccupied_property_claim_is_declined_for_breach_of_a_minimum_heating_or_mains_off_endorsement AND insurer_has_not_shown_the_breach_was_causally_connected_to_the_specific_loss_location_or_mechanism THEN decline_is_not_reasonable_and_claim_should_be_settled_with_interest_and_distress_compensation</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4825238.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="80" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-032</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>DRN-4834556</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>4 Jul 2024</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Property Owners insurance (leasehold flat) — escape of water from a washing machine in the flat above; insurer declined because the insured flat had been unoccupied since December 2021 (no tenant) and the policy provides no escape-of-water peril for unoccupied properties, notwithstanding the leaseholder's regular visits and occasional overnight stays</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Flat untenanted since December 2021 while put up for sale; leaseholder regularly visited and stayed overnight roughly every thirty days, evidenced by diary logs, estate agent visit logs and utility bills showing periodic increased usage, but no one lived there on a continuous basis</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Leasehold flat (unoccupied, up for sale)</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Policy's insured perils for unoccupied properties don't include escape of water, and the flat met the policy's own definition of unoccupied (not lived in by the tenant or an authorised person for more than 30 consecutive days)</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Mr M: provided diary logs, estate agent logs and utility bills showing he and others visited and stayed overnight regularly; relied on general service guidance that a property visited regularly shouldn't be deemed unoccupied. SoL: the policy's own clear definition of unoccupied (not lived in for more than 30 consecutive days) applied regardless of periodic visits, and escape of water simply isn't an insured peril once that threshold is met. FOS: accepted the visit evidence but found a visit roughly every thirty days, even with an overnight stay, doesn't amount to someone living in the property; the general 'regularly visited' guidance on the Service's website only applies where a policy's own wording lacks a clear definition of unoccupied — here SoL's definition was clear, fair and not misleading, so it was correctly applied</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — SoL's clear policy definition of unoccupied was fairly applied, and escape of water is not an insured peril once the flat met that definition</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P33" s="3" t="inlineStr">
+        <is>
+          <t>Where a policy's definition of 'unoccupied' is stated clearly (e.g. not lived in for more than 30 consecutive days by the tenant or an authorised person), this Service will not substitute a broader 'regularly visited' interpretation for it — that general guidance is reserved for cases where the policy wording itself does not clearly define unoccupied; periodic overnight stays roughly once every 30 days do not amount to a property being 'lived in' even where supported by diary logs, third-party visit records and utility bill evidence</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — the visit and overnight-stay evidence was accepted as genuine; the dispute was over whether that pattern met the policy's 'lived in' threshold, not whether the visits occurred</t>
+        </is>
+      </c>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>Mr M's evidence of regular visits and occasional overnight stays was accepted, but the policy's clear 30-consecutive-day definition of unoccupied does not require continuous absence — it requires that no one lives there, and a periodic overnight stay does not meet that bar; the Service's general 'regularly visited' guidance doesn't override a clear contractual definition; SoL was entitled to define what risks it would insure and price accordingly, and had done so clearly here</t>
+        </is>
+      </c>
+      <c r="S33" s="3" t="inlineStr">
+        <is>
+          <t>Distinguish 'regularly visited' from 'lived in' when a policy has its own clear unoccupied definition — periodic overnight stays (e.g. once every 30 days) do not meet a 'lived in' threshold even if they would satisfy this Service's general guidance for policies that lack a clear definition; check the specific policy wording before applying that general guidance</t>
+        </is>
+      </c>
+      <c r="T33" s="3" t="inlineStr">
+        <is>
+          <t>IF policy_defines_unoccupied_clearly_as_not_lived_in_for_more_than_N_consecutive_days AND policyholder_only_visited_or_stayed_overnight_periodically_without_meeting_regular_living_activities THEN property_is_unoccupied_under_the_policy_regardless_of_general_service_guidance_on_regularly_visited_properties</t>
+        </is>
+      </c>
+      <c r="U33" s="3" t="inlineStr">
+        <is>
+          <t>DRN-4834556.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="80" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4891194</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2 Aug 2024</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Home emergency policy (plumbing and drainage) — mains water leak at a property following the policyholder's death; claim was accepted and repairs carried out, but the executor disputed the number of visits and time taken (77 days across five visits) to locate and fix the leak, and claimed related travel, hotel, heating and other consequential costs</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Property unoccupied following the policyholder's death in October 2022; the executor visited periodically to meet engineer appointments; a separate home insurance policy's unoccupied-property terms required the heating to be maintained or the system drained over winter, relevant context for costs claimed but not itself the subject of this complaint</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (unoccupied following owner's death; estate administration)</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Claim Quantum Dispute</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — the leak repair claim itself was accepted and completed; the dispute concerned only the number of visits/time taken and the consequential costs and compensation claimed as a result</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Executor: it should have taken only a couple of days to locate and fix the leak, not 77; sought reimbursement for travel, hotel, heating costs, delay to the property sale/estate administration, and distress. Aviva: accepted the repair should have taken three visits rather than the five that occurred (one of which was missed entirely), and offered £240 compensation plus reimbursement of travel/hotel/food costs for the two unnecessary visits. FOS: given the nature and eventual location of the leak, three visits were likely sufficient and reasonably necessary — five visits (including one missed) was more than should reasonably have been needed, so the two extra visits' costs were properly reimbursable; heating and consequential losses (delayed sale, estate administration costs) fell under a general exclusion for indirect losses in the policy and weren't shown to result from negligence; distress and inconvenience compensation cannot be awarded to the executor personally since the policy wasn't transferred to him and he wasn't an eligible complainant in his own right</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Aviva required to reimburse the executor's travel and hotel costs (with receipts) and pay £37 taxi/bus plus £20 per person per night for each of the two unnecessary visits, and to pay the £240 compensation already offered if not already paid; no further award for heating costs, sale delay, structural damage, or personal distress to the executor</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>No — Quantum Only</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>A general exclusion for consequential or indirect losses (covering only direct costs expressly provided for by the policy, unless caused by the insurer's or its agents'/suppliers' negligence) bars claims for indirect losses such as a delayed property sale or estate administration costs, even where the insurer accepts its own service fell short of the number of visits it says should have been needed; this Service cannot award distress and inconvenience compensation to a complainant who is not an eligible complainant in their own right — an executor acting on behalf of an estate, where the policy was never transferred into their name, cannot personally recover such compensation even where the insurer has offered it</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>Evidence that the leak or the time taken to fix it caused structural damage to the property — none seen</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>The nature of leaks means they can't always be located and fixed in one visit; three visits (Aviva's own estimate) was a reasonable number given the leak's nature and eventual location, so five visits (one missed) was excessive by two; reimbursement of costs tied to those two unnecessary visits was fair, as was the £240 already offered; heating and system-drain requirements for the unoccupied property derived from a separate home insurance policy and would have applied regardless of the leak, so Aviva wasn't responsible for those costs; the general exclusion for indirect losses barred the sale-delay and estate-administration cost claims absent evidence of negligence; the executor, not being an eligible complainant in his own right, could not personally receive distress and inconvenience compensation, though Aviva's already-offered £240 should still be paid to him</t>
+        </is>
+      </c>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>When an executor brings a complaint on behalf of an estate (rather than as a transferred policyholder), distress and inconvenience compensation cannot be awarded to the executor personally, even though direct cost reimbursement (e.g. travel/hotel for excess visits) can still be ordered; assess the reasonable number of visits for a repair against the nature of the specific fault, not the policyholder's expectation of a minimum number</t>
+        </is>
+      </c>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>IF claim_is_accepted_and_dispute_concerns_only_number_of_visits_or_time_taken_to_complete_repairs THEN assess_reasonable_number_of_visits_based_on_nature_of_fault_not_policyholders_expectation; IF complainant_is_an_executor_acting_on_behalf_of_an_estate_and_policy_was_not_transferred_to_them THEN distress_and_inconvenience_compensation_cannot_be_awarded_to_the_executor_personally_though_direct_cost_reimbursement_can_still_be_ordered</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4891194.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="80" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-034</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>DRN-4915511</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>15 Aug 2024</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Holiday home insurance — escape of water from a frozen and burst pipe during winter; insurer declined citing the unoccupied-property exclusion, since the property wasn't 'lived in' within the normal meaning during the winter months and neither the mains-off/drain nor minimum-heating condition had been met</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Holiday home visited only occasionally, including a few days' overnight stay at the start of December 2022, but not lived in per the normal meaning (regular bathing, cooking, sleeping) during the relevant winter months; policy defines unoccupied as insufficiently furnished, or furnished but not lived in for more than 60 consecutive days, or not lived in overnight between 1 November and 31 March</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Holiday home (seasonal, occupancy disputed)</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>Property was unoccupied under the policy definition during the winter exclusion period, and neither the mains-off/drain nor the 15°C minimum-heating condition required for unoccupied-property escape-of-water cover had been met</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>RSA: the property couldn't be let out during winter months and, while Mrs T visited, it wasn't lived in during that period. Mrs T: as a holiday home there will inevitably be times it's unoccupied, and she did stay overnight for a few days at the start of December 2022. FOS: RSA was reasonable to treat the property as unoccupied, since staying occasionally for a few days doesn't amount to regularly carrying out normal living activities (bathing, cooking, sleeping); as neither unoccupied-property condition was met and the proximate cause was identified as a pipe freezing, bursting then thawing, this was material to the claim since compliance with either condition might have prevented the loss</t>
+        </is>
+      </c>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>Coverage decline itself found reasonable; complaint upheld solely for poor claims handling (initial claim set against the wrong insurer, lack of meaningful communication from the loss adjuster, decision communicated with little empathy) — RSA required to pay the £500 compensation it had already offered</t>
+        </is>
+      </c>
+      <c r="N35" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P35" s="3" t="inlineStr">
+        <is>
+          <t>A holiday home's occasional or seasonal use does not meet a policy's 'lived in' definition (regular bathing, cooking, sleeping) even where the policyholder does stay overnight for a short period; where neither the mains-off/drain condition nor the minimum-heating condition for an unoccupied property has been met, and the loss mechanism is a freeze-related pipe burst, the breach is material to that specific loss and entitles the insurer to decline the claim, even though separate compensation for poor claims handling may still be due</t>
+        </is>
+      </c>
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — the occupancy pattern (a few days' stay only) was undisputed; the dispute was over its legal characterisation as 'lived in' or not</t>
+        </is>
+      </c>
+      <c r="R35" s="3" t="inlineStr">
+        <is>
+          <t>Objectively, staying at a holiday home occasionally for a few days doesn't amount to normal living activities being regularly carried out, so RSA was reasonable to treat the property as unoccupied for the winter period; as neither the mains-off/drain nor the minimum-heating condition was satisfied, and the proximate cause was a freeze-related pipe failure, the breach was material and the decline was fair; separately, RSA's handling of the claim (wrong insurer initially, poor communication, blunt/unsympathetic outcome delivery) fell short and warranted the £500 compensation already offered</t>
+        </is>
+      </c>
+      <c r="S35" s="3" t="inlineStr">
+        <is>
+          <t>For a holiday home, assess 'lived in' against the normal meaning of regular day-to-day habitation, not mere physical presence for a few days; poor claims-handling compensation can be awarded to a policyholder even where the underlying coverage decline itself is upheld as reasonable — record such cases' outcome as an uphold limited to service failure, not as reversing the coverage decision</t>
+        </is>
+      </c>
+      <c r="T35" s="3" t="inlineStr">
+        <is>
+          <t>IF property_is_a_holiday_home_visited_only_occasionally_or_for_a_few_days_at_a_time AND policy_requires_regular_habitation_to_be_lived_in THEN occasional_visits_do_not_meet_the_lived_in_threshold; IF neither_mains_off_drain_nor_minimum_heating_condition_was_met_AND_loss_mechanism_is_a_freeze_related_pipe_burst THEN breach_is_material_and_coverage_decline_is_reasonable_even_if_handling_compensation_is_separately_due</t>
+        </is>
+      </c>
+      <c r="U35" s="3" t="inlineStr">
+        <is>
+          <t>DRN-4915511.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="80" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4962775</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Gresham Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>25 Dec 2024</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Home insurance (inherited/estate property) — escape of water from a frozen pipe compression fitting; insurer declined citing the unoccupied-property exclusion, since the property had been unoccupied for more than 60 consecutive days and the beneficiaries' practice of alternating one week in every six did not meet the policy's 'lived in' definition</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Property became unoccupied in February 2023 following the owner's death; contents cover was removed from the policy at that point; the April 2023 renewal recorded the property as unoccupied for more than 60 consecutive days; beneficiaries alternated staying roughly one week in every six for upkeep; the escape of water occurred in January 2024, more than eight months into the unoccupied period, well beyond the 60-day free-cover window</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (estate property, unoccupied following bereavement)</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>After the first 60 consecutive unoccupied days, damage from frozen pipes was excluded; alternating occupation of one week in every six did not meet the policy's 'lived in' definition (bathing, cooking, eating, sleeping regularly carried out)</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Executor: the one-week-in-six pattern was intended to meet the policy's requirements, and the terms weren't specific about the number of days or frequency needed. Gresham: a recorded call at the March 2023 policy amendment confirmed the executor told it no one would use the property as a main residence, and its agent repeated the 60-day exclusion several times without challenge. FOS: a handwritten note of stay dates provided as evidence was internally inconsistent with the actual 2023 calendar and wasn't persuasive; utility bills for the relevant months showed usage largely made up of standing charges, far below what would be expected at an occupied property; alternating occupation of one week in six does not amount to activities of daily living being 'regularly' carried out</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Gresham's 60-day unoccupied exclusion was clearly communicated at renewal and on the recorded amendment call, and was fairly applied given the property wasn't 'lived in' as defined</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>A 'lived in' definition requiring regular day-to-day activities (bathing, cooking, eating, sleeping) is not met by beneficiaries or family members alternating occupation for one week in every six; a recorded call in which the policyholder's representative confirms no one is using the property as a main residence, combined with the insurer's agent repeating a time-limited unoccupancy exclusion multiple times without challenge, is strong evidence the exclusion was clearly communicated and understood</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>Persuasive evidence (consistent dated logs, meaningful utility usage) that the property was genuinely lived in during the relevant weeks — the handwritten occupancy note was internally inconsistent with the calendar, and utility bills showed negligible usage consistent with an empty property</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>The policy's 60-day unoccupied exclusion for frozen-pipe damage was clearly set out in the April 2023 renewal documents; the executor's handwritten note of alternating stay dates didn't match the actual 2023 calendar and so wasn't reliable evidence of occupation; utility bills showed usage consistent with an empty property; the recorded March 2023 call confirmed the executor told Gresham no one used the property as a main residence, and the 60-day exclusion was repeated multiple times without any query from him; one week in six does not meet a requirement for day-to-day living activities to be 'regularly' carried out</t>
+        </is>
+      </c>
+      <c r="S36" s="2" t="inlineStr">
+        <is>
+          <t>When assessing occupancy claims based on a rotating or alternating family stay pattern, cross-check any handwritten or informal occupancy log against the actual calendar for internal consistency, and weigh utility usage data against what would be expected for a genuinely occupied property; a recorded call where the policyholder's representative confirms no main-residence use is strong evidence against a later claim of sufficient occupancy</t>
+        </is>
+      </c>
+      <c r="T36" s="2" t="inlineStr">
+        <is>
+          <t>IF beneficiaries_or_family_alternate_staying_at_a_property_for_one_week_in_every_N_weeks_for_upkeep_purposes AND policy_requires_regular_day_to_day_living_activities_to_be_lived_in THEN rotating_occasional_stays_do_not_meet_the_lived_in_definition; IF handwritten_occupancy_log_is_internally_inconsistent_with_the_calendar_or_utility_bills_show_negligible_usage THEN occupancy_evidence_is_not_persuasive</t>
+        </is>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4962775.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="80" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-036</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>DRN-4979244</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>The Salvation Army General Insurance Corporation Ltd</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>30 Dec 2024</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Property owners insurance (rented property) — theft claim following a break-in at an unoccupied property (tenant abandoned around August 2022); insurer declined citing breach of an unoccupancy condition requiring inspections every 14 days with a maintained log once the property had been vacant for more than 31 consecutive days</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Tenant abandoned the property around August 2022; property vacant thereafter; two prior break-ins occurred at the same property within roughly the same 10-month period (April 2022, not claimed, believed unoccupied; September 2022, claim paid on the basis it was occupied); the February 2023 break-in (forced entry through a rear window with a metal security sheet removed) is the subject of this claim</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Rented residential property (unoccupied after tenant abandonment)</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>Policyholders couldn't provide an inspection log evidencing compliance with the condition requiring internal and external inspections every 14 days, with a written log retained, once the property had been vacant for more than 31 consecutive days</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>SAGIC: a regular inspection regime would have demonstrated a deterrent presence and/or alerted the owners to the break-in sooner, as had happened via the local authority during a prior incident. Owners: they'd added metal security sheeting to the property after prior incidents (which was itself forcibly removed during this break-in), showing they'd taken reasonable preventive steps despite not keeping a formal inspection log. FOS: agreed the 14-day inspection condition had been breached, but found no evidence the breach increased the risk of, or was otherwise connected to, the February 2023 break-in specifically — a materially similar break-in had occurred at the same property only months earlier while it was accepted by SAGIC as occupied, undermining any argument that an inspection regime for the unoccupied period would have prevented this incident</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>SAGIC required to reconsider the claim in line with the remaining policy terms and conditions, including 8% simple interest per year on any claim-related repair costs already paid by the policyholders, from the date of payment to the date of settlement</t>
+        </is>
+      </c>
+      <c r="N37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P37" s="3" t="inlineStr">
+        <is>
+          <t>A breach of an unoccupied-property inspection condition (e.g. inspections every 14 days with a maintained log) only entitles an insurer to decline a claim if it can show the breach increased the risk of the loss that actually occurred, or is otherwise connected to it — where the insurer's own claims history shows a materially identical type of loss (e.g. a break-in) occurred at the same property while it was accepted as occupied (i.e. regardless of any inspection regime), this undermines an argument that non-compliant inspections were causally connected to the unoccupied-period loss</t>
+        </is>
+      </c>
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>Evidence connecting the missed 14-day inspections to the increased risk or occurrence of the February 2023 break-in specifically — SAGIC did not produce this</t>
+        </is>
+      </c>
+      <c r="R37" s="3" t="inlineStr">
+        <is>
+          <t>The inspection condition was breached, but SAGIC's own claims history showed a similar break-in occurred at the same property in September 2022 while it was treated as occupied — undermining its argument that a 14-day inspection regime for the unoccupied period would have prevented or mitigated the February 2023 incident; the metal security sheeting the owners had already added (and which was forcibly removed in this break-in) showed reasonable preventive steps had been taken independent of the formal inspection log requirement; SAGIC's argument that inspections would merely have alerted the owners sooner (as the local authority did previously), rather than prevented the loss, was not sufficient to show the breach was connected to the loss</t>
+        </is>
+      </c>
+      <c r="S37" s="3" t="inlineStr">
+        <is>
+          <t>When an insurer relies on a breach of an inspection or monitoring condition to decline an unoccupied-property claim, check the insurer's own claims history for the same property — a materially similar loss occurring while the property was accepted as occupied undermines any argument that the missing inspections were the connecting cause of an unoccupied-period loss</t>
+        </is>
+      </c>
+      <c r="T37" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_declines_unoccupied_property_claim_citing_breach_of_periodic_inspection_condition AND insurer_cannot_show_the_breach_increased_the_risk_of_or_is_connected_to_the_specific_loss_that_occurred THEN decline_is_not_reasonable_and_claim_should_be_reconsidered; IF a_materially_similar_loss_previously_occurred_at_the_same_property_while_it_was_accepted_as_occupied THEN this_undermines_an_argument_that_missed_unoccupied_period_inspections_caused_or_contributed_to_the_loss</t>
+        </is>
+      </c>
+      <c r="U37" s="3" t="inlineStr">
+        <is>
+          <t>DRN-4979244.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="80" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5010249</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Covea Insurance plc</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>14 Nov 2024</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Leasehold block property insurance (via the freeholder's policy) — escape of water from a leak in the flat above; insurer declined citing the vacant/unoccupied exclusion since the leaseholder had moved out and hadn't complied with the required 7-day inspection condition</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Leaseholder moved out of his flat in mid-2023 intending to sell; visited and checked the property roughly weekly, supplemented by estate agent viewings; his last confirmed visit/viewing was 22 December 2023; the leak was discovered 17 days later on 8 January 2024, exceeding the policy's required 7-day inspection interval</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Leasehold flat (vacant, for sale)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Premises were vacant/unoccupied (not actively used) for more than 30 days, and it was a condition precedent to liability that the property be internally and externally inspected every 7 days with a written record — the 17-day gap since the last visit before the loss breached that condition</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Mr M: said he checked the flat weekly, plus there were estate agent viewings, so he'd complied with the inspection requirement. Insurer/FOS: the evidence showed his actual last visit before the loss was 22 December 2023, and the leak was found 17 days later — exceeding the required 7-day interval regardless of his general weekly practice; photos of the empty, unfurnished property supported it being genuinely unoccupied rather than merely infrequently visited</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — the vacant/unoccupied classification and the resulting breach of the 7-day inspection condition were both reasonable and material to the loss</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>Where a policy requires an unoccupied property to be inspected at set intervals (e.g. every 7 days) as a condition precedent to liability, an insurer can rely on breach of that condition where the policyholder's own evidence establishes a gap between inspections exceeding the required interval immediately before the loss was discovered, even if the policyholder otherwise visited 'weekly' on average</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>Evidence of any inspection between 22 December 2023 and the discovery of the leak on 8 January 2024 — a 17-day gap with no recorded inspection</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>The property was empty and unfurnished, consistent with being genuinely unoccupied rather than merely infrequently visited; the requirement under the policy for unoccupied properties is a visit at least once every 7 days, and visiting once a week would have satisfied that condition, but the specific gap immediately before this loss (22 December to 8 January, 17 days) exceeded it; an unoccupied property presents a greater risk, and the damage may well have been less if the flat had been checked within the required interval, so the breach was material to the loss</t>
+        </is>
+      </c>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>When assessing compliance with a fixed-interval unoccupied-property inspection condition, calculate the actual gap between the last confirmed inspection or visit and the date the loss was discovered — an average or typical visiting frequency doesn't establish compliance if the specific pre-loss gap exceeds the required interval</t>
+        </is>
+      </c>
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>IF unoccupied_property_policy_requires_inspections_at_fixed_intervals_of_N_days_as_a_condition_precedent AND the_gap_between_the_last_confirmed_inspection_and_the_discovery_of_the_loss_exceeds_N_days THEN the_condition_is_breached_regardless_of_the_policyholders_average_or_typical_visiting_frequency</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5010249.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="80" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-038</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>DRN5130555</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>5 May 2016</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Landlord insurance — no claim or loss involved; complaint that UKI didn't disclose at the point of sale that it would cancel the policy on notice if part of the insured property became unoccupied</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Newly incepted landlord policy; shortly after inception one of the tenants left, triggering UKI's undisclosed practice of giving notice to cancel cover for a partially-unoccupied let property, rather than any loss event</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Rented residential property (landlord policy; part of the let property became unoccupied)</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — no claim was made; the complaint concerned an undisclosed cancellation-on-unoccupancy practice, not a declined claim</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>Mr A: wouldn't have proceeded with the policy had he known UKI would cancel it on a tenant leaving. UKI: it can only insure occupied premises, and the policy required notification of important changes; it's not feasible to tell customers about every circumstance in which it might exercise its general cancel-on-notice condition. FOS: the policy's own Unoccupancy condition implied continued (not automatically cancelled) cover for a partially-unoccupied let property, so UKI's actual intention to cancel on notice in that scenario should fairly have been disclosed at the outset, since it's in the nature of letting property that tenants leave from time to time and UKI knew what it would do about that but Mr A didn't</t>
+        </is>
+      </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>UKI not required to refund the premium for the period it was on risk, but required to pay Mr A £100 compensation for the trouble and upset of having to arrange replacement cover at short notice</t>
+        </is>
+      </c>
+      <c r="N39" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="O39" s="3" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P39" s="3" t="inlineStr">
+        <is>
+          <t>Where a landlord or rental-property policy's own Unoccupancy condition implies continuing (rather than automatically cancelled) cover for a partially-unoccupied let property, an insurer's undisclosed internal practice of exercising a general cancel-on-notice condition specifically because of that unoccupancy should be disclosed to the policyholder at the point of sale; failure to do so doesn't entitle the policyholder to a refund of premium already earned for time on risk, but can attract distress and inconvenience compensation for the disruption of arranging replacement cover at short notice</t>
+        </is>
+      </c>
+      <c r="Q39" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — no loss or claim was in dispute; the issue was one of disclosure at the point of sale</t>
+        </is>
+      </c>
+      <c r="R39" s="3" t="inlineStr">
+        <is>
+          <t>The Unoccupancy condition in the policy, on its face, implied cover would continue (with restrictions) rather than be cancelled outright if part of the property became unoccupied, so UKI's actual practice of cancelling on notice in that scenario came as a surprise that should have been flagged up front; UKI was nonetheless entitled to a premium for the period it had genuinely been on risk; £100 compensation was fair to reflect the trouble and upset of the unexpected cancellation and the need to arrange replacement cover, though Mr A should have started looking for alternative cover immediately once notice was given</t>
+        </is>
+      </c>
+      <c r="S39" s="3" t="inlineStr">
+        <is>
+          <t>When a landlord policy is cancelled on notice specifically because a let property became unoccupied, check whether the policy's own Unoccupancy condition implies continued cover — if so, the insurer's practice of using a general cancellation clause to end cover in that scenario should have been disclosed at sale, and non-disclosure can support a distress and inconvenience award even where no premium refund is due beyond the period genuinely on risk</t>
+        </is>
+      </c>
+      <c r="T39" s="3" t="inlineStr">
+        <is>
+          <t>IF landlord_or_rental_property_policy_contains_an_unoccupancy_condition_implying_continued_cover_for_partial_unoccupancy AND insurer_has_an_undisclosed_practice_of_cancelling_on_notice_specifically_because_of_unoccupancy THEN insurer_should_have_disclosed_this_intention_at_the_point_of_sale_and_non_disclosure_can_attract_distress_and_inconvenience_compensation_even_without_a_premium_refund_beyond_the_period_on_risk</t>
+        </is>
+      </c>
+      <c r="U39" s="3" t="inlineStr">
+        <is>
+          <t>DRN5130555.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="80" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>DRN5197867</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>9 Feb 2015</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Home insurance — escape of water claim declined citing the unoccupied-property exclusion (not lived in for more than 60 days) while the policyholder, due to a medical condition, had been living with a friend for over a year and was unable to manage his own affairs; the friend inspected the property weekly but hadn't notified the insurer of the change</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Policyholder living with a friend for more than a year due to a medical condition that left him unable to deal with his day-to-day affairs; the friend inspected the insured property weekly and collected post, but didn't inform the insurer at renewal that the home had been unoccupied for more than 60 days</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (owner unable to reside due to medical condition, informally monitored)</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Home had not been lived in ('slept in frequently') by the policyholder or anyone with his permission for more than 60 days in a row</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Mr D: the term was inherently unfair since it would pay a claim within the first 60 days of absence but not after, even if the property continued to be checked weekly, and his medical incapacity should be taken into account. RSA: it wasn't told of the change in circumstances, and had it known, it would have applied unoccupancy terms and a significantly higher premium. FOS: the unoccupied-property term was clear and had been sufficiently drawn to Mr D's attention in the renewal documentation; weekly inspection by a friend, however diligent, doesn't satisfy a 'lived in'/'slept in frequently' requirement, and is a separate matter from the obligation to notify the insurer of extended unoccupancy — which the friend, already handling Mr D's correspondence by the time of the renewal, could have done</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — RSA's reliance on the clear unoccupied-property exclusion was reasonable, notwithstanding Mr D's medical circumstances and his friend's diligent weekly inspections</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>A policy definition of 'lived in' as 'slept in frequently' is not satisfied by a third party's diligent weekly inspection and mail collection on the policyholder's behalf, however conscientious; an unoccupancy notification obligation triggered by the insured being away from the property for an extended period is separate from having someone check on it, and a policyholder's medical incapacity (through no fault of their own) does not, without more, excuse non-compliance where someone else was already managing the policyholder's affairs and correspondence during the relevant period</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — the underlying facts (friend's weekly checks, failure to notify RSA) were undisputed; the dispute was over their legal sufficiency</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>Unoccupied-property terms of this kind are not unusual and were clearly set out in the renewal documentation; problems are generally noted earlier, or may not happen at all, when a property is genuinely occupied, justifying the distinction insurers draw; Mr D's friend was diligently checking the property weekly and, by the time of renewal, was also handling his correspondence, but this didn't amount to the property being lived in, nor did it negate the separate requirement to tell RSA about the extended unoccupancy — something the friend could have done while already managing his post; RSA's investigation (including sending an assessor after the complaint) and internal escalation of the complaint were handled reasonably even though communication with Mr D himself could have been clearer</t>
+        </is>
+      </c>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>When a policyholder's medical condition or incapacity is raised as an excuse for non-disclosure of extended unoccupancy, check whether someone else was already managing the policyholder's correspondence or affairs during the relevant period — if so, the incapacity argument is weakened because that person could have made the required notification</t>
+        </is>
+      </c>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>IF policy_defines_lived_in_as_slept_in_frequently AND property_is_only_being_checked_or_inspected_weekly_by_a_third_party_without_anyone_sleeping_there THEN the_lived_in_threshold_is_not_met_regardless_of_inspection_diligence; IF policyholder_cites_medical_incapacity_as_the_reason_for_not_notifying_extended_unoccupancy AND_a_third_party_was_already_managing_the_policyholders_correspondence_during_that_period THEN the_incapacity_argument_is_weakened_since_that_person_could_have_made_the_notification</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>DRN5197867.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="80" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-040</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>DRN-5222573</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Sainsbury's Bank Plc</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>16 Jan 2025</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Mis-sale complaint (not a declined claim decision itself) — home insurance sold online by Sainsbury's Bank on a non-advised basis; policyholder declared the property unoccupied at application, triggering a fire/lightning/explosion/earthquake (FLEE) only restricted-cover endorsement; a later escape-of-water loss fell outside that restricted cover and the policyholder said the restriction hadn't been made clear to her</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Property declared unoccupied (left empty more than 60 consecutive days) at the point of sale in September 2023, triggering the FLEE-only endorsement and a companion condition requiring weekly inspections; a burst-pipe escape-of-water loss occurred later and fell outside the FLEE-restricted cover</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Residential property (declared unoccupied at inception)</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable to this decision — the underlying insurer's decline of the escape-of-water claim (cover being restricted to FLEE perils only) was not itself disputed here; this complaint concerned whether Sainsbury's, as seller, adequately highlighted the FLEE restriction at the point of sale</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Mrs N: the FLEE restriction wasn't drawn to her attention and the policy wording (which still listed an escape-of-water excess) was confusing. Sainsbury's: the sale was non-advised, and a mandatory tick-box confirmed she'd read and understood the FLEE/unoccupied endorsement information, which was also repeated on page two of the policy schedule. FOS: the endorsement was clearly and prominently presented at both the point of sale (mandatory tick-box) and in the follow-up documentation; Mrs N's own compliance with the accompanying weekly-inspection requirement — set out immediately below the FLEE restriction in the same clause — showed she was in fact aware of that part of the same endorsement, undermining her argument that the FLEE limitation itself hadn't been highlighted</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Sainsbury's had done enough, at both the point of sale and in follow-up documentation, to highlight the FLEE cover restriction</t>
+        </is>
+      </c>
+      <c r="N41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t>On a non-advised sale, a mandatory tick-box confirming the customer has read and understood a cover-restricting endorsement (e.g. a FLEE-only restriction triggered by a declared-unoccupied property), repeated on page two of the subsequent policy schedule, is sufficient to discharge the seller's obligation to present the information clearly, fairly and prominently — even where other parts of the same policy wording are confusingly inconsistent (e.g. still quoting an escape-of-water excess); a policyholder's demonstrated compliance with a companion condition within the same endorsement (e.g. weekly inspections) is evidence she was in fact aware of the endorsement as a whole</t>
+        </is>
+      </c>
+      <c r="Q41" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — the point-of-sale and documentation record was complete; the dispute was over whether it was sufficiently prominent, not whether it existed</t>
+        </is>
+      </c>
+      <c r="R41" s="3" t="inlineStr">
+        <is>
+          <t>The FLEE endorsement and unoccupied-property conditions were prominently set out in a mandatory 'important information' tick-box at the point of sale and repeated on page two of the policy schedule; while the policy wording elsewhere confusingly still referenced an escape-of-water excess, this didn't undermine the clarity of the FLEE restriction itself, which was set out in one clear line; Mrs N's own compliance with the weekly-inspection requirement, immediately below the FLEE restriction in the same clause, showed she had read and engaged with that part of the endorsement, undermining her claim that the restriction wasn't brought to her attention</t>
+        </is>
+      </c>
+      <c r="S41" s="3" t="inlineStr">
+        <is>
+          <t>When assessing whether a cover-restricting endorsement (e.g. FLEE-only for a declared-unoccupied property) was adequately disclosed on a non-advised online sale, check for (a) a mandatory acknowledgment step at the point of sale and (b) repetition in the follow-up policy schedule — both present is strong evidence of adequate disclosure, and a policyholder's later compliance with a companion condition in the same endorsement clause is corroborating evidence of awareness, even if she claims not to have understood a different part of the same clause</t>
+        </is>
+      </c>
+      <c r="T41" s="3" t="inlineStr">
+        <is>
+          <t>IF non_advised_online_sale_requires_a_mandatory_tickbox_acknowledging_a_specific_cover_restricting_endorsement AND the_same_endorsement_is_repeated_in_the_subsequent_policy_schedule THEN the_seller_has_adequately_disclosed_the_restriction_even_if_other_parts_of_the_policy_wording_are_confusing; policyholders_demonstrated_compliance_with_a_companion_condition_within_the_same_endorsement_is_evidence_of_awareness_of_the_endorsement_as_a_whole</t>
+        </is>
+      </c>
+      <c r="U41" s="3" t="inlineStr">
+        <is>
+          <t>DRN-5222573.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="80" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>DRN5276115</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>RGA Underwriting Limited</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>30 May 2018</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Landlord property insurance (broker mis-sale complaint) — malicious damage claim was accepted, but insurer applied a £2,500 minimum excess (instead of the standard £250) because the property was unoccupied at the time of the damage; policyholder complained the increased unoccupied-property excess wasn't clearly disclosed at the point of sale</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Landlord property; the £2,500 minimum-excess condition for unoccupied properties was set out on page 27 of the January 2016 policy documentation but wasn't included on the statement of fact form sent to the policyholder, and the broker said it hadn't been able to highlight it specifically because the policyholder hadn't told it the property was unoccupied</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Rented residential property (landlord insurance)</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — the malicious damage claim itself was accepted; the dispute concerned only whether the resulting £2,500 unoccupied-property excess (rather than the standard £250) had been adequately disclosed at the point of sale</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Mr H: the increase in excess for an unoccupied property wasn't made clear in the policy documentation provided when the policy was sold. RGA: the increase was covered in the documentation (page 27) which stated the minimum excess would be £2,500 for each and every claim on an unoccupied policy; it also said it couldn't have highlighted this specifically since Mr H hadn't told it the property was unoccupied, and that landlords get a 14-day cooling-off period and prominent renewal reminders to read their documents. FOS: as a landlord, there was a real chance the property could become unoccupied, so a tenfold increase in excess for that scenario was a significant term that should have been proactively highlighted rather than left on page 27 of the booklet and omitted from the statement of fact</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>RGA required to pay Mr H £2,250 (the difference between the £2,500 and £250 excess) plus 8% simple interest per year from the date the excess was paid to the date of settlement</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>2250</v>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>Where a landlord policy imposes a materially higher excess (here £2,500 versus a standard £250) specifically for claims arising while the property is unoccupied, this is a significant term that a seller must proactively highlight to a landlord policyholder — particularly given the inherent likelihood that a rented property will become unoccupied between tenancies — rather than leaving it to be found only deep within the policy booklet and omitted from the statement of fact; a seller cannot excuse non-disclosure of a standard policy term on the basis that the policyholder hadn't yet flagged the specific circumstance (unoccupancy) that would trigger it</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — the documentation gap itself (excess increase omitted from the statement of fact, buried on page 27 of the booklet) was not disputed</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>As a landlord, Mr H had specifically added unoccupancy cover to his buildings policy, which itself showed the risk of unoccupancy was significant to him and should have been recognised as such by RGA; the £2,500 minimum excess for unoccupied-property claims was buried on page 27 of the policy documentation and omitted from the statement of fact form, so wasn't adequately highlighted; had it been, Mr H would likely have sought an alternative policy with a lower unoccupied-property excess at a similar price, so RGA should put him in that position by refunding the difference with interest</t>
+        </is>
+      </c>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>For landlord policies, a materially increased excess or exclusion specifically triggered by unoccupancy should be treated as inherently significant and proactively disclosed, since landlords face an ordinary risk of a property becoming unoccupied between tenancies — this differs from a general residential policyholder for whom unoccupancy might be a more remote scenario; omitting such a term from a statement of fact form, even if technically present elsewhere in the policy booklet, is not adequate disclosure</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>IF landlord_policy_imposes_a_materially_higher_excess_or_exclusion_specifically_triggered_by_unoccupancy AND this_term_is_omitted_from_the_statement_of_fact_form_or_buried_deep_in_the_policy_booklet THEN the_term_was_not_adequately_disclosed_and_seller_should_refund_the_difference_between_the_disclosed_and_actual_excess_with_interest</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>DRN5276115.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="80" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-042</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>DRN-5338495</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>18 Mar 2025</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Home buildings insurance — escape of water from a burst pipe; insurer avoided the policy from the date the claim was reported and declined the claim, saying occupancy evidence (energy/council tax bills, absence of food/clothes) showed the property hadn't been occupied in line with its 'slept in frequently' definition</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Insurer's loss adjuster raised concerns about occupancy after the claim was reported in December 2022; requested supporting information including energy and council tax bills; on review it concluded the property hadn't been occupied in accordance with the policy's definition and voided the policy back to the date of the claim report</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Residential property (occupancy status disputed)</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>RSA said Ms T had misrepresented her occupancy of the property when the policy was taken out (a qualifying misrepresentation under CIDRA), entitling it to avoid the policy; it also said the property hadn't been occupied in line with the policy's definition of 'lived in' (slept in frequently), citing absent food/clothes and low energy usage</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Ms T: said she did sleep at the property frequently, satisfying the policy's own definition; the absence of clothes was because she'd removed them to prevent damp damage, and a council tax letter confirmed the unoccupied status previously recorded had been inaccurate and was removed effective 1 July 2021. RSA: initially couldn't provide the sales-call recording or the questions asked about occupancy at inception, but later located and provided a recording; the property showed no food/clothes and low energy use, indicating it wasn't lived in as required. FOS: without the original evidence of what was asked, RSA couldn't show a misrepresentation had occurred; having subsequently listened to the recorded sales call, RSA's agent asked only whether the home would be left unoccupied for more than 60 days in a year (answered 'no, never') and never explained what 'occupied' meant beyond that, so Ms T was entitled to rely on the policy's own 'slept in frequently' definition; RSA's additional criteria (food in the fridge, clothes in wardrobes) weren't set out in the policy terms, so couldn't be used to show she'd failed to meet the occupancy requirement</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>RSA required to remove any record of the avoidance and cancellation from internal and external databases, reconsider the claim without reliance on the unoccupancy exclusion, and pay Ms T £600 compensation for distress and inconvenience</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t>Where a policy defines an occupied property narrowly as one that is 'lived in' (meaning slept in frequently), an insurer cannot rely on additional, undocumented criteria (e.g. food in the fridge, clothes in wardrobes, council tax status) to argue the property wasn't occupied — if the insurer wanted a wider meaning of occupied, this should have been made clear in the policy terms; to avoid a policy for misrepresentation about occupancy, the insurer must be able to show what questions were actually asked and what answers were given (ideally via a call recording or documented statement of fact) — a policyholder is entitled to rely on the policy's own definition where the insurer's agent didn't explain a wider meaning during the sales call</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t>Initially, any record of the questions asked about occupancy at the September/February 2022 policy inception — RSA said it couldn't access this, then later located and provided a call recording, which the ombudsman found did not support RSA's misrepresentation argument once actually reviewed</t>
+        </is>
+      </c>
+      <c r="R43" s="3" t="inlineStr">
+        <is>
+          <t>Provisionally, without the call recording, RSA hadn't shown what Ms T was asked about occupancy, so a misrepresentation couldn't be established; the policy's own definition of 'lived in' as 'slept in frequently' was clear and Ms T's account that she slept there frequently wasn't contradicted by reliable evidence, since her explanations for the absent clothes and inaccurate council tax record were reasonable; having subsequently listened to the recorded sales call RSA provided, the agent asked only about being unoccupied for more than 60 days a year and never explained a wider meaning of occupied, so the provisional findings stood; a higher compensation of £600 (rather than the £300 initially proposed) was warranted given the significant, ongoing distress (anxiety, sleep problems, medication) and the length of time involved, tempered by the property not being Ms T's main residence</t>
+        </is>
+      </c>
+      <c r="S43" s="3" t="inlineStr">
+        <is>
+          <t>When an insurer relies on a suspected occupancy misrepresentation to avoid a policy, first check what the policy's own definition of 'occupied'/'lived in' actually requires and whether the insurer can produce contemporaneous evidence (call recording, statement of fact) of the specific questions asked and answers given at inception — general circumstantial evidence (utility usage, absence of personal items) cannot substitute for that, especially where it relies on criteria not set out in the policy definition itself</t>
+        </is>
+      </c>
+      <c r="T43" s="3" t="inlineStr">
+        <is>
+          <t>IF policy_defines_occupied_narrowly_as_lived_in_meaning_slept_in_frequently AND insurer_relies_on_additional_criteria_not_set_out_in_that_definition_to_argue_non_occupancy THEN those_additional_criteria_cannot_be_used_to_defeat_the_claim; IF insurer_avoids_policy_for_occupancy_misrepresentation_but_cannot_produce_a_call_recording_or_documented_record_of_the_actual_questions_asked_and_answers_given THEN the_misrepresentation_is_not_established_and_avoidance_should_be_reversed</t>
+        </is>
+      </c>
+      <c r="U43" s="3" t="inlineStr">
+        <is>
+          <t>DRN-5338495.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="80" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5434926</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Gresham Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>20 May 2025</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Home buildings insurance — no claim or loss involved; complaint that Gresham ceased offering cover for an unoccupied property at renewal and failed to communicate effectively, since renewal/non-renewal correspondence was sent to the (unoccupied) insured address rather than an alternative address, and the policyholder — unable to live at home following a serious accident — didn't see it</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Policyholder unable to live at her home since a serious accident in 2021; informed the insurer in 2021 (discussed again in September 2021) and the policy was updated with unoccupied-property exclusions; renewal documents were sent by post to the insured (unoccupied) address in June 2022 and July 2023; a June 2024 letter to the same address explained the policy would not be renewed at its August 2024 expiry, which the policyholder didn't see as she wasn't living there</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (owner unable to reside due to serious accident/poor health)</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — no claim was made; the complaint concerned Gresham's decision not to continue unoccupied-property cover at renewal, and whether it communicated that decision effectively</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Miss W: didn't see the August 2024 non-renewal correspondence because she wasn't living at the insured address due to her poor health, and Gresham should have asked about an alternative contact address given her known circumstances. Gresham: it's the policyholder's responsibility to keep contact details current; all mail was sent to the confirmed address; no mail was returned and she never asked it to use a different address or method; its underwriting criteria meant it couldn't continue to offer cover in her circumstances. FOS: having listened to the April 2021 call, Gresham's agent acted professionally and explained the unoccupied-property restrictions and weekly-inspection requirement, but could reasonably have queried whether a different correspondence address was needed; however, Miss W had over three years (multiple renewals) during which she could have told Gresham she wasn't receiving her post, especially since she was shown to be aware of mail-redirection services generally; the June 2024 non-renewal letter gave five weeks' notice and included contact details for a specialist unoccupied-property insurer</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Gresham applied its underwriting criteria consistently, gave adequate notice and assistance to find alternative cover, and Miss W had ample opportunity over several years to update her correspondence preferences</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>An insurer's decision on what unoccupied-property risks it's prepared to continue to underwrite, and at what price, is a commercial decision this Service won't interfere with, provided its underwriting criteria are applied consistently; where a policyholder disclosed at the outset that correspondence would be difficult to receive at the insured address (e.g. due to a medical condition preventing residence there), an insurer's agent could reasonably be expected to query an alternative address at that point, but a policyholder who then has multiple renewal cycles over several years without querying missed post bears responsibility for not updating their contact preferences, particularly where they are shown to be otherwise aware of mail-redirection options</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — the facts (address never updated, mail never returned as undelivered) were undisputed; the dispute was over whether Gresham should nonetheless have proactively queried the address</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>The April 2021 call was thorough and professional but didn't address a change of correspondence address, which the agent could have raised; however Miss W had over three years and several renewal cycles to notice she wasn't receiving documentation and to ask Gresham to use a different address or method (e.g. email), and her use of a mail-redirection service for part of the period showed she was aware such options existed; the June 2024 non-renewal letter gave five weeks' notice and signposted a specialist alternative insurer, which was reasonable assistance; Gresham's underwriting criteria (reviewed but commercially sensitive) confirmed it genuinely couldn't offer cover in her circumstances, and this was applied consistently, not unfairly, to her</t>
+        </is>
+      </c>
+      <c r="S44" s="2" t="inlineStr">
+        <is>
+          <t>Where a policyholder is known to be unable to reside at the insured address for an extended period (e.g. due to a medical condition), flag at the point that circumstance is first disclosed whether a different correspondence address or method should be used — but a policyholder who goes multiple renewal cycles over several years without confirming receipt of documentation, despite being shown to be capable of arranging mail redirection, bears significant responsibility for the resulting missed communications</t>
+        </is>
+      </c>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>IF policyholder_discloses_at_the_outset_that_they_cannot_reside_at_or_reliably_receive_post_at_the_insured_address THEN insurer_should_query_an_alternative_correspondence_address_or_method_at_that_point; IF policyholder_then_has_multiple_renewal_cycles_over_several_years_without_querying_missed_documentation AND_insurer_sent_all_correspondence_to_the_confirmed_address_with_no_returned_mail THEN insurer_is_not_responsible_for_the_policyholder_not_receiving_a_subsequent_non_renewal_notice</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5434926.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="80" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-044</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>DRN5611706</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>CIS General Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Home buildings insurance (late father's property) — escape of water claim declined citing the unoccupied-property exclusion (60 consecutive days), after the policyholder took out the policy specifically to cover the known-unoccupied property but says she was only told about a theft exclusion, not the wider unoccupied-property exclusions</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Policy taken out at a local branch in May 2011 on the policyholder's late father's property, which she explained was furnished but unoccupied; renewed May 2012; escape of water claim made October 2012, more than 60 consecutive days into the unoccupied period</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Residential property (late father's estate, furnished but unoccupied)</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>Property had been unoccupied for more than 60 days, and under the policy most insured perils (including escape of water) are excluded while the buildings are unoccupied</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Ms L: she specifically wanted a policy to cover an unoccupied property and was told at the branch only that theft wouldn't be covered — not that escape of water and other perils were also excluded while unoccupied; had she known the full extent of the exclusions, she'd have sought different insurance. CIS: it was 'highly unlikely' an adviser would mention only one exclusion and not others; the exclusions were also clearly set out in the policy booklet (page 7) and summary (page 5); Ms L had renewed since and received updated documents; it later also argued (on the ombudsman's provisional decision) that cover was in fact wider than described, only excluding theft, vandalism, escape of water and frozen-system claims while occupied peril claims like fire, flood and storm remained covered. FOS: there was no recording or note of what was actually said at the branch sale, and Ms L's account (that she was told about the theft exclusion but not others) was accepted over CIS's speculative 'would have' account; having a policy's exclusions merely present in the booklet and summary wasn't sufficient given it appeared some exclusions had been actively explained and others hadn't; it also wasn't clear any proper investigation was made into whether the property in fact met the policy's furnished/unoccupied definition given Ms L said she'd told the adviser it was fully furnished</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>CIS required to deal with the escape of water claim under the remaining policy terms and conditions (adding 8% simple interest to any cash settlement from the date of the claim) and pay Ms L £200 compensation for the inconvenience and upset caused by its handling of the claim</t>
+        </is>
+      </c>
+      <c r="N45" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="O45" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P45" s="3" t="inlineStr">
+        <is>
+          <t>Where a policyholder specifically sought cover for a known-unoccupied property and can show she was told about one specific exclusion (e.g. theft) at the point of sale but not the wider range of exclusions that also apply while unoccupied, an insurer cannot rely on the exclusions simply being present in the policy booklet and summary to defeat that evidence — if some exclusions were actively explained at the point of sale and others weren't, this suggests an incomplete explanation rather than no explanation at all, and the insurer bears the consequence of that gap; an insurer relying on an unoccupancy exclusion should also verify the property in fact met the policy's specific definition of unoccupied (e.g. furnishing status) before applying it</t>
+        </is>
+      </c>
+      <c r="Q45" s="3" t="inlineStr">
+        <is>
+          <t>Any recording or contemporaneous note of what was said during the May 2011 branch sale — the original adviser was no longer employed by CIS and no notes existed, leaving only Ms L's testimony against CIS's speculation about what 'would have' been said</t>
+        </is>
+      </c>
+      <c r="R45" s="3" t="inlineStr">
+        <is>
+          <t>Ms L specifically sought cover for a property she knew would be empty for a while, so it would be odd for her to have selectively absorbed only the theft exclusion and ignored the others if all had genuinely been explained; CIS could not evidence what was actually said and relied only on inference about what an adviser would 'highly unlikely' have omitted; the exclusions being present on page seven of the booklet and page five of the summary was not enough given the apparent selective explanation at the point of sale; it also wasn't established that the property failed to meet the policy's furnished/unoccupied definition, since Ms L said she'd told the adviser the house was fully furnished; on balance, CIS could not reasonably rely on the exclusion here</t>
+        </is>
+      </c>
+      <c r="S45" s="3" t="inlineStr">
+        <is>
+          <t>When a policyholder says only one of several unoccupied-property exclusions was explained to them at sale (e.g. theft but not escape of water), and the insurer cannot produce a contemporaneous record of the sale, treat the selective/incomplete explanation as more probable than a policyholder inventing a partial account — a policy booklet and summary containing the full exclusions does not cure a demonstrably incomplete verbal explanation at the point of sale; separately verify the property's furnishing status against the policy's specific unoccupied definition before relying on the exclusion</t>
+        </is>
+      </c>
+      <c r="T45" s="3" t="inlineStr">
+        <is>
+          <t>IF policyholder_credibly_states_only_one_of_several_unoccupied_property_exclusions_was_explained_at_the_point_of_sale AND insurer_cannot_produce_a_contemporaneous_record_of_what_was_actually_said THEN the_insurer_cannot_rely_on_the_unexplained_exclusions_to_decline_the_claim_even_if_they_appear_in_the_policy_booklet_and_summary; insurer_relying_on_an_unoccupancy_exclusion_should_verify_the_property_actually_met_the_policys_specific_furnished_or_unoccupied_definition_before_applying_it</t>
+        </is>
+      </c>
+      <c r="U45" s="3" t="inlineStr">
+        <is>
+          <t>DRN5611706.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="80" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5849071</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>28 Oct 2025</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Landlord insurance (three rental properties on one policy) — no claim or loss involved; complaint that UKI unfairly cancelled the entire policy (covering three properties) after the policyholder said she couldn't comply with an unoccupancy endorsement applied to just one of the properties</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Policyholder told UKI in July 2024 that one of her three insured rental properties (property A) would be unoccupied for more than 30 consecutive days; UKI applied an unoccupancy endorsement to property A requiring services to be switched off at the mains; in September 2024 she said she couldn't comply because tradesmen working at the property needed services switched on; UKI subsequently cancelled the whole policy, covering all three properties, rather than removing only property A from cover</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Rented residential properties (landlord policy covering three properties; one unoccupied and under repair)</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — no claim was made; UKI decided it couldn't offer cover for the unoccupied property (property A) if the mains-off endorsement couldn't be met, and then cancelled the entire three-property policy rather than removing only property A</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Mrs S: UKI cancelled her whole policy without adequate further contact, leaving her embarrassed at having to disclose a cancelled policy and inconvenienced by arranging replacement cover for all three properties at short notice; she'd since found alternative cover and didn't want the UKI policy reinstated, but wanted an apology, compensation, and any cancellation record removed. UKI: it was entitled to decide it couldn't insure property A if the mains-off endorsement couldn't be met, and its cancellation policy operates for the policy as a whole; it also later suggested a September 2024 call raised 'concern' about Mrs S's consistency, though this wasn't the reason given for cancellation at the time and no recording was provided to support it. FOS: the policy schedule listed the three properties separately with their own sums insured, and UKI's own correspondence (the endorsement, the reminder letter) treated property A separately from the other two — so cancelling the whole policy over an issue confined to property A wasn't reasonable; UKI's belated 'concern' justification wasn't put to Mrs S at the time and wasn't supported by evidence, so couldn't be relied on retrospectively</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>UKI's decision not to offer cover for the unoccupied property (property A) without mains-off compliance found reasonable, but cancelling the entire policy (rather than removing only property A) found unfair; UKI required to pay Mrs S a global compensation award of £400 reflecting the likely financial impact of the unfair whole-policy cancellation and the distress and inconvenience caused, and to mark the policy as cancelled by Mrs S (not UKI) on any internal or external record</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>Where a landlord policy separately lists multiple insured properties with their own sums insured, and an insurer applies an unoccupancy endorsement to only one of those properties (treating it separately in its own correspondence), it is not fair or reasonable for the insurer to cancel the entire policy — covering all the properties — solely because the endorsement condition can't be met on the one affected property; an insurer's general policy-wide cancellation-on-notice term does not override this property-specific treatment once the insurer has itself administered the endorsement on a per-property basis; a justification for cancellation raised only after the event, and not put to the policyholder at the time or supported by evidence such as a call recording, cannot retrospectively justify the decision</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>A recording of the September 2024 call UKI later relied on to suggest 'concern' about Mrs S's consistency — UKI asked the ombudsman to rely on this call but didn't provide a copy</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>UKI was entitled to decide it wouldn't insure an unoccupied property (property A) if the mains-off endorsement couldn't be met — that's a legitimate underwriting decision; but its own documentation (endorsement applied only to property A, reminder letter naming only property A) showed it was treating the properties separately, making whole-policy cancellation disproportionate and unexplained; UKI's later suggestion that cancellation was really about a 'concern' raised in a September call wasn't the reason given to Mrs S at the time, wasn't evidenced by a recording despite being asked for one, and so could not fairly be relied upon; a global award (rather than working out exact premium differences, which weren't fully evidenced by Mrs S) was the simplest fair remedy</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="inlineStr">
+        <is>
+          <t>When a multi-property landlord policy has an unoccupancy endorsement applied to only one of the insured properties, and that endorsement can't be complied with, the correct remedy is to remove that specific property from cover, not cancel the whole policy — check the insurer's own correspondence for whether it has been treating the affected property separately (its own endorsement letters, schedules) before accepting a policy-wide cancellation as justified; a retrospective justification not given to the policyholder at the time, and unsupported by requested evidence, should be disregarded</t>
+        </is>
+      </c>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
+          <t>IF multi_property_landlord_policy_lists_properties_separately_with_their_own_sums_insured AND an_unoccupancy_endorsement_condition_cannot_be_met_on_only_one_of_those_properties THEN insurer_should_remove_only_that_property_from_cover_not_cancel_the_whole_policy; IF insurer_offers_a_new_justification_for_a_past_cancellation_that_was_not_given_to_the_policyholder_at_the_time_and_is_unsupported_by_requested_evidence_eg_a_call_recording THEN that_justification_cannot_be_relied_on_retrospectively</t>
+        </is>
+      </c>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5849071.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="80" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-046</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>DRN-5892113</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Fort Advice Bureau Limited</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>21 Apr 2026</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Property owners insurance (broker mis-advice complaint) — escape of water claim on an unoccupied property undergoing renovation was accepted by the underwriter, but reduced by 45.4% for underinsurance after the underwriter said the true rebuild value (£229,000) was far higher than the £125,000 set at inception; policyholder said the broker, not it, was responsible for the inaccurate rebuild figure</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Property owners policy taken out August 2024 for an unoccupied property undergoing building works (contract works value £8,000, cosmetic refurbishment), with rebuild value set at £125,000; escape of water claim made in the same policy year; underwriter said the rebuild value should have been £229,000 and reduced the £12,690 claim to 54.6% of its value for underinsurance</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Unoccupied property undergoing renovation (owned by a limited company)</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Accepted — With Deductions</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable to a full decline — the escape of water claim was accepted by the underwriter but paid at only 54.6% of its value, applying a condition of average for underinsurance based on a rebuild value it said should have been £229,000 rather than the £125,000 recorded at inception</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>Mr A (for B, the policyholder company): the £125,000 rebuild value was effectively supplied by the broker's own agent during the sales call, and it was absurd to suggest cosmetic works costing around £8,000 could have increased the rebuild value to £229,000 within months. Fort Advice: this was an advised sale, but the £125,000 figure was agreed between Mr A and its agent and confirmed by Mr A without change when he paid; it also said the works had enhanced the rebuild value and this hadn't been disclosed to the underwriter. FOS (having listened to the broker/underwriter sales call): Fort Advice's own agent, when asked the rebuild cost, said 'I don't know, probably 125 grand' and then confirmed this was simply the purchase price, not a value from a rebuild calculator, surveyor's report or other recognised method; as a professional broker on an advised sale, Fort Advice was responsible for supporting the policyholder in obtaining an accurate rebuild figure and hadn't done so; the only evidence of the scope of works (Fort Advice's own fact-find, recording ~£8,000 of cosmetic refurbishment) didn't support an increase of over £100,000, and if Fort Advice genuinely believed the works would increase the rebuild value so significantly, the £125,000 figure it put forward at inception would itself have been known to be inadequate</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M47" s="3" t="inlineStr">
+        <is>
+          <t>Fort Advice required to pay the difference between the full value of the escape of water claim and the reduced sum already paid by the underwriter, plus 8% simple interest per year from the date of the underwriter's cash settlement to the date of Fort Advice's settlement</t>
+        </is>
+      </c>
+      <c r="N47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" s="3" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P47" s="3" t="inlineStr">
+        <is>
+          <t>On an advised sale, a broker arranging property owners insurance for an unoccupied property under renovation is responsible for supporting the policyholder in obtaining an accurate rebuild value using a recognised method (e.g. an online build calculator or a professional survey) — a broker's own agent supplying a property's purchase price as a rebuild value, with an acknowledged 'I don't know', does not satisfy that obligation, and the broker (not the policyholder) bears responsibility for the resulting underinsurance and reduced claim settlement, even where the policyholder later confirms the figure without objection when paying</t>
+        </is>
+      </c>
+      <c r="Q47" s="3" t="inlineStr">
+        <is>
+          <t>Any evidence that the ~£8,000 of cosmetic refurbishment works actually carried out could plausibly have increased the property's rebuild value from £125,000 to £229,000 within a few months — none provided by Fort Advice</t>
+        </is>
+      </c>
+      <c r="R47" s="3" t="inlineStr">
+        <is>
+          <t>This was an advised sale, so Fort Advice had to ensure the policy (and its key figures, like rebuild value) was suitable for B's needs; its own agent supplied the £125,000 figure on the sales call by equating it to the purchase price, explicitly saying 'I don't know' rather than using a recognised valuation method, despite being the professional party responsible for the recommendation; Mr A wasn't the expert and wasn't shown to have been given guidance on how a rebuild value should be calculated; the only documented scope of works (~£8,000 cosmetic) couldn't explain an increase of over £100,000, and Fort Advice's own inconsistency (suggesting the works caused the shortfall while also having put forward the £125,000 figure itself) undermined its position; responsibility for the underinsurance and resulting reduced settlement therefore fell to Fort Advice</t>
+        </is>
+      </c>
+      <c r="S47" s="3" t="inlineStr">
+        <is>
+          <t>When an underinsurance penalty is applied to a reduced claim settlement on an advised-sale property policy, check the sales call/documentation for how the rebuild value was actually arrived at — if the broker's own agent supplied the figure without using a recognised valuation method (and said as much on the call), responsibility for underinsurance shifts to the broker rather than the policyholder, regardless of the policyholder later confirming the figure without objection, since the policyholder is not expected to independently verify a professional's figure</t>
+        </is>
+      </c>
+      <c r="T47" s="3" t="inlineStr">
+        <is>
+          <t>IF broker_conducts_an_advised_sale_of_property_owners_insurance AND brokers_own_agent_supplies_the_rebuild_value_by_equating_it_to_purchase_price_without_using_a_recognised_valuation_method THEN broker_not_policyholder_is_responsible_for_resulting_underinsurance_and_reduced_claim_settlement; policyholder_confirming_a_professionally_supplied_rebuild_figure_without_objection_when_paying_does_not_shift_that_responsibility_back_to_the_policyholder</t>
+        </is>
+      </c>
+      <c r="U47" s="3" t="inlineStr">
+        <is>
+          <t>DRN-5892113.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="80" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>DRN5978513</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Tesco Personal Finance Plc</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>15 May 2020</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Home insurance (broker/administrator mis-sale complaint) — escape of water claim declined by the underwriter citing the unoccupied-property exclusion (60 days), after the policyholder's son told Tesco at renewal that the property (owner moving into a care home) would become unoccupied, but Tesco never explained the resulting restricted cover</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Policyholder moved into a care home; her son told Tesco at the February 2018 renewal call that the property would be empty pending clearance and sale; Tesco renewed the policy without amending the schedule to reflect unoccupied status or explaining the resulting exclusions; leak (from a loft overflow pipe) discovered in August 2018, more than 60 days into the unoccupied period</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (owner in care home; property to be sold once cleared)</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable to a decision by Tesco directly — the underlying insurer declined the claim because the property had been unoccupied for 60 days; this complaint concerned whether Tesco (as the arranging administrator) should have made the policyholder's son aware of the resulting restricted cover at renewal</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Mr Z (on his mother's behalf): Tesco never called him back as promised to explain the unoccupied-property restrictions after he told it the property would be empty; the renewed schedule sent to him still recorded the property as normally occupied, giving him no reason to think cover had changed. Tesco: accepted it should have called back and offered £75 compensation for the error, but said even without the occupancy issue the claim wouldn't have been payable anyway because the damage occurred gradually. FOS: agreed the damage had occurred gradually and so wouldn't have been covered even absent the unoccupancy issue in isolation — but the correct approach was to ask what would have happened had Tesco not made its error; if Tesco had properly explained the loss of cover for unoccupied properties (not just escape of water, but theft, vandalism, malicious acts too), Mr Z would likely have sought a bespoke unoccupied-property policy instead, which would likely have required precautions like turning off the water supply — meaning the escape of water would probably never have happened at all</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Tesco required to cover the cost of repairing the escape of water damage (cash settlement, as the customer's chosen contractor's costs, unless both parties agreed Tesco would do the repairs itself) and pay Mrs Z £150 compensation for distress and inconvenience</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>Where an administrator/broker is told at renewal that a property will become unoccupied but fails to explain the resulting loss of cover (for escape of water and other perils) or amend the policy schedule to reflect it, the correct remedy analysis is counterfactual: even if the specific loss claimed (e.g. gradually-occurring damage) would independently have been excluded on its own facts, the seller's failure can still cause compensable loss if a properly-informed policyholder would likely have taken out a different, precaution-requiring unoccupied-property policy that would have prevented the loss mechanism (e.g. a frozen/burst pipe) from occurring in the first place</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>A recording of the original renewal call — none was available; the fact the policyholder's son told Tesco about the unoccupancy, and that Tesco's adviser said they'd call back but never did, wasn't disputed</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>Tesco admitted its error in not calling back, but argued this didn't matter because the gradual nature of the damage would have defeated the claim regardless of the unoccupancy exclusion; the ombudsman agreed on that narrow point but reframed the analysis around what would likely have happened but for Tesco's error — a bespoke unoccupied-property policy (which Mr Z did in fact seek out once he later learned of the restricted cover) would likely have required precautions such as turning off the water supply, and Mr Z would likely have complied; this would probably have prevented the escape of water occurring at all, so Tesco's failure did disadvantage the policyholder notwithstanding the gradual-damage point</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="inlineStr">
+        <is>
+          <t>When a seller's disclosure failure is met with a defence that the claim would have failed anyway on unrelated grounds (e.g. gradual damage), don't stop at that narrower point — assess what type of policy and precautions the policyholder would likely have taken up if properly informed, and whether those precautions would probably have prevented the loss mechanism itself from occurring, not just whether the same claim would have been covered under the same (undisclosed) policy</t>
+        </is>
+      </c>
+      <c r="T48" s="2" t="inlineStr">
+        <is>
+          <t>IF broker_or_administrator_fails_to_explain_unoccupied_property_exclusions_after_being_told_a_property_will_become_unoccupied AND insurer_argues_the_specific_claim_would_have_failed_anyway_on_unrelated_grounds THEN assess_whether_a_properly_informed_policyholder_would_likely_have_taken_a_different_precaution_requiring_unoccupied_property_policy_that_would_have_prevented_the_loss_mechanism_itself_from_occurring; if_so_the_brokers_disclosure_failure_remains_the_effective_cause_of_the_loss</t>
+        </is>
+      </c>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>DRN5978513.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="80" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-048</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>DRN-5990244</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>2 Apr 2026</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — flat damaged by a water leak while the policyholder was living abroad; insurer declined citing the unoccupied-property exclusion (not slept in on a regular basis for more than 60 days), disputing whether the policyholder's brother had genuinely been living there as claimed</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder living abroad since September 2024; said her brother had been living in her flat for the 18 months before the leak following his marriage breakdown, leaving briefly (23 December) to spend Christmas with friends; leak discovered by a neighbour in early January 2025; insurer's loss adjuster raised multiple concerns about the brother's true residency (no supporting evidence of 18 months' occupancy, high 'residency scores' at a previous address, driving licence/bank statements/credit applications still showing that address, relatively low utility usage, no damaged belongings of his)</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Residential flat (occupancy of resident brother disputed)</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Insufficient evidence that the policyholder's brother was living at the property on a regular basis, as required for the property to be 'occupied' under the policy's more-than-60-days exclusion</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>UKI: multiple indicators (no supporting evidence from Mr S himself, credit and licence records showing a different address, relatively low utility usage for two occupants, none of Mr S's belongings damaged) suggested he wasn't genuinely living at the flat. Ms S: her brother had been living there for 18 months, and utility bills and a neighbour's message enquiring when he was due back supported this. FOS: the policy only required someone to be sleeping at the property regularly, not that it be their sole or official residence, so the absence of official records (licence, bank statements) at that address wasn't determinative; electricity usage, while lower than average for two occupants, showed a meaningful drop precisely when the policyholder left and further still when the brother went away for Christmas — consistent with one person living there before dropping to zero occupancy over the holiday; the loss adjuster noted the property was furnished with 'some evidence of habitation'; a neighbour's contemporaneous message asking when the brother was due back (sent before occupancy had even been queried by UKI) was unlikely to have been fabricated to support a claim</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>UKI required to reconsider Ms S's claim based on the remaining policy terms, without relying on the unoccupancy exclusion</t>
+        </is>
+      </c>
+      <c r="N49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P49" s="3" t="inlineStr">
+        <is>
+          <t>Where a policy's unoccupancy exclusion requires only that someone was 'sleeping there on a regular basis' (rather than that the property be their sole, official or registered residence), an insurer cannot treat the absence of official records (driving licence, bank statements, credit applications) at that address as determinative of non-occupancy — a meaningful, timing-consistent drop in utility usage coinciding with residents leaving, corroborated by contemporaneous third-party evidence (e.g. a neighbour's message) generated before occupancy was even disputed, can outweigh an insurer's circumstantial residency-scoring evidence in a finely balanced case; the burden remains on the insurer to show, on the balance of probabilities, that the exclusion applied</t>
+        </is>
+      </c>
+      <c r="Q49" s="3" t="inlineStr">
+        <is>
+          <t>Official documentary evidence (bank statements, driving licence, credit applications) showing the brother resident at the insured flat — absent, but not required by the policy's actual 'sleeping there regularly' wording</t>
+        </is>
+      </c>
+      <c r="R49" s="3" t="inlineStr">
+        <is>
+          <t>The policy wording required only regular sleeping at the property, not sole/registered residence, so UKI's reliance on official-address records elsewhere wasn't determinative; utility usage fell in a pattern consistent with the policyholder's own departure and then her brother's temporary absence over Christmas, rather than the flat being empty throughout; the loss adjuster's own observation of 'some evidence of habitation' supported occupation; a neighbour's unprompted, pre-dispute message asking when the brother was due back was strong corroborating evidence not generated to support a claim; on balance, in this finely balanced case, UKI hadn't done enough to show it was more likely than not that the brother wasn't sleeping there regularly</t>
+        </is>
+      </c>
+      <c r="S49" s="3" t="inlineStr">
+        <is>
+          <t>When assessing an unoccupancy exclusion that only requires someone to be 'sleeping there regularly' (not registered residence), don't treat mismatched official records (licence, bank address, credit applications) as determinative — instead weigh utility-usage timing patterns against the claimed occupancy timeline, and give weight to contemporaneous third-party evidence (e.g. neighbour messages) generated before the insurer had even raised an occupancy dispute, since such evidence is less likely to have been created to support the claim</t>
+        </is>
+      </c>
+      <c r="T49" s="3" t="inlineStr">
+        <is>
+          <t>IF policy_unoccupancy_exclusion_requires_only_that_someone_sleeps_at_the_property_regularly_not_that_it_be_their_registered_or_sole_residence THEN mismatched_official_address_records_elsewhere_are_not_determinative_of_non_occupancy; IF utility_usage_timing_pattern_is_consistent_with_the_claimed_occupancy_and_departure_dates AND contemporaneous_third_party_evidence_predating_any_insurer_occupancy_dispute_corroborates_occupancy THEN this_evidence_should_be_weighed_favourably_against_an_insurers_circumstantial_non_occupancy_indicators</t>
+        </is>
+      </c>
+      <c r="U49" s="3" t="inlineStr">
+        <is>
+          <t>DRN-5990244.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="80" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>DRN-6146897</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Liverpool Victoria Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>12 Mar 2026</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Home insurance — burst pipe caused water damage after the policyholders had moved out to relocate; insurer initially validated the claim, then declined it on discovering the property had actually been unoccupied since well before the extended-cover period it had granted, applying its unoccupied-property exclusion</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Policyholders moved out in August 2024 to relocate while the property remained on the market; in December 2024 they told LV the property was unoccupied; LV said it didn't cover unoccupied properties but would extend cover for 60 days (to 18 February 2025) to allow time to arrange specialist unoccupied-property insurance elsewhere, without asking when the property had actually become unoccupied; a pipe burst in January 2025, and LV later discovered the property had in fact been empty since August 2024 — well over 60 days before the loss</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (vacated for relocation, up for sale)</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Property had been unoccupied for more than 60 consecutive days at the time of the loss, which the policy excludes for perils including escape of water</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Mr and Mrs O: LV's agent never asked when they'd moved out during the December 2024 call, despite Mr O opening the call by saying 'it's been a while', and the agent gave the impression full cover would continue for a further 60 days (to 18 February 2025) — they relied on that understanding and hadn't sought alternative cover sooner. LV: the policy wording on unoccupancy was clear, and it had upheld a separate complaint about delay in handling the claim (paying £12,977.48 towards mitigation works) while maintaining its decline of the underlying claim was correct. FOS: having listened to the December call recording, LV's agent failed to pick up on Mr O's opening comment and never asked when the property became unoccupied, instead assuming the unoccupancy period started from the date of the call — had it asked, it would have discovered the property was already well past the 60-day threshold, meaning the 'extended cover' offer was illusory; it was reasonable for Mr and Mrs O to have understood from the call that they had full cover for a further 60 days</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>LV required to meet the claim in full under the remaining policy terms and pay Mr and Mrs O £750 compensation for distress and inconvenience</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="n">
+        <v>750</v>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>Where an insurer is told during a call that a property has become unoccupied and offers an extension of cover to allow time to arrange specialist unoccupied-property insurance, it must ask when the unoccupancy actually began rather than assuming it started from the date of the call — an extension offer calculated from the wrong start date is illusory if the property was already past the exclusion threshold, and a policyholder who reasonably relied on being told they had continued cover cannot fairly have a later-discovered unoccupancy start date used against them to decline a claim that arose during what they believed was the extension period</t>
+        </is>
+      </c>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — LV's own December 2024 call recording, once properly reviewed, showed the agent's failure to ask the key question about the unoccupancy start date</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>Mr O's opening remark ('it's been a while') was a cue LV's agent should have followed up, but didn't; the agent assumed the unoccupancy period started from the date of the December 2024 call and offered 60 days' extended cover on that (incorrect) basis, without ever asking Mr O directly when the property had actually become empty; had it asked, it would have learned the property had been empty since August 2024 — already beyond the 60-day exclusion threshold — meaning no meaningful extension was ever actually available; it was reasonable for Mr O to have believed, based on what LV told him, that full cover applied until 18 February 2025; LV's separate acknowledgment of delay (and its mitigation-cost payment) didn't address the underlying unfairness of declining the claim on this basis</t>
+        </is>
+      </c>
+      <c r="S50" s="2" t="inlineStr">
+        <is>
+          <t>When a policyholder reports a property has become unoccupied and an insurer offers a grace-period extension before cover lapses, the call handler must establish the actual date unoccupancy began — assuming it started from the date of the call, without asking, risks offering an illusory extension to a policyholder who is already past the exclusion threshold and will reasonably rely on the (incorrect) impression that cover continues</t>
+        </is>
+      </c>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>IF insurer_offers_a_grace_period_extension_of_cover_after_being_told_a_property_has_become_unoccupied AND insurer_does_not_ask_when_the_unoccupancy_actually_began_and_instead_assumes_it_started_from_the_date_of_the_call THEN any_later_decline_based_on_the_true_unoccupancy_start_date_is_unfair_if_the_policyholder_reasonably_relied_on_the_extension_offer_as_given</t>
+        </is>
+      </c>
+      <c r="U50" s="2" t="inlineStr">
+        <is>
+          <t>DRN-6146897.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="80" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-050</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>DRN6665775</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Groupama Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — theft of home contents discovered on the policyholder's return from time away from the UK; insurer declined citing the unoccupied-property exclusion (not lived in for more than 60 consecutive days), despite a friend visiting the property every two days while the policyholder was away</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder away from the UK for an extended period; arranged for a friend to visit the property every two days while he was away; contents went missing during this period, discovered on his return</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Residential property (regularly visited but policyholder absent)</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>Property had not been lived in by the policyholder or his family for more than 60 consecutive days, so theft cover was excluded under the unoccupied-property exclusion</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>Mr J: a friend visited his home every two days while he was away, which he said should be enough to avoid the property being treated as unoccupied; separately said the theft exclusion for unoccupied properties hadn't been brought to his attention when the policy was sold (considered under a separate complaint reference). Groupama: regular visits by a third party don't amount to the property being 'lived in' by the policyholder or his family as the policy requires. FOS: agreed that visits by an arranged third party every two days, while helpful for security, don't on balance amount to the property being lived in for policy purposes, so the exclusion was correctly applied; separately, Groupama's own delay in providing a clear explanation of its decision when Mr J asked for clarification was excessive and amounted to poor service, which Groupama didn't substantively dispute but argued shouldn't attract compensation because other customers who don't complain don't receive it either — an argument the ombudsman rejected as irrelevant to whether Mr J personally was entitled to redress</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M51" s="3" t="inlineStr">
+        <is>
+          <t>The coverage decline itself (theft excluded due to unoccupancy) found reasonable and not disturbed; Groupama required to pay Mr J £100 compensation for the distress and inconvenience caused by its poor customer service in explaining its decision</t>
+        </is>
+      </c>
+      <c r="N51" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="O51" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P51" s="3" t="inlineStr">
+        <is>
+          <t>Regular visits by a third party (e.g. a friend checking the property every two days) arranged by the policyholder while they are away do not, on balance, amount to the property being 'lived in' by the policyholder or their family for the purposes of a standard unoccupied-property exclusion — this is consistent with how other unoccupancy definitions in this database treat periodic visits/inspections as distinct from actual habitation; an insurer's argument that compensating one complainant for poor service would be 'unfair' to other customers who didn't complain is not a valid basis for withholding otherwise-warranted distress and inconvenience compensation</t>
+        </is>
+      </c>
+      <c r="Q51" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — the visiting arrangement (a friend every two days) was undisputed; the dispute was over whether it met the 'lived in' threshold</t>
+        </is>
+      </c>
+      <c r="R51" s="3" t="inlineStr">
+        <is>
+          <t>Consistent with this Service's general approach, having someone visit a property periodically while the policyholder is away does not on balance constitute the property being lived in, so Groupama's application of the unoccupied-property exclusion to the theft claim was reasonable; however, the length of time Groupama took to give Mr J a comprehensive explanation of its decision was excessive and amounted to poor service; Groupama's argument that paying compensation would be unfair to non-complaining customers was irrelevant to whether Mr J, who did complain and was genuinely inconvenienced, should be compensated; a modest £100 award (consistent with this Service's general approach to such awards) was fair</t>
+        </is>
+      </c>
+      <c r="S51" s="3" t="inlineStr">
+        <is>
+          <t>Even where an insurer's unoccupied-property coverage decline is found entirely reasonable and upheld, separately assess the quality and timeliness of its explanation to the policyholder once queried — poor or delayed communication about a correctly-made decision can still attract distress and inconvenience compensation independent of the coverage outcome; an insurer's 'fairness to other customers' argument against paying complaint-driven compensation should be disregarded as irrelevant</t>
+        </is>
+      </c>
+      <c r="T51" s="3" t="inlineStr">
+        <is>
+          <t>IF third_party_visits_a_property_periodically_eg_every_two_days_while_policyholder_is_away AND policy_requires_the_property_to_be_lived_in_by_the_policyholder_or_family THEN periodic_third_party_visits_do_not_meet_the_lived_in_threshold_and_unoccupancy_exclusion_applies_reasonably; IF insurer_took_an_excessive_time_to_explain_a_correctly_made_coverage_decision_when_queried THEN this_independently_warrants_modest_distress_and_inconvenience_compensation_regardless_of_the_coverage_outcome</t>
+        </is>
+      </c>
+      <c r="U51" s="3" t="inlineStr">
+        <is>
+          <t>DRN6665775.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="80" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>DRN7122779</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>24 Aug 2019</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Unoccupied residential property policy (executors of a deceased owner's estate) — escape of water from a burst pipe; insurer declined citing breach of a policy condition requiring the central heating to be set to operate continuously at not less than 12°C between 1 November and 31 March</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Policy taken out by the executors in February 2018 specifically to cover their late relative's former home, unoccupied pending sale; a buyer had already been found; burst pipe discovered 10 March 2018, about two weeks after cover started (24 February 2018)</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (deceased owner's estate, unoccupied pending sale)</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Insurer's loss adjuster didn't think the executors had complied with the policy condition requiring continuous heating at a minimum of 12°C between 1 November and 31 March, based on a comparison of utility bills between the relevant period in 2018 and the same period the year before</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>Executors: they had every reason to keep the heating on given a buyer had already been found and there'd be little point taking out an unoccupied property policy for such a short period without intending to comply with its terms. SOL: gas usage for January-April 2018 (£72.36) was far lower than the equivalent 2017 period (£327.29, when the property was occupied by an elderly, infirm former owner and his carer), and it also implied the executors delayed the loss adjuster's visit to allow time to turn the heating back on and inflate usage. FOS: the relevant compliance window was only about two weeks (24 February to 10 March) during which a thermostatically-controlled system cycles on and off rather than running continuously, and no hot water use would register either; the loss adjuster's own April 2018 visit found the thermostat set to 15°C, above the 12°C minimum; the delay in the loss adjuster's visit was because one executor was awaiting a hospital operation, not to manipulate usage; the boiler needed repairs after the leak, giving further reason to leave heating off pending inspection; and the prior year's higher usage reflected genuine occupation by an elderly, infirm resident, which would naturally run warmer than an empty property on a minimum-temperature setting</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>SOL required to settle the claim (repair costs) subject to the remaining policy terms and conditions, pay 8% simple interest on any reimbursement from the date payment was made by the executors, and pay £200 compensation for trouble and upset; SOL not required to cover ongoing property-maintenance costs pending sale, as these aren't covered by the policy</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>Where an insurer relies on a lower-than-comparable-period utility bill to infer breach of a minimum-continuous-heating condition, the burden remains on the insurer to show the shortfall isn't otherwise explained — a short compliance window (where a thermostatic system cycles on/off rather than running continuously and no hot water is used), a documented reason for delaying reconnection after a loss (e.g. awaiting boiler repair or the policyholder's ill health), and a comparator period reflecting materially different circumstances (e.g. genuine occupation by an elderly resident versus an empty property on a minimum setting) can all undermine an insurer's inference of non-compliance from bill comparison alone</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>Direct evidence of the thermostat setting at the time of the loss (the loss adjuster's reading of 15°C was taken a month later, in April 2018) — not available, requiring the ombudsman to weigh circumstantial usage evidence instead</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>This was a finely balanced case, but SOL hadn't done enough to show non-compliance with the heating condition given: the short (roughly two-week) compliance window before the loss, during which a thermostatically-controlled system wouldn't run continuously and no hot water would be used; a documented, credible reason (one executor's upcoming hospital operation) for delaying the loss adjuster's visit rather than any attempt to manipulate usage; a plausible reason (awaiting boiler repair, living some distance away) for not immediately turning heating back on post-loss; and the prior year's higher comparator usage reflecting genuine occupation by an elderly, infirm resident rather than the same type of unoccupied-property heating regime</t>
+        </is>
+      </c>
+      <c r="S52" s="2" t="inlineStr">
+        <is>
+          <t>When assessing a suspected breach of a minimum-continuous-heating condition via utility bill comparison, check (a) how short the actual compliance window was between cover starting and the loss (a thermostatic system won't show continuous draw), (b) whether there's a credible non-fraudulent reason for any delay in the insurer's inspection or in reconnecting services post-loss, and (c) whether the comparator period reflects a materially different occupancy status (e.g. a previously occupied elderly resident versus a minimum-heated empty property) before relying on the bill differential alone</t>
+        </is>
+      </c>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>IF insurer_relies_on_lower_utility_usage_compared_to_a_prior_period_to_infer_breach_of_a_minimum_continuous_heating_condition AND the_actual_compliance_window_before_the_loss_was_short_and_a_thermostatic_system_would_not_show_continuous_draw AND there_are_credible_non_fraudulent_explanations_for_any_inspection_or_reconnection_delay THEN the_bill_comparison_alone_does_not_establish_non_compliance_and_the_claim_should_be_settled</t>
+        </is>
+      </c>
+      <c r="U52" s="2" t="inlineStr">
+        <is>
+          <t>DRN7122779.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="80" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-052</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>DRN7223290</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>5 Jun 2020</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Joint home insurance — escape of water discovered February 2018; insurer declined citing the unoccupied-property exclusion (not permanently lived in for more than 60 consecutive days), after an initial fraud allegation (later retracted) that the policyholder had knowingly misrepresented the property as occupied</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder said he'd been the sole occupant since the property was refurbished in August 2017, working shifts and having caring responsibilities elsewhere; insurer's loss adjuster/investigator found a lack of furniture and food, a council tax record showing the property as unfurnished/unoccupied since purchase, extremely low water usage (£3.27 over six months), the policyholder still listed at a different address on his driving licence, car insurance and electoral roll, and no evidence he was registered with a doctor or had utilities/broadband near the insured address</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Residential property (occupancy status disputed; not the policyholder's confirmed sole residence)</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Multiple evidentiary indicators (utility usage, council tax status, driving licence/insurance address, electoral roll, absence of local medical registration or utility contracts) showed the property wasn't permanently lived in by the policyholder for more than 60 consecutive days</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Mr J: said he lived there normally and had furnished the kitchen, bedroom and other rooms, was registered to vote there, and used shower facilities at work explaining low water usage; he wasn't present at the time of the incident due to bad weather. AXA: retracted its fraud allegation but maintained the occupancy exclusion applied, citing the cumulative weight of independent evidence (utility usage, council tax, driving licence, electoral/GP registration, absence of local utility contracts) rather than any single factor. FOS: while any one indicator might be explained individually (e.g. showering at work), the cumulative pattern — very low water usage, driving licence and car insurance only updated to the insured address after the incident, no council tax liability being collected since the purchase date, no local GP registration, no TV or broadband contracts at the address, and legal advice sought near his other address rather than the insured one — was more consistent with him not permanently living there</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M53" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — AXA's reliance on the unoccupied-property exclusion was reasonable given the weight of independent evidence, though any reference to the retracted fraud allegation should be removed from the policyholder's insurance records</t>
+        </is>
+      </c>
+      <c r="N53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P53" s="3" t="inlineStr">
+        <is>
+          <t>When assessing whether a policyholder was 'permanently living' at a property for occupancy-exclusion purposes, no single piece of circumstantial evidence (e.g. low water usage alone, or an out-of-date driving licence alone) needs to be individually conclusive — an insurer can rely on the cumulative, mutually-reinforcing weight of several independent indicators (utility usage, council tax liability status, official address records across multiple institutions, absence of local medical/utility registrations, and even where the policyholder sought legal advice) even where the policyholder offers plausible individual explanations for some of them</t>
+        </is>
+      </c>
+      <c r="Q53" s="3" t="inlineStr">
+        <is>
+          <t>Contemporaneous evidence corroborating the policyholder's claimed sole occupancy (e.g. updated official address records, GP registration, local utility contracts) predating the escape of water — the documents he did provide (including his driving licence) were dated after the incident</t>
+        </is>
+      </c>
+      <c r="R53" s="3" t="inlineStr">
+        <is>
+          <t>Individually, low water usage might be explained by showering at work, and forgetting to update a driving licence is common — but taken together with the council tax record (unoccupied since purchase, no liability collected), the absence of any local GP registration or utility/broadband contracts, and the fact he sought legal advice and had his car insurance registered near his other address rather than the insured one, the cumulative picture was more consistent with him not permanently living at the insured property; AXA's retraction of the fraud allegation was appropriate but didn't change the underlying occupancy conclusion</t>
+        </is>
+      </c>
+      <c r="S53" s="3" t="inlineStr">
+        <is>
+          <t>When assessing a disputed occupancy claim, don't evaluate each circumstantial indicator (utility usage, address records, registrations) in isolation against an innocent explanation — assess the cumulative pattern across multiple independent sources; a policyholder providing innocent explanations for individual data points doesn't defeat an occupancy exclusion if the totality of independent evidence still points the other way</t>
+        </is>
+      </c>
+      <c r="T53" s="3" t="inlineStr">
+        <is>
+          <t>IF multiple_independent_occupancy_indicators_eg_utility_usage_council_tax_status_official_address_records_local_registrations ALL_POINT_AWAY_FROM_the_policyholders_claimed_occupancy THEN the_cumulative_weight_of_evidence_can_support_the_unoccupancy_exclusion_even_where_each_individual_indicator_has_a_plausible_innocent_explanation</t>
+        </is>
+      </c>
+      <c r="U53" s="3" t="inlineStr">
+        <is>
+          <t>DRN7223290.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="80" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>DRN7626527</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Ageas 50 Limited (trading as RIAS plc)</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Home insurance (broker mis-sale complaint) — theft claim declined by the underlying insurer citing the unoccupied-property exclusion (not lived in for more than 60 consecutive days) after the policyholder returned from time outside the UK to find contents missing; complaint concerned whether the broker had adequately brought the exclusion to his attention at sale</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Policyholder was outside the UK for an extended period; on application and at each renewal he was asked whether the home would be left unoccupied for more than 60 consecutive days and answered 'No'; he was sent a 'Policy Summary' booklet (which he says was the only documentation he received) confirming exclusions applied for unoccupied properties, and the broker said a full policy booklet was also sent though the policyholder said he didn't receive it</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (occupancy status disputed while policyholder travelled)</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable to a decision by the broker directly — the underlying insurer declined the theft claim under the unoccupied-property exclusion; this complaint concerned only whether the broker adequately brought that exclusion to the policyholder's attention at the point of sale and renewal</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Mr G: the 'Policy Summary' booklet he received didn't adequately bring the unoccupied-property exclusions to his attention, and even though he'd confirmed at application that the home wouldn't be left empty for more than 60 days, the significance of that answer hadn't been explained to him. RIAS: it had asked him directly whether the property would be unoccupied for more than 60 days (he said no) and sent documentation at inception and each renewal referencing the unoccupied-property exclusions. FOS: the 'Policy Summary' itself stated it didn't contain the full policy conditions and that these were in the separate policy wording; if Mr G hadn't received that fuller wording, he could reasonably have called RIAS to request it; the Policy Summary he did receive still confirmed exclusions applied to unoccupied properties, and the direct question-and-answer at application/renewal indicated to RIAS that the unoccupied exclusion wouldn't be a significant limitation for him, given his own repeated 'No' answers</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — RIAS sufficiently brought the unoccupied-property exclusion to Mr G's attention through the direct application/renewal questions and the Policy Summary documentation; no award made</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>Where a broker directly asks a policyholder at both application and each renewal whether the property will be left unoccupied for more than a specified number of days, and the policyholder repeatedly confirms it won't be, this exchange itself is evidence the broker sufficiently brought the significance of the unoccupied-property exclusion to the policyholder's attention — even where a summary document (rather than the full policy wording) is the only documentation the policyholder says they actually received, provided that summary itself flags that exclusions apply to unoccupied properties and that fuller wording is available on request</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — whether the full policy booklet was actually received by Mr G was disputed but not determinative, since the Policy Summary and the direct application questions were sufficient on their own</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>The direct question asked at application and each subsequent renewal — whether the property would be left unoccupied for more than 60 consecutive days — put Mr G on notice that this was a relevant factor for his cover, and his repeated 'No' answers meant RIAS reasonably understood the exclusion wasn't a live concern for him; even accepting he only received the Policy Summary (not the full wording), that document itself flagged unoccupied-property exclusions existed and directed him to the full wording if he wanted more detail, which he could have requested but didn't</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>When a broker asks a direct, unambiguous question about a policy-relevant circumstance (e.g. extended unoccupancy) at both sale and every renewal, and the policyholder consistently answers in a way that would rule out the exclusion applying, this exchange itself can satisfy the broker's disclosure duty — a summary document that flags an exclusion exists and signposts fuller wording on request need not itself contain every detail, provided the policyholder wasn't prevented from requesting more information</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>IF broker_asks_a_direct_unambiguous_question_about_a_time_limited_unoccupancy_threshold_at_both_sale_and_every_renewal AND policyholder_consistently_answers_in_a_way_ruling_out_the_exclusion_applying THEN this_exchange_together_with_a_summary_document_flagging_the_exclusions_exist_satisfies_the_brokers_disclosure_duty_even_if_the_full_policy_wording_was_not_confirmed_received</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>DRN7626527.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="80" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-054</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>DRN7714548</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Landlords household / property insurance — escape of water from a burst loft pipe during refurbishment between tenancies; insurer declined citing the property had been unoccupied for more than 30 days (and separately, breach of a 14-day unoccupancy endorsement requiring services turned off and drained), amid significant confusion over which of several conflicting policy documents actually applied</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Following the end of a tenancy, the policyholder arranged extensive refurbishment/maintenance to re-let the property and kept the heating on throughout (both to protect the property from cold and because contractors were working in it); more than two months after the tenant left, during exceptionally cold weather, the boiler failed and a loft pipe burst; the policyholder and letting agent visited regularly and contractors were present on a scheduled basis throughout, though RSA said the property had nonetheless been 'unoccupied' since the tenant moved out</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Rental property between tenancies, undergoing refurbishment</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>RSA said the property had been unoccupied (defined in its policy documentation as 'the part or whole of the property not lived in by a person authorised by You') for more than 30/60 days, and separately that the policyholder hadn't complied with a 14-day unoccupancy endorsement requiring gas and water supplies to be turned off and the system drained</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder: the property was effectively never left unoccupied for more than a few days at a time given the frequency of contractor visits and her and her partner's own visits to check progress and collect mail; keeping the heating on for the workmen and to protect the property against cold weather was reasonable in the circumstances. RSA: supplied conflicting, inconsistent policy documentation across several requests (a 'Property Insurance Policy' booklet, a 'Summary of Cover' referencing a combined 'Property Policy'/'Unoccupied Property Policy', and at one point a different 'Let Property Flexilet' booklet entirely), none of which matched the endorsement referenced on the policyholder's own certificate. FOS: given the unresolved documentation confusion, the policyholder's own certificate (specific to her policy, correct property and cover period) was the most reliable indicator of the actual endorsements in place, and RSA's supplied booklets likely weren't the correct documents; but even assuming they were correct, the policy's 'unoccupied' definition ('not lived in by a person authorised by You') was a significantly unusual definition that wasn't adequately drawn to the policyholder's attention despite being prominently set out in the Summary of Cover — without knowing that specific, unusual definition, she couldn't appreciate the significance of the exclusions and limitations referencing it, so the ordinary meaning of 'unoccupied' should apply instead, under which the property (given the frequency of contractor and personal visits) shouldn't be treated as unoccupied at all</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M55" s="3" t="inlineStr">
+        <is>
+          <t>RSA required to settle the claim in accordance with the remaining policy terms and conditions, and pay 8% simple interest per year on any cash payment from the date of loss to the date of payment</t>
+        </is>
+      </c>
+      <c r="N55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P55" s="3" t="inlineStr">
+        <is>
+          <t>Where an insurer cannot reliably establish which of several conflicting policy documents it has supplied actually governs the claim, the policyholder's own certificate (specific to their policy, property and cover period) is the more reliable indicator of the endorsements actually in place; separately, where a policy defines 'unoccupied' in a way significantly different from its ordinary meaning (e.g. 'not lived in by a person authorised by You', rather than the Service's usual approach recognising regular visits/contractor presence as occupation), the insurer must adequately draw that unusual definition to the policyholder's attention — merely including it in a summary of cover alongside numerous other unoccupancy exclusions and limitations is not necessarily adequate; without such notice, the ordinary meaning of 'unoccupied' should be applied instead</t>
+        </is>
+      </c>
+      <c r="Q55" s="3" t="inlineStr">
+        <is>
+          <t>A single, consistent, agreed-correct policy document — RSA identified three different, mutually-inconsistent booklets across its various responses as 'the' correct policy document</t>
+        </is>
+      </c>
+      <c r="R55" s="3" t="inlineStr">
+        <is>
+          <t>The significant confusion in RSA's own document production (three different, non-matching policy booklets identified as correct at different points) meant the policyholder's own certificate — which matched the property, cover period and premium — was the more reliable record of her actual policy terms; even if RSA's supplied booklets were assumed correct, the unusual 'unoccupied' definition they contained was significantly different from the ordinary meaning and wasn't adequately highlighted, so it would not be reasonable to allow RSA to rely on it; applying the ordinary meaning instead, the frequency of contractor and personal visits meant the property shouldn't be treated as unoccupied</t>
+        </is>
+      </c>
+      <c r="S55" s="3" t="inlineStr">
+        <is>
+          <t>When an insurer supplies inconsistent or conflicting policy documentation across a complaint investigation, treat the policyholder's own certificate (matching the specific property, cover period, sums insured and premium) as the more reliable record of actual policy terms; separately, always check whether a policy's definition of 'unoccupied' departs significantly from the ordinary meaning of the word — if so, it must be clearly and specifically highlighted (not merely present somewhere in a summary of cover) or the ordinary meaning should govern instead</t>
+        </is>
+      </c>
+      <c r="T55" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_supplies_multiple_inconsistent_policy_documents_during_a_claim_investigation THEN the_policyholders_own_certificate_matching_the_specific_property_cover_period_and_premium_is_the_more_reliable_record_of_actual_terms; IF policy_defines_unoccupied_significantly_differently_from_its_ordinary_meaning AND this_unusual_definition_was_not_specifically_and_clearly_highlighted_to_the_policyholder THEN the_ordinary_meaning_of_unoccupied_should_govern_instead_and_regular_visits_or_contractor_presence_may_mean_the_property_is_not_unoccupied</t>
+        </is>
+      </c>
+      <c r="U55" s="3" t="inlineStr">
+        <is>
+          <t>DRN7714548.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="80" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>DRN7954504</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>International Insurance Company of Hannover SE</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>16 Feb 2018</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Home insurance — burglary claim; insurer voided the policy for misrepresentation about main residence status, after evidence showed the policyholder didn't actually live at the insured address as declared at inception and each renewal</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Insurer's loss adjuster reported the policyholder told them the property had been unoccupied since 2013 (the policyholder later called this a 'clerical error'); electoral roll entries for the policyholder and his wife showed a different address since 2013; a signed statement to the loss adjuster said the family lived at the insured address until 2012 and mainly at another address since 2013, visiting the insured address roughly every six weeks</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (main residence status disputed)</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Policyholder was asked clear questions at inception (confirming the property was his main residence, unoccupied no more than 30 days a year) and this was untrue based on his own signed statement, electoral roll registration elsewhere, and the loss adjuster's account — a qualifying misrepresentation entitling the insurer to void the policy, since it wouldn't offer cover for a property that wasn't the policyholder's main residence</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Mr E: said whether the property was his 'main residence' was irrelevant since he'd complied with the 45-day unoccupancy requirement he understood applied, visited weekly, and took safety precautions; said it was IICH's 'clerical error' that it recorded him telling the loss adjuster the property had been unoccupied since 2013. IICH: clear, specific questions were asked at the outset about main residence status and expected unoccupancy, confirmed again via a Statement of Insurance sent for him to check and at each renewal without amendment; his own signed statement to the loss adjuster (that he and his family lived mainly elsewhere since 2013, visiting the insured address roughly every six weeks, with his wife not visiting for over six months) contradicted his 'main residence' declaration; electoral roll records supported this. FOS: Mr E's own account across different communications was contradictory (variously saying the property was never unoccupied for more than 45 days, that main residence status was irrelevant since he visited regularly, and later that it was his main residence at the time of the burglary), but his signed statement to the loss adjuster — the most contemporaneous and detailed account — was the more reliable evidence, and it clearly showed the insured address wasn't his main residence</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — IICH acted fairly and in accordance with the policy terms in voiding the policy for misrepresentation about main residence status; no further action required</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>Where a policy is specifically conditioned on the insured property being the policyholder's main residence (a materially different, and often more significant, question than simply whether unoccupancy exceeded a day threshold), and the policyholder's own signed, contemporaneous statement to a loss adjuster describes an actual living pattern inconsistent with that declaration (e.g. living mainly elsewhere, visiting only periodically), that statement is generally more reliable than the policyholder's later, shifting explanations to the insurer or this Service; a general unoccupancy day-count compliance argument (e.g. 'never unoccupied for more than 45 days') doesn't answer a separate 'main residence' misrepresentation question</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable — the signed statement to the loss adjuster and the electoral roll records were treated as sufficiently reliable, contemporaneous evidence despite Mr E's later attempts to characterise parts of it as a 'clerical error'</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>Mr E's account across different points in the process was contradictory and shifted depending on what argument he was making, whereas his signed statement to the loss adjuster gave a detailed, specific account (mainly living elsewhere since 2013, visiting the insured address every six weeks, wife not visiting for over six months) that was corroborated by independent electoral roll records; this showed the insured address wasn't genuinely his main residence, contrary to what was declared at inception and confirmed unamended at each renewal; IICH's evidence that it wouldn't have offered cover on the correct facts (since it doesn't insure unoccupied properties) supported voiding being fair and reasonable</t>
+        </is>
+      </c>
+      <c r="S56" s="2" t="inlineStr">
+        <is>
+          <t>When a policyholder's account of their living arrangements shifts across different stages of a complaint (to the loss adjuster, then in correspondence, then to this Service), give the most weight to the earliest, most detailed, contemporaneous and specific account (e.g. a signed statement to a loss adjuster) rather than later, more generalised or self-serving reformulations; distinguish a 'main residence' declaration question from a simple unoccupancy day-count question, since compliance with one doesn't answer the other</t>
+        </is>
+      </c>
+      <c r="T56" s="2" t="inlineStr">
+        <is>
+          <t>IF policyholders_account_of_living_arrangements_shifts_across_different_stages_of_a_complaint THEN give_most_weight_to_the_earliest_most_detailed_contemporaneous_signed_statement_over_later_reformulations; policy_conditioned_on_main_residence_status_is_a_distinct_question_from_a_general_unoccupancy_day_count_requirement_and_compliance_with_one_does_not_establish_compliance_with_the_other</t>
+        </is>
+      </c>
+      <c r="U56" s="2" t="inlineStr">
+        <is>
+          <t>DRN7954504.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="80" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-056</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>DRN8194702</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>14 Jan 2018</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Landlord insurance (two properties on one policy) — escape of water claim on the unoccupied property was accepted, but the policyholder disputed the quantum of the loss-of-rent payment, non-renewal of the whole policy because one property was unoccupied, and a service error (excess withheld twice)</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>One of two properties on a joint landlord policy became unoccupied from February 2016; leak damage reported September 2016 was initially repudiated for unoccupancy but reconsidered once it was shown the leak occurred during an earlier claim within 30 days of the property becoming unoccupied; UKI declined to renew the whole two-property policy at its next renewal because of the unoccupied property, rather than removing only that property from cover</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Rented residential properties (two properties on one landlord policy; one became unoccupied)</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Claim Quantum Dispute</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Accepted — With Deductions</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable to a full decline — the escape of water claim was accepted, with some damage attributed to uncovered gradual-deterioration maintenance issues rather than the leak itself; the loss-of-rent element was paid at the policy's maximum sum insured (£14,400) rather than the higher monthly rate the policyholder said she could have achieved on the open market</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Miss A: disputed the loss-of-rent rate (£1,200pcm applied versus £1,300-1,400pcm she believed achievable, supported by a letting agent's estimate), wanted rent paid until repairs were actually completed (not capped at the 12-month indemnity period), was unhappy the whole two-property policy wasn't renewed rather than just the unoccupied property, and was unhappy a £200 excess was mistakenly withheld twice. UKI: the sum insured (£14,400, based on £1,200pcm) was the contractual maximum for the 12-month indemnity period regardless of a higher achievable rate; it wasn't obliged to renew cover for an unoccupied property, and since both properties were on one combined contract, ending cover for one meant it wasn't unreasonable to end the whole contract rather than assume she wanted to renew only the unaffected property; the double excess withholding was a system error, corrected and refunded promptly. FOS: the loss-of-rent sum insured was a contractual cap properly applied; investigating a complex claim (including potential unoccupancy grounds to decline it) before accepting liability wasn't inherently unreasonable delay; declining to renew unoccupied-property cover is a legitimate commercial underwriting decision this Service won't interfere with, and ending the whole combined-property contract (rather than assuming a split was wanted) wasn't unreasonable; the excess error was promptly corrected</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — the loss-of-rent payment was correctly capped at the policy limit, non-renewal of the combined two-property policy because of the unoccupied property was a reasonable commercial decision, and the excess/payment-timing errors were promptly and adequately corrected</t>
+        </is>
+      </c>
+      <c r="N57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" s="3" t="inlineStr">
+        <is>
+          <t>No — Quantum Only</t>
+        </is>
+      </c>
+      <c r="P57" s="3" t="inlineStr">
+        <is>
+          <t>A 'loss of rent receivable' indemnity is capped at the policy's stated sum insured for the maximum indemnity period, regardless of a higher market rent the policyholder believes could have been achieved, unless the insurer's own breach or negligence caused a reasonably foreseeable uninsured loss beyond that; where two properties are combined under one landlord insurance contract and one becomes unoccupied, an insurer declining to renew the whole combined contract (rather than assuming the policyholder wants to split cover and retain only the unaffected property) is a legitimate commercial underwriting decision</t>
+        </is>
+      </c>
+      <c r="Q57" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — the facts (rent achieved historically, letting agent's estimate, the excess double-withholding) were undisputed; the dispute was over the correct contractual quantum and remedy</t>
+        </is>
+      </c>
+      <c r="R57" s="3" t="inlineStr">
+        <is>
+          <t>The policy's loss-of-rent section indemnifies up to the stated sum insured for the indemnity period (12 months), which UKI paid in full (£14,400, at £1,200pcm); a letting agent's estimate of a higher achievable rent didn't change the contractual cap, and rent couldn't be paid beyond the indemnity period simply because repairs were delayed while UKI investigated a complex, potentially unoccupancy-affected claim; investigating before accepting liability on a claim with potential grounds to decline wasn't unreasonable delay; ending the whole combined policy (rather than only the unoccupied property) was UKI's legitimate commercial decision, since it covered two properties under one contract and total premium; the double-excess error was a system glitch, corrected promptly upon discovery</t>
+        </is>
+      </c>
+      <c r="S57" s="3" t="inlineStr">
+        <is>
+          <t>For loss-of-rent disputes, check whether the payment matches the policy's stated sum insured and indemnity period cap — a higher achievable market rent (even if independently estimated by a letting agent) doesn't override a contractual limit; when an insurer declines to renew a multi-property policy because one property became unoccupied, treat this as a legitimate single commercial decision rather than requiring the insurer to have offered a split renewal for the unaffected property</t>
+        </is>
+      </c>
+      <c r="T57" s="3" t="inlineStr">
+        <is>
+          <t>IF loss_of_rent_claim_payment_matches_the_policys_stated_sum_insured_and_indemnity_period THEN a_higher_market_estimate_from_a_letting_agent_does_not_entitle_the_policyholder_to_more_than_the_contractual_cap; IF multiple_properties_are_combined_under_one_landlord_policy_and_one_becomes_unoccupied THEN insurer_declining_to_renew_the_whole_combined_contract_rather_than_offering_a_split_renewal_is_a_legitimate_commercial_decision</t>
+        </is>
+      </c>
+      <c r="U57" s="3" t="inlineStr">
+        <is>
+          <t>DRN8194702.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="80" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-057</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>DRN8309060</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Lloyds Bank General Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>11 Apr 2016</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Home insurance — malicious damage and arson claims; insurer found evidence the policyholder hadn't lived at the property for a long time and backdated cancellation of cover to a year after it believed he stopped living there, declining the two claims that arose after that backdated cancellation date</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Insurer believed the policyholder hadn't lived at the property since late 2012 or earlier, based on extremely low electricity usage (2-7% of an average household from 2011-2013) and a post-fire assessor's report indicating the property had been unoccupied and used as a meeting place by local youths for some time; insurer's stated approach was to provide a lower level of cover for unoccupied properties for one year, then no cover after that, and it backdated cancellation to 1 December 2013 (a year after the date it believed occupancy ceased)</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Residential property (occupancy status disputed over an extended period)</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Policyholder hadn't told the insurer he'd stopped living at the property as required by the policy, and the insurer's evidence indicated he'd stopped living there more than a year before the two declined claims — beyond the one year of reduced unoccupied-property cover it said it would have provided</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Mr C: said he was living at the property until a burglary in late November 2013 (paid by Lloyds, as it preceded the cancellation date) made it uninhabitable, and offered to provide witness statements supporting this. Lloyds: electricity usage during 2012 was only 2-7% of an average household, a post-fire assessor's report described the property as unoccupied and used by local youths as a meeting place, and earlier 2013 theft claims hadn't mentioned any change in occupancy despite Lloyds believing he'd already moved out by then. FOS: the electricity usage evidence, considered against Mr C's explanation (long hours as a taxi driver), still indicated no more than occasional visits rather than genuine residence; the assessor's report of youths using the property as a meeting place independently corroborated non-occupancy; witness statements weren't accepted as equivalent to independent evidence like utility bills, and Lloyds had already given Mr C a list of acceptable evidence types which he hadn't otherwise provided</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Lloyds acted reasonably in backdating cancellation to a year after it believed occupancy ceased, based on persuasive independent evidence (utility usage, assessor's report), and in declining the two claims that fell after that date</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>An insurer's stated commercial approach of providing a reduced level of cover for an unoccupied property for a fixed period (e.g. one year) and no cover thereafter is a legitimate underwriting decision; where independent evidence (extremely low utility usage compared to an average household, and an independent assessor's observations, e.g. of unauthorised use by local youths) points to a specific date occupancy ceased, an insurer can fairly backdate a policy cancellation to that date plus its stated grace period, and decline claims falling after it; witness statements from the policyholder's own contacts are not treated as equivalent to independent documentary evidence (e.g. utility bills) when assessing disputed occupancy</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>Independent documentary evidence (of the type Lloyds' agent had previously told Mr C would be acceptable) corroborating his claimed occupancy through to late November 2013 — he offered only witness statements, which weren't treated as sufficient</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>Electricity usage in 2012 at only 2-7% of an average household consumption was not adequately explained by Mr C's long working hours as a taxi driver, and indicated no more than occasional visits; an independent post-fire assessor separately reported signs the property had been unoccupied and used as a meeting place by local youths, corroborating the low-usage finding; witness statements from Mr C's own contacts weren't independent in the way utility bills are, and he hadn't provided any of the other acceptable evidence types Lloyds' agent had already identified for him; on balance, it was reasonable for Lloyds to conclude occupancy had ceased around November 2012 and to backdate cancellation a year from that date</t>
+        </is>
+      </c>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>When assessing disputed long-term occupancy, weigh independent documentary evidence (utility usage compared to household averages, independent assessor observations) more heavily than witness statements from the policyholder's own contacts, which lack independence; where an insurer's stated policy is to provide reduced unoccupied-property cover for a fixed grace period before cover lapses entirely, backdating cancellation to that period's end from the evidenced date occupancy ceased is a reasonable approach to claims arising after that point</t>
+        </is>
+      </c>
+      <c r="T58" s="2" t="inlineStr">
+        <is>
+          <t>IF independent_evidence_eg_utility_usage_far_below_household_average_and_independent_assessor_observations_indicate_a_specific_date_occupancy_ceased THEN insurer_may_backdate_cancellation_to_that_date_plus_its_stated_unoccupied_property_grace_period_and_decline_claims_arising_after_it; witness_statements_from_the_policyholders_own_contacts_are_not_equivalent_to_independent_documentary_evidence_when_assessing_disputed_long_term_occupancy</t>
+        </is>
+      </c>
+      <c r="U58" s="2" t="inlineStr">
+        <is>
+          <t>DRN8309060.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="80" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-058</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>DRN8328581</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Ageas 50 Limited</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance (broker administration complaint) — escape of water claim from a burst loft pipe declined by the underlying insurer citing the unoccupied-property exclusion, after the broker added a specific term excluding escape-of-water cover for the entire duration of the policyholder's 90-day holiday but never called back to explain this as promised</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder proactively called her broker to disclose a 90-day holiday during which her home would be unoccupied; broker's in-house underwriters added a term excluding escape-of-water damage for the entire holiday (not just the usual 60-day threshold), and sent an amended schedule, but never called back as twice promised to explain the new term; policyholder's daughter discovered a burst loft pipe during the holiday</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Residential property (long holiday absence, proactively disclosed)</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable to a decision by the broker directly — the underlying insurer declined the escape of water claim under the newly-added unoccupancy term; this complaint concerned whether the broker adequately explained that new term to the policyholder after she proactively disclosed her holiday</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Ms F: she specifically rang her broker to disclose the extended holiday and was told twice she'd be called back to confirm what terms, if any, would apply — that call never came, and she was left with only an amended schedule she didn't realise contained a new, more restrictive term; had she known, she'd have paid extra for full cover. Ageas: there was no change to the general unoccupancy position (she'd never been covered for escape of water beyond 60 days), she'd taken an extended holiday before, and it always communicated in writing without any indication this didn't suit her. FOS: Ageas's response missed the point — the actual term added was materially different from the usual 60-day threshold, excluding escape-of-water cover for the entire 90-day holiday from day one, and this specific alteration wasn't adequately drawn to Ms F's attention; having proactively called to disclose her holiday and been promised a follow-up call that never came, she was entitled to assume the information had been noted and cover would continue as before</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>Ageas required to deal with the escape of water claim as if it were the insurer (instructing an independent loss adjuster, cash-settling at open market reinstatement rates if applicable, with 8% simple interest from the date of claim), and pay Ms F £400 compensation for distress and inconvenience</t>
+        </is>
+      </c>
+      <c r="N59" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="O59" s="3" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P59" s="3" t="inlineStr">
+        <is>
+          <t>Where a policyholder proactively discloses an extended absence to their broker and is explicitly told they'll receive a follow-up call to confirm what terms will apply, a broker's failure to make that promised call — instead relying on an amended schedule alone to convey a newly added, materially more restrictive exclusion (here, escape-of-water cover excluded for the entire holiday rather than only after the usual 60-day threshold) — does not adequately draw the new term to the policyholder's attention; a general awareness of a standard unoccupancy exclusion doesn't put a policyholder on notice of a specific, non-standard alteration made in response to their particular disclosure</t>
+        </is>
+      </c>
+      <c r="Q59" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — that no follow-up call was made, despite being promised twice, was not disputed</t>
+        </is>
+      </c>
+      <c r="R59" s="3" t="inlineStr">
+        <is>
+          <t>The broker's argument that Ms F was already generally aware of the standard 60-day unoccupancy exclusion missed the point, since the actual term added for this holiday was materially different (excluding escape-of-water for the whole 90 days, not just beyond 60); having proactively disclosed her holiday and been told twice she'd receive a call to confirm applicable terms, Ms F was entitled to assume, in the absence of that call, that her disclosure had simply been noted and standard cover would continue; had she known the true position she would likely have sought alternative unoccupied-property cover or taken precautions like draining the water system, so the broker's failure caused real detriment</t>
+        </is>
+      </c>
+      <c r="S59" s="3" t="inlineStr">
+        <is>
+          <t>When a policyholder proactively discloses a change in circumstances (e.g. an extended absence) and is promised a follow-up call to confirm resulting policy changes, a broker cannot rely on a passively-sent amended schedule alone to satisfy that promise — especially where the resulting term is materially more restrictive than the policyholder's prior, general understanding of the standard exclusion; assess what specifically changed against what the policyholder could reasonably have already known, not just whether an unoccupancy exclusion of some kind existed generally</t>
+        </is>
+      </c>
+      <c r="T59" s="3" t="inlineStr">
+        <is>
+          <t>IF policyholder_proactively_discloses_an_extended_absence_to_a_broker_and_is_promised_a_follow_up_call_to_confirm_applicable_terms AND broker_fails_to_make_that_call_and_instead_relies_only_on_a_passively_sent_amended_schedule_containing_a_materially_more_restrictive_new_term THEN the_new_term_was_not_adequately_disclosed_regardless_of_the_policyholders_general_prior_awareness_of_a_standard_unoccupancy_exclusion</t>
+        </is>
+      </c>
+      <c r="U59" s="3" t="inlineStr">
+        <is>
+          <t>DRN8328581.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="80" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>UNOC-059</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>DRN8482133</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>14 Dec 2015</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Unoccupied property insurance (two rental flats) — theft and malicious damage claim declined citing a restricted 'FLEE' (fire, lightning, earthquake, explosion) cover term issued when the flats were unoccupied for renovation, even though the insurer's own published policy change meant full cover should have applied by the time of the loss</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Flats insured in 2013 while undergoing internal (non-structural) renovation for a planned 12-week period, with a restricted FLEE-only policy issued on that basis; by 2014 (when the theft/malicious damage claim arose) the properties had become tenanted as planned; insurer declined citing the restricted cover, saying it hadn't been told the flats had become tenanted</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Rental flats (unoccupied for renovation, later re-let as planned)</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Only restricted 'FLEE' cover applied to the policy (issued while the flats were unoccupied for renovation), and the insurer hadn't been informed the properties had since become tenanted</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Mr R: pointed to the insurer's own 2012 customer newsletter, which said that from 1 April 2012 its Unoccupied Property cover would provide full cover at all times unless restricted cover was specifically requested or structural work was being undertaken — neither of which applied to him (he'd only requested cover for minor, non-structural renovation and hadn't asked for restricted cover); there was also no policy requirement to notify the insurer once the properties became tenanted. Lloyd's: said its underwriter wouldn't have offered full cover in Mr R's circumstances, and that the newsletter's increased cover only applied to subsidence or accidental damage. FOS: Lloyd's hadn't explained how its position accorded with the newsletter's clear wording, which imposed no such peril-specific limitation and applied to Mr R's exact situation (non-structural renovation, no restricted cover requested); since the flats becoming tenanted didn't need to be reported and there was no evidence full cover would have been refused once occupied, the claim should be dealt with as if full (unoccupied property) cover applied throughout</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's required to deal with Mr R's claim as if full cover applied, subject to the remaining policy terms and conditions, and pay £200 compensation for the inconvenience caused by its handling of the claim</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Where an insurer has published a general customer communication (e.g. a newsletter) stating that its unoccupied-property cover will provide full cover at all times unless restricted cover is specifically requested or structural work is being undertaken, and a policyholder's actual circumstances (non-structural renovation, no restricted cover requested) fall squarely within that stated full-cover scenario, the insurer cannot later assert an unexplained, undocumented limitation (e.g. that the increased cover applied only to certain perils) to justify declining a claim under a narrower restricted-cover term — it must show how its position accords with what it told policyholders generally it would do</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>Any explanation from Lloyd's of how its asserted peril-specific limitation (that increased unoccupied-property cover applied only to subsidence or accidental damage) was consistent with, or derived from, the newsletter's unqualified statement of full cover — none was provided despite being asked</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>The 2012 newsletter's language was unqualified: full cover applies to unoccupied properties at all times unless restricted cover is requested or structural work is underway; Mr R's disclosed circumstances (minor, non-structural renovation, no restricted cover requested) matched this exactly, so he was entitled to expect full cover; Lloyd's assertion that it wouldn't have offered full cover, and that the newsletter's increase was peril-limited, was unsupported and inconsistent with the newsletter's actual wording; there being no requirement to report the flats becoming tenanted, and no evidence full cover would have been withdrawn once they were, the claim should be dealt with as though full cover had applied throughout</t>
+        </is>
+      </c>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>When an insurer relies on a restricted-cover term to decline a claim, check whether the insurer has separately published general customer communications (newsletters, cover-change notices) describing a more generous default position that would apply to the policyholder's actual disclosed circumstances — an insurer cannot decline a claim under a narrower term without explaining how that's consistent with what it told policyholders generally it would do in that scenario</t>
+        </is>
+      </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>IF insurer_has_published_a_general_customer_communication_stating_a_more_generous_default_unoccupied_property_cover_position AND policyholders_actual_disclosed_circumstances_fall_within_the_scenario_described_in_that_communication THEN insurer_cannot_rely_on_a_narrower_restricted_cover_term_to_decline_the_claim_without_explaining_how_this_is_consistent_with_the_published_communication</t>
+        </is>
+      </c>
+      <c r="U60" s="2" t="inlineStr">
+        <is>
+          <t>DRN8482133.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="80" customHeight="1">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>UNOC-060</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>DRN9942137</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>L. P. Dawe</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>10 Jul 2015</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance (broker mis-sale complaint) — inherited property insured via a broker; escape of water claim declined and the policy cancelled by the insurer, after the broker recommended a renewal policy without updating stale information about the policyholder's living circumstances, resulting in a policy unsuited to the property being a second (frequently empty) home rather than her permanent residence</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder inherited the property from her late mother in 2010; broker's original 2010 file note recorded she would 'eventually be living in' it once she sold her own home, with the property unoccupied at times in the meantime; when her original insurer stopped offering this type of policy, the broker recommended a replacement with a second insurer in 2011/2012 using the same year-old assumptions, without checking whether she'd actually moved in; by the July 2013 escape of water claim, she was still living at her own home with her mother's house standing empty for extended periods</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Inherited residential property (never became the policyholder's permanent residence as originally assumed)</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable to a decision by the broker directly — the second insurer refused to consider the escape of water claim and cancelled the policy; this complaint concerned only whether the broker had sold/renewed her into an unsuitable policy</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>Miss B: the broker sold her an inappropriate policy that didn't cover her actual circumstances (the property being a second home, empty for significant periods) rather than her main residence. L P Dawe: it had originally been given information (via the solicitors administering the estate) that she intended to move into the property once she sold her own home, justifying a policy suited to that plan; the policy's statement of facts (listing the property as her 'permanent residence') was sent to her and she never queried or corrected it. FOS: the 2010 recommendation was suitable based on the information available at the time (her stated intention to move in once her own home sold); however, when the original insurer stopped offering the product and L P Dawe had to recommend a replacement policy for the 2011/2012 renewal, it simply reused the year-old assumption that she'd moved in as planned, without checking her actual current circumstances — this fell short of what an advising broker should do at each renewal, especially given a change of insurer/product was involved, not just a routine like-for-like renewal</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>L P Dawe required to pay Miss B the amount an insurer would probably have paid had she been sold a policy suited to the property being a second home left empty for significant periods (via agreement or a jointly-instructed loss adjuster's assessment, at L P Dawe's expense), arrange removal of the cancellation record from the insurer's internal and external databases (or provide a letter confirming the cancellation was its error), and pay Miss B £200 for distress and inconvenience</t>
+        </is>
+      </c>
+      <c r="N61" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="O61" s="3" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P61" s="3" t="inlineStr">
+        <is>
+          <t>A broker's recommendation for an initial policy can be suitable when based on the customer's stated intentions at the time (e.g. an intention to move into an inherited property once a current home is sold) — but at each subsequent renewal, particularly where a change of insurer or product is required (not simply a routine like-for-like renewal), the broker must update its understanding of the customer's actual current circumstances rather than reusing stale assumptions; a customer's failure to proactively correct an inaccurate 'permanent residence' assumption printed in a statement of facts does not excuse the broker from its own duty to actively re-verify suitability when arranging a new policy at renewal</t>
+        </is>
+      </c>
+      <c r="Q61" s="3" t="inlineStr">
+        <is>
+          <t>Any updated information-gathering by L P Dawe at the 2011/2012 renewal about whether Miss B had actually moved into the inherited property as originally planned — none was obtained; it simply carried forward the 2010 assumption</t>
+        </is>
+      </c>
+      <c r="R61" s="3" t="inlineStr">
+        <is>
+          <t>L P Dawe's 2010 file note showed a reasonable, suitable recommendation based on Miss B's stated plan to eventually live in the inherited property; but when the original insurer withdrew from this product and a new policy with a different insurer had to be arranged for the next renewal, L P Dawe simply carried forward the same year-old assumption without re-checking whether she'd actually moved in — this was not good enough advising practice, particularly given a change of insurer/product (as opposed to a routine renewal) specifically calls for re-verification; as a result she was sold a policy that didn't suit her real circumstances (property remaining a second, often-empty home), and when she came to claim, this mismatch caused her claim to be refused and her policy cancelled</t>
+        </is>
+      </c>
+      <c r="S61" s="3" t="inlineStr">
+        <is>
+          <t>When a broker has to move a customer to a new insurer or product at renewal (rather than a routine like-for-like renewal with the same insurer), treat this as a trigger to actively re-verify the customer's current circumstances rather than carrying forward assumptions from the original sale — this is especially important for unoccupied/second-home situations where an original stated intention (e.g. to move in) may not have materialised by the time of a later renewal</t>
+        </is>
+      </c>
+      <c r="T61" s="3" t="inlineStr">
+        <is>
+          <t>IF broker_must_arrange_a_new_policy_with_a_different_insurer_or_product_at_renewal_rather_than_a_routine_like_for_like_renewal AND broker_carries_forward_a_stale_assumption_about_the_customers_occupancy_circumstances_from_the_original_sale_without_re_verifying_it THEN broker_is_responsible_for_any_resulting_unsuitable_policy_and_the_consequences_of_a_claim_being_refused_on_that_basis</t>
+        </is>
+      </c>
+      <c r="U61" s="3" t="inlineStr">
+        <is>
+          <t>DRN9942137.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>